<commit_message>
Utilities limited to BEMC and Brunswick County; Verizon and Focus Broadband moved to Phone & Internet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -375,7 +375,7 @@
         <v>20789.8</v>
       </c>
       <c r="G10" s="6">
-        <f>SUM(G7:G9)</f>
+        <f>F10/4</f>
         <v>5197.45</v>
       </c>
     </row>
@@ -568,7 +568,7 @@
         <v>5833.15</v>
       </c>
       <c r="G18" s="6">
-        <f>SUM(G13:G17)</f>
+        <f>F18/4</f>
         <v>1458.29</v>
       </c>
     </row>
@@ -642,595 +642,540 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
-        </is>
-      </c>
-      <c r="B23" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A23,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Utilities</t>
+        </is>
+      </c>
+      <c r="B23" s="6">
+        <f>SUM(B21:B22)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C23" s="6">
+        <f>SUM(C21:C22)</f>
+        <v>336.35</v>
+      </c>
+      <c r="D23" s="6">
+        <f>SUM(D21:D22)</f>
+        <v>586.29</v>
+      </c>
+      <c r="E23" s="6">
+        <f>SUM(E21:E22)</f>
+        <v>503.92</v>
+      </c>
+      <c r="F23" s="6">
+        <f>SUM(F21:F22)</f>
+        <v>1505.4</v>
+      </c>
+      <c r="G23" s="6">
+        <f>F23/4</f>
+        <v>376.35</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Phone &amp; Internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
+        </is>
+      </c>
+      <c r="B26" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A26,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>80.79</v>
       </c>
-      <c r="C23" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A23,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C26" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A26,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D23" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A23,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D26" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A26,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>161.58</v>
       </c>
-      <c r="E23" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A23,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E26" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A26,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>80.79</v>
       </c>
-      <c r="F23" s="3">
-        <f>SUM(B23:E23)</f>
+      <c r="F26" s="3">
+        <f>SUM(B26:E26)</f>
         <v>323.16</v>
       </c>
-      <c r="G23" s="3">
-        <f>F23/4</f>
+      <c r="G26" s="3">
+        <f>F26/4</f>
         <v>80.79</v>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
-      <c r="B24" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A24,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B27" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A27,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>294.57</v>
       </c>
-      <c r="C24" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A24,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C27" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A27,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>294.8</v>
       </c>
-      <c r="D24" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A24,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D27" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A27,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>436.02</v>
       </c>
-      <c r="E24" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A24,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E27" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A27,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>386.85</v>
       </c>
-      <c r="F24" s="3">
-        <f>SUM(B24:E24)</f>
+      <c r="F27" s="3">
+        <f>SUM(B27:E27)</f>
         <v>1412.24</v>
       </c>
-      <c r="G24" s="3">
-        <f>F24/4</f>
+      <c r="G27" s="3">
+        <f>F27/4</f>
         <v>353.06</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Utilities</t>
-        </is>
-      </c>
-      <c r="B25" s="6">
-        <f>SUM(B21:B24)</f>
-        <v>454.2</v>
-      </c>
-      <c r="C25" s="6">
-        <f>SUM(C21:C24)</f>
-        <v>631.15</v>
-      </c>
-      <c r="D25" s="6">
-        <f>SUM(D21:D24)</f>
-        <v>1183.89</v>
-      </c>
-      <c r="E25" s="6">
-        <f>SUM(E21:E24)</f>
-        <v>971.56</v>
-      </c>
-      <c r="F25" s="6">
-        <f>SUM(F21:F24)</f>
-        <v>3240.8</v>
-      </c>
-      <c r="G25" s="6">
-        <f>SUM(G21:G24)</f>
-        <v>810.2</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Phone &amp; Internet</t>
+        </is>
+      </c>
+      <c r="B28" s="6">
+        <f>SUM(B26:B27)</f>
+        <v>375.36</v>
+      </c>
+      <c r="C28" s="6">
+        <f>SUM(C26:C27)</f>
+        <v>294.8</v>
+      </c>
+      <c r="D28" s="6">
+        <f>SUM(D26:D27)</f>
+        <v>597.6</v>
+      </c>
+      <c r="E28" s="6">
+        <f>SUM(E26:E27)</f>
+        <v>467.64</v>
+      </c>
+      <c r="F28" s="6">
+        <f>SUM(F26:F27)</f>
+        <v>1735.4</v>
+      </c>
+      <c r="G28" s="6">
+        <f>F28/4</f>
+        <v>433.85</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Debt Payments</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
-      <c r="B28" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A28,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B31" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A31,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>160.37</v>
       </c>
-      <c r="C28" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A28,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C31" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A31,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>160.37</v>
       </c>
-      <c r="D28" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A28,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D31" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A31,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>160.37</v>
       </c>
-      <c r="E28" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A28,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E31" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A31,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>160.37</v>
       </c>
-      <c r="F28" s="3">
-        <f>SUM(B28:E28)</f>
+      <c r="F31" s="3">
+        <f>SUM(B31:E31)</f>
         <v>641.48</v>
       </c>
-      <c r="G28" s="3">
-        <f>F28/4</f>
+      <c r="G31" s="3">
+        <f>F31/4</f>
         <v>160.37</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Debt Payments</t>
         </is>
       </c>
-      <c r="B29" s="6">
-        <f>SUM(B28:B28)</f>
+      <c r="B32" s="6">
+        <f>SUM(B31:B31)</f>
         <v>160.37</v>
       </c>
-      <c r="C29" s="6">
-        <f>SUM(C28:C28)</f>
+      <c r="C32" s="6">
+        <f>SUM(C31:C31)</f>
         <v>160.37</v>
       </c>
-      <c r="D29" s="6">
-        <f>SUM(D28:D28)</f>
+      <c r="D32" s="6">
+        <f>SUM(D31:D31)</f>
         <v>160.37</v>
       </c>
-      <c r="E29" s="6">
-        <f>SUM(E28:E28)</f>
+      <c r="E32" s="6">
+        <f>SUM(E31:E31)</f>
         <v>160.37</v>
       </c>
-      <c r="F29" s="6">
-        <f>SUM(F28:F28)</f>
+      <c r="F32" s="6">
+        <f>SUM(F31:F31)</f>
         <v>641.48</v>
       </c>
-      <c r="G29" s="6">
-        <f>SUM(G28:G28)</f>
+      <c r="G32" s="6">
+        <f>F32/4</f>
         <v>160.37</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Food</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Food</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Groceries</t>
         </is>
       </c>
-      <c r="B32" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A32,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B35" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A35,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1529.75</v>
       </c>
-      <c r="C32" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A32,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C35" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A35,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D32" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A32,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D35" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A35,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1190.12</v>
       </c>
-      <c r="E32" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A32,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E35" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A35,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F32" s="3">
-        <f>SUM(B32:E32)</f>
+      <c r="F35" s="3">
+        <f>SUM(B35:E35)</f>
         <v>5201.61</v>
       </c>
-      <c r="G32" s="3">
-        <f>F32/4</f>
+      <c r="G35" s="3">
+        <f>F35/4</f>
         <v>1300.4</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
-        </is>
-      </c>
-      <c r="B33" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A33,'All Transactions'!$A$5:$A$436,B$4)</f>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+        </is>
+      </c>
+      <c r="B36" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A36,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1019.45</v>
       </c>
-      <c r="C33" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A33,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C36" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A36,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>935.1</v>
       </c>
-      <c r="D33" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A33,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D36" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A36,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>962.62</v>
       </c>
-      <c r="E33" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A33,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E36" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A36,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>872.56</v>
       </c>
-      <c r="F33" s="3">
-        <f>SUM(B33:E33)</f>
+      <c r="F36" s="3">
+        <f>SUM(B36:E36)</f>
         <v>3789.73</v>
       </c>
-      <c r="G33" s="3">
-        <f>F33/4</f>
+      <c r="G36" s="3">
+        <f>F36/4</f>
         <v>947.43</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="7" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Food</t>
         </is>
       </c>
-      <c r="B34" s="6">
-        <f>SUM(B32:B33)</f>
+      <c r="B37" s="6">
+        <f>SUM(B35:B36)</f>
         <v>2549.2</v>
       </c>
-      <c r="C34" s="6">
-        <f>SUM(C32:C33)</f>
+      <c r="C37" s="6">
+        <f>SUM(C35:C36)</f>
         <v>2214.34</v>
       </c>
-      <c r="D34" s="6">
-        <f>SUM(D32:D33)</f>
+      <c r="D37" s="6">
+        <f>SUM(D35:D36)</f>
         <v>2152.74</v>
       </c>
-      <c r="E34" s="6">
-        <f>SUM(E32:E33)</f>
+      <c r="E37" s="6">
+        <f>SUM(E35:E36)</f>
         <v>2075.06</v>
       </c>
-      <c r="F34" s="6">
-        <f>SUM(F32:F33)</f>
+      <c r="F37" s="6">
+        <f>SUM(F35:F36)</f>
         <v>8991.34</v>
       </c>
-      <c r="G34" s="6">
-        <f>SUM(G32:G33)</f>
+      <c r="G37" s="6">
+        <f>F37/4</f>
         <v>2247.83</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Transportation</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Gas &amp; Convenience Stores</t>
         </is>
       </c>
-      <c r="B37" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A37,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B40" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A40,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>108.9</v>
       </c>
-      <c r="C37" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A37,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C40" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A40,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>277.87</v>
       </c>
-      <c r="D37" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A37,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D40" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A40,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>167.24</v>
       </c>
-      <c r="E37" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A37,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E40" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A40,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>238.98</v>
       </c>
-      <c r="F37" s="3">
-        <f>SUM(B37:E37)</f>
+      <c r="F40" s="3">
+        <f>SUM(B40:E40)</f>
         <v>792.99</v>
       </c>
-      <c r="G37" s="3">
-        <f>F37/4</f>
+      <c r="G40" s="3">
+        <f>F40/4</f>
         <v>198.25</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Tolls &amp; Parking</t>
         </is>
       </c>
-      <c r="B38" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A38,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B41" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A41,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>5.84</v>
       </c>
-      <c r="C38" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A38,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C41" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A41,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D38" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A38,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D41" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A41,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>18.44</v>
       </c>
-      <c r="E38" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A38,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E41" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A41,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>74.24</v>
       </c>
-      <c r="F38" s="3">
-        <f>SUM(B38:E38)</f>
+      <c r="F41" s="3">
+        <f>SUM(B41:E41)</f>
         <v>98.52</v>
       </c>
-      <c r="G38" s="3">
-        <f>F38/4</f>
+      <c r="G41" s="3">
+        <f>F41/4</f>
         <v>24.63</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="7" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Transportation</t>
         </is>
       </c>
-      <c r="B39" s="6">
-        <f>SUM(B37:B38)</f>
+      <c r="B42" s="6">
+        <f>SUM(B40:B41)</f>
         <v>114.74</v>
       </c>
-      <c r="C39" s="6">
-        <f>SUM(C37:C38)</f>
+      <c r="C42" s="6">
+        <f>SUM(C40:C41)</f>
         <v>277.87</v>
       </c>
-      <c r="D39" s="6">
-        <f>SUM(D37:D38)</f>
+      <c r="D42" s="6">
+        <f>SUM(D40:D41)</f>
         <v>185.68</v>
       </c>
-      <c r="E39" s="6">
-        <f>SUM(E37:E38)</f>
+      <c r="E42" s="6">
+        <f>SUM(E40:E41)</f>
         <v>313.22</v>
       </c>
-      <c r="F39" s="6">
-        <f>SUM(F37:F38)</f>
+      <c r="F42" s="6">
+        <f>SUM(F40:F41)</f>
         <v>891.51</v>
       </c>
-      <c r="G39" s="6">
-        <f>SUM(G37:G38)</f>
+      <c r="G42" s="6">
+        <f>F42/4</f>
         <v>222.88</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="5" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming</t>
         </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Streaming – YouTube TV (Google)</t>
-        </is>
-      </c>
-      <c r="B42" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A42,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>100.78</v>
-      </c>
-      <c r="C42" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A42,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.78</v>
-      </c>
-      <c r="D42" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A42,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>89.0</v>
-      </c>
-      <c r="E42" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A42,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>132.43</v>
-      </c>
-      <c r="F42" s="3">
-        <f>SUM(B42:E42)</f>
-        <v>422.99</v>
-      </c>
-      <c r="G42" s="3">
-        <f>F42/4</f>
-        <v>105.75</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
-        </is>
-      </c>
-      <c r="B43" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A43,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>13.87</v>
-      </c>
-      <c r="C43" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A43,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>13.87</v>
-      </c>
-      <c r="D43" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A43,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>13.87</v>
-      </c>
-      <c r="E43" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A43,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>13.87</v>
-      </c>
-      <c r="F43" s="3">
-        <f>SUM(B43:E43)</f>
-        <v>55.48</v>
-      </c>
-      <c r="G43" s="3">
-        <f>F43/4</f>
-        <v>13.87</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
-        </is>
-      </c>
-      <c r="B44" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A44,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>20.27</v>
-      </c>
-      <c r="C44" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A44,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>20.27</v>
-      </c>
-      <c r="D44" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A44,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>20.27</v>
-      </c>
-      <c r="E44" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A44,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>20.27</v>
-      </c>
-      <c r="F44" s="3">
-        <f>SUM(B44:E44)</f>
-        <v>81.08</v>
-      </c>
-      <c r="G44" s="3">
-        <f>F44/4</f>
-        <v>20.27</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – HBO Max</t>
+          <t xml:space="preserve">Streaming – YouTube TV (Google)</t>
         </is>
       </c>
       <c r="B45" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A45,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>19.74</v>
+        <v>100.78</v>
       </c>
       <c r="C45" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A45,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>19.74</v>
+        <v>100.78</v>
       </c>
       <c r="D45" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A45,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>89.0</v>
       </c>
       <c r="E45" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A45,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>132.43</v>
       </c>
       <c r="F45" s="3">
         <f>SUM(B45:E45)</f>
-        <v>39.48</v>
+        <v>422.99</v>
       </c>
       <c r="G45" s="3">
         <f>F45/4</f>
-        <v>9.87</v>
+        <v>105.75</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Hulu</t>
+          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
         </is>
       </c>
       <c r="B46" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A46,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>13.87</v>
       </c>
       <c r="C46" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A46,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>12.8</v>
+        <v>13.87</v>
       </c>
       <c r="D46" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A46,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>12.8</v>
+        <v>13.87</v>
       </c>
       <c r="E46" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A46,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>13.87</v>
       </c>
       <c r="F46" s="3">
         <f>SUM(B46:E46)</f>
-        <v>25.6</v>
+        <v>55.48</v>
       </c>
       <c r="G46" s="3">
         <f>F46/4</f>
-        <v>6.4</v>
+        <v>13.87</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Peacock (via Roku)</t>
+          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
         </is>
       </c>
       <c r="B47" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A47,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>11.73</v>
+        <v>20.27</v>
       </c>
       <c r="C47" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A47,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>11.73</v>
+        <v>20.27</v>
       </c>
       <c r="D47" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A47,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>20.27</v>
       </c>
       <c r="E47" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A47,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>20.27</v>
       </c>
       <c r="F47" s="3">
         <f>SUM(B47:E47)</f>
-        <v>23.46</v>
+        <v>81.08</v>
       </c>
       <c r="G47" s="3">
         <f>F47/4</f>
-        <v>5.87</v>
+        <v>20.27</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Frndly TV</t>
+          <t xml:space="preserve">Streaming – HBO Max</t>
         </is>
       </c>
       <c r="B48" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A48,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>22.41</v>
+        <v>19.74</v>
       </c>
       <c r="C48" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A48,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>22.41</v>
+        <v>19.74</v>
       </c>
       <c r="D48" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A48,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>22.41</v>
+        <v>0</v>
       </c>
       <c r="E48" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A48,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>22.41</v>
+        <v>0</v>
       </c>
       <c r="F48" s="3">
         <f>SUM(B48:E48)</f>
-        <v>89.64</v>
+        <v>39.48</v>
       </c>
       <c r="G48" s="3">
         <f>F48/4</f>
-        <v>22.41</v>
+        <v>9.87</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Netflix</t>
+          <t xml:space="preserve">Streaming – Hulu</t>
         </is>
       </c>
       <c r="B49" s="3">
@@ -1239,11 +1184,11 @@
       </c>
       <c r="C49" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A49,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>12.8</v>
       </c>
       <c r="D49" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A49,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>12.8</v>
       </c>
       <c r="E49" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A49,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1251,399 +1196,399 @@
       </c>
       <c r="F49" s="3">
         <f>SUM(B49:E49)</f>
-        <v>0</v>
+        <v>25.6</v>
       </c>
       <c r="G49" s="3">
         <f>F49/4</f>
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Streaming – Peacock (via Roku)</t>
+        </is>
+      </c>
+      <c r="B50" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A50,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>11.73</v>
+      </c>
+      <c r="C50" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A50,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>11.73</v>
+      </c>
+      <c r="D50" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A50,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E50" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A50,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F50" s="3">
+        <f>SUM(B50:E50)</f>
+        <v>23.46</v>
+      </c>
+      <c r="G50" s="3">
+        <f>F50/4</f>
+        <v>5.87</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Streaming – Frndly TV</t>
+        </is>
+      </c>
+      <c r="B51" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A51,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>22.41</v>
+      </c>
+      <c r="C51" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A51,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>22.41</v>
+      </c>
+      <c r="D51" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A51,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>22.41</v>
+      </c>
+      <c r="E51" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A51,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>22.41</v>
+      </c>
+      <c r="F51" s="3">
+        <f>SUM(B51:E51)</f>
+        <v>89.64</v>
+      </c>
+      <c r="G51" s="3">
+        <f>F51/4</f>
+        <v>22.41</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Streaming – Netflix</t>
+        </is>
+      </c>
+      <c r="B52" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A52,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C52" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A52,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D52" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A52,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E52" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A52,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F52" s="3">
+        <f>SUM(B52:E52)</f>
+        <v>0</v>
+      </c>
+      <c r="G52" s="3">
+        <f>F52/4</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="7" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Streaming</t>
         </is>
       </c>
-      <c r="B50" s="6">
-        <f>SUM(B42:B49)</f>
+      <c r="B53" s="6">
+        <f>SUM(B45:B52)</f>
         <v>188.8</v>
       </c>
-      <c r="C50" s="6">
-        <f>SUM(C42:C49)</f>
+      <c r="C53" s="6">
+        <f>SUM(C45:C52)</f>
         <v>201.6</v>
       </c>
-      <c r="D50" s="6">
-        <f>SUM(D42:D49)</f>
+      <c r="D53" s="6">
+        <f>SUM(D45:D52)</f>
         <v>158.35</v>
       </c>
-      <c r="E50" s="6">
-        <f>SUM(E42:E49)</f>
+      <c r="E53" s="6">
+        <f>SUM(E45:E52)</f>
         <v>188.98</v>
       </c>
-      <c r="F50" s="6">
-        <f>SUM(F42:F49)</f>
+      <c r="F53" s="6">
+        <f>SUM(F45:F52)</f>
         <v>737.73</v>
       </c>
-      <c r="G50" s="6">
-        <f>SUM(G42:G49)</f>
-        <v>184.44</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="5" t="inlineStr">
+      <c r="G53" s="6">
+        <f>F53/4</f>
+        <v>184.43</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Subscriptions</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="12" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Software &amp; Online Subscriptions</t>
         </is>
       </c>
-      <c r="B53" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A53,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B56" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A56,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>141.73</v>
       </c>
-      <c r="C53" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A53,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C56" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A56,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>161.05</v>
       </c>
-      <c r="D53" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A53,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D56" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A56,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>65.98</v>
       </c>
-      <c r="E53" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A53,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E56" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A56,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F53" s="3">
-        <f>SUM(B53:E53)</f>
+      <c r="F56" s="3">
+        <f>SUM(B56:E56)</f>
         <v>368.76</v>
       </c>
-      <c r="G53" s="3">
-        <f>F53/4</f>
+      <c r="G56" s="3">
+        <f>F56/4</f>
         <v>92.19</v>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="7" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Subscriptions</t>
         </is>
       </c>
-      <c r="B54" s="6">
-        <f>SUM(B53:B53)</f>
+      <c r="B57" s="6">
+        <f>SUM(B56:B56)</f>
         <v>141.73</v>
       </c>
-      <c r="C54" s="6">
-        <f>SUM(C53:C53)</f>
+      <c r="C57" s="6">
+        <f>SUM(C56:C56)</f>
         <v>161.05</v>
       </c>
-      <c r="D54" s="6">
-        <f>SUM(D53:D53)</f>
+      <c r="D57" s="6">
+        <f>SUM(D56:D56)</f>
         <v>65.98</v>
       </c>
-      <c r="E54" s="6">
-        <f>SUM(E53:E53)</f>
+      <c r="E57" s="6">
+        <f>SUM(E56:E56)</f>
         <v>0</v>
       </c>
-      <c r="F54" s="6">
-        <f>SUM(F53:F53)</f>
+      <c r="F57" s="6">
+        <f>SUM(F56:F56)</f>
         <v>368.76</v>
       </c>
-      <c r="G54" s="6">
-        <f>SUM(G53:G53)</f>
+      <c r="G57" s="6">
+        <f>F57/4</f>
         <v>92.19</v>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="5" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Health</t>
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="12" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Medical &amp; Pharmacy</t>
         </is>
       </c>
-      <c r="B57" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A57,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B60" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A60,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>160.07</v>
       </c>
-      <c r="C57" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A57,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C60" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A60,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>100.93</v>
       </c>
-      <c r="D57" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A57,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D60" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A60,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>850.9</v>
       </c>
-      <c r="E57" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A57,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E60" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A60,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>160.28</v>
       </c>
-      <c r="F57" s="3">
-        <f>SUM(B57:E57)</f>
+      <c r="F60" s="3">
+        <f>SUM(B60:E60)</f>
         <v>1272.18</v>
       </c>
-      <c r="G57" s="3">
-        <f>F57/4</f>
+      <c r="G60" s="3">
+        <f>F60/4</f>
         <v>318.05</v>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="7" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Health</t>
         </is>
       </c>
-      <c r="B58" s="6">
-        <f>SUM(B57:B57)</f>
+      <c r="B61" s="6">
+        <f>SUM(B60:B60)</f>
         <v>160.07</v>
       </c>
-      <c r="C58" s="6">
-        <f>SUM(C57:C57)</f>
+      <c r="C61" s="6">
+        <f>SUM(C60:C60)</f>
         <v>100.93</v>
       </c>
-      <c r="D58" s="6">
-        <f>SUM(D57:D57)</f>
+      <c r="D61" s="6">
+        <f>SUM(D60:D60)</f>
         <v>850.9</v>
       </c>
-      <c r="E58" s="6">
-        <f>SUM(E57:E57)</f>
+      <c r="E61" s="6">
+        <f>SUM(E60:E60)</f>
         <v>160.28</v>
       </c>
-      <c r="F58" s="6">
-        <f>SUM(F57:F57)</f>
+      <c r="F61" s="6">
+        <f>SUM(F60:F60)</f>
         <v>1272.18</v>
       </c>
-      <c r="G58" s="6">
-        <f>SUM(G57:G57)</f>
+      <c r="G61" s="6">
+        <f>F61/4</f>
         <v>318.05</v>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Personal</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="12" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
         </is>
       </c>
-      <c r="B61" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A61,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B64" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A64,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>182.5</v>
       </c>
-      <c r="C61" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A61,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C64" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A64,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D61" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A61,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D64" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A64,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>182.5</v>
       </c>
-      <c r="E61" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A61,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E64" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A64,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>114.5</v>
       </c>
-      <c r="F61" s="3">
-        <f>SUM(B61:E61)</f>
+      <c r="F64" s="3">
+        <f>SUM(B64:E64)</f>
         <v>479.5</v>
       </c>
-      <c r="G61" s="3">
-        <f>F61/4</f>
+      <c r="G64" s="3">
+        <f>F64/4</f>
         <v>119.88</v>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="7" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Personal</t>
         </is>
       </c>
-      <c r="B62" s="6">
-        <f>SUM(B61:B61)</f>
+      <c r="B65" s="6">
+        <f>SUM(B64:B64)</f>
         <v>182.5</v>
       </c>
-      <c r="C62" s="6">
-        <f>SUM(C61:C61)</f>
+      <c r="C65" s="6">
+        <f>SUM(C64:C64)</f>
         <v>0</v>
       </c>
-      <c r="D62" s="6">
-        <f>SUM(D61:D61)</f>
+      <c r="D65" s="6">
+        <f>SUM(D64:D64)</f>
         <v>182.5</v>
       </c>
-      <c r="E62" s="6">
-        <f>SUM(E61:E61)</f>
+      <c r="E65" s="6">
+        <f>SUM(E64:E64)</f>
         <v>114.5</v>
       </c>
-      <c r="F62" s="6">
-        <f>SUM(F61:F61)</f>
+      <c r="F65" s="6">
+        <f>SUM(F64:F64)</f>
         <v>479.5</v>
       </c>
-      <c r="G62" s="6">
-        <f>SUM(G61:G61)</f>
+      <c r="G65" s="6">
+        <f>F65/4</f>
         <v>119.88</v>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="5" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Retail</t>
         </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Walmart</t>
-        </is>
-      </c>
-      <c r="B65" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A65,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C65" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A65,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>132.66</v>
-      </c>
-      <c r="D65" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A65,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1732.6</v>
-      </c>
-      <c r="E65" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A65,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.63</v>
-      </c>
-      <c r="F65" s="3">
-        <f>SUM(B65:E65)</f>
-        <v>1897.89</v>
-      </c>
-      <c r="G65" s="3">
-        <f>F65/4</f>
-        <v>474.47</v>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Belk (store card payments)</t>
-        </is>
-      </c>
-      <c r="B66" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A66,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>386.69</v>
-      </c>
-      <c r="C66" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A66,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>948.04</v>
-      </c>
-      <c r="D66" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A66,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E66" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A66,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F66" s="3">
-        <f>SUM(B66:E66)</f>
-        <v>1334.73</v>
-      </c>
-      <c r="G66" s="3">
-        <f>F66/4</f>
-        <v>333.68</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Marshalls</t>
-        </is>
-      </c>
-      <c r="B67" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C67" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D67" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E67" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>41.59</v>
-      </c>
-      <c r="F67" s="3">
-        <f>SUM(B67:E67)</f>
-        <v>41.59</v>
-      </c>
-      <c r="G67" s="3">
-        <f>F67/4</f>
-        <v>10.4</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ross</t>
+          <t xml:space="preserve">Retail – Walmart</t>
         </is>
       </c>
       <c r="B68" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A68,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>48.03</v>
+        <v>0</v>
       </c>
       <c r="C68" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A68,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>132.66</v>
       </c>
       <c r="D68" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A68,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1732.6</v>
       </c>
       <c r="E68" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A68,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>16.32</v>
+        <v>32.63</v>
       </c>
       <c r="F68" s="3">
         <f>SUM(B68:E68)</f>
-        <v>64.35</v>
+        <v>1897.89</v>
       </c>
       <c r="G68" s="3">
         <f>F68/4</f>
-        <v>16.09</v>
+        <v>474.47</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dillard's</t>
+          <t xml:space="preserve">Retail – Belk (store card payments)</t>
         </is>
       </c>
       <c r="B69" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A69,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>386.69</v>
       </c>
       <c r="C69" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A69,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>948.04</v>
       </c>
       <c r="D69" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A69,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>174.74</v>
+        <v>0</v>
       </c>
       <c r="E69" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A69,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1651,22 +1596,22 @@
       </c>
       <c r="F69" s="3">
         <f>SUM(B69:E69)</f>
-        <v>174.74</v>
+        <v>1334.73</v>
       </c>
       <c r="G69" s="3">
         <f>F69/4</f>
-        <v>43.69</v>
+        <v>333.68</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Target</t>
+          <t xml:space="preserve">Retail – Marshalls</t>
         </is>
       </c>
       <c r="B70" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>58.98</v>
+        <v>0</v>
       </c>
       <c r="C70" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1678,26 +1623,26 @@
       </c>
       <c r="E70" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>41.59</v>
       </c>
       <c r="F70" s="3">
         <f>SUM(B70:E70)</f>
-        <v>58.98</v>
+        <v>41.59</v>
       </c>
       <c r="G70" s="3">
         <f>F70/4</f>
-        <v>14.74</v>
+        <v>10.4</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – HomeSense</t>
+          <t xml:space="preserve">Retail – Ross</t>
         </is>
       </c>
       <c r="B71" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>48.03</v>
       </c>
       <c r="C71" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1705,25 +1650,25 @@
       </c>
       <c r="D71" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>88.7</v>
+        <v>0</v>
       </c>
       <c r="E71" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>16.32</v>
       </c>
       <c r="F71" s="3">
         <f>SUM(B71:E71)</f>
-        <v>88.7</v>
+        <v>64.35</v>
       </c>
       <c r="G71" s="3">
         <f>F71/4</f>
-        <v>22.18</v>
+        <v>16.09</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Hobby Lobby</t>
+          <t xml:space="preserve">Retail – Dillard's</t>
         </is>
       </c>
       <c r="B72" s="3">
@@ -1736,30 +1681,30 @@
       </c>
       <c r="D72" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>165.67</v>
+        <v>174.74</v>
       </c>
       <c r="E72" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>37.33</v>
+        <v>0</v>
       </c>
       <c r="F72" s="3">
         <f>SUM(B72:E72)</f>
-        <v>203.0</v>
+        <v>174.74</v>
       </c>
       <c r="G72" s="3">
         <f>F72/4</f>
-        <v>50.75</v>
+        <v>43.69</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
+          <t xml:space="preserve">Retail – Target</t>
         </is>
       </c>
       <c r="B73" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A73,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>27.67</v>
+        <v>58.98</v>
       </c>
       <c r="C73" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A73,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1767,25 +1712,25 @@
       </c>
       <c r="D73" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A73,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>171.55</v>
+        <v>0</v>
       </c>
       <c r="E73" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A73,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>85.27</v>
+        <v>0</v>
       </c>
       <c r="F73" s="3">
         <f>SUM(B73:E73)</f>
-        <v>284.49</v>
+        <v>58.98</v>
       </c>
       <c r="G73" s="3">
         <f>F73/4</f>
-        <v>71.12</v>
+        <v>14.74</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Tractor Supply</t>
+          <t xml:space="preserve">Retail – HomeSense</t>
         </is>
       </c>
       <c r="B74" s="3">
@@ -1798,7 +1743,7 @@
       </c>
       <c r="D74" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>29.86</v>
+        <v>88.7</v>
       </c>
       <c r="E74" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1806,17 +1751,17 @@
       </c>
       <c r="F74" s="3">
         <f>SUM(B74:E74)</f>
-        <v>29.86</v>
+        <v>88.7</v>
       </c>
       <c r="G74" s="3">
         <f>F74/4</f>
-        <v>7.46</v>
+        <v>22.18</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
+          <t xml:space="preserve">Retail – Hobby Lobby</t>
         </is>
       </c>
       <c r="B75" s="3">
@@ -1825,34 +1770,34 @@
       </c>
       <c r="C75" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>63.61</v>
+        <v>0</v>
       </c>
       <c r="D75" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>165.67</v>
       </c>
       <c r="E75" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>37.33</v>
       </c>
       <c r="F75" s="3">
         <f>SUM(B75:E75)</f>
-        <v>63.61</v>
+        <v>203.0</v>
       </c>
       <c r="G75" s="3">
         <f>F75/4</f>
-        <v>15.9</v>
+        <v>50.75</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ulta Beauty</t>
+          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
         </is>
       </c>
       <c r="B76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>134.71</v>
+        <v>27.67</v>
       </c>
       <c r="C76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1860,30 +1805,30 @@
       </c>
       <c r="D76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>171.55</v>
       </c>
       <c r="E76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>85.27</v>
       </c>
       <c r="F76" s="3">
         <f>SUM(B76:E76)</f>
-        <v>134.71</v>
+        <v>284.49</v>
       </c>
       <c r="G76" s="3">
         <f>F76/4</f>
-        <v>33.68</v>
+        <v>71.12</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
+          <t xml:space="preserve">Retail – Tractor Supply</t>
         </is>
       </c>
       <c r="B77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>51.31</v>
+        <v>0</v>
       </c>
       <c r="C77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1891,7 +1836,7 @@
       </c>
       <c r="D77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>29.86</v>
       </c>
       <c r="E77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1899,17 +1844,17 @@
       </c>
       <c r="F77" s="3">
         <f>SUM(B77:E77)</f>
-        <v>51.31</v>
+        <v>29.86</v>
       </c>
       <c r="G77" s="3">
         <f>F77/4</f>
-        <v>12.83</v>
+        <v>7.46</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
         </is>
       </c>
       <c r="B78" s="3">
@@ -1918,11 +1863,11 @@
       </c>
       <c r="C78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>5.87</v>
+        <v>63.61</v>
       </c>
       <c r="D78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>17.35</v>
+        <v>0</v>
       </c>
       <c r="E78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1930,22 +1875,22 @@
       </c>
       <c r="F78" s="3">
         <f>SUM(B78:E78)</f>
-        <v>23.22</v>
+        <v>63.61</v>
       </c>
       <c r="G78" s="3">
         <f>F78/4</f>
-        <v>5.81</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+          <t xml:space="preserve">Retail – Ulta Beauty</t>
         </is>
       </c>
       <c r="B79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.03</v>
+        <v>134.71</v>
       </c>
       <c r="C79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1957,652 +1902,652 @@
       </c>
       <c r="E79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>119.97</v>
+        <v>0</v>
       </c>
       <c r="F79" s="3">
         <f>SUM(B79:E79)</f>
-        <v>228.0</v>
+        <v>134.71</v>
       </c>
       <c r="G79" s="3">
         <f>F79/4</f>
+        <v>33.68</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
+        </is>
+      </c>
+      <c r="B80" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>51.31</v>
+      </c>
+      <c r="C80" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D80" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E80" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F80" s="3">
+        <f>SUM(B80:E80)</f>
+        <v>51.31</v>
+      </c>
+      <c r="G80" s="3">
+        <f>F80/4</f>
+        <v>12.83</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+        </is>
+      </c>
+      <c r="B81" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C81" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>5.87</v>
+      </c>
+      <c r="D81" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>17.35</v>
+      </c>
+      <c r="E81" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F81" s="3">
+        <f>SUM(B81:E81)</f>
+        <v>23.22</v>
+      </c>
+      <c r="G81" s="3">
+        <f>F81/4</f>
+        <v>5.81</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+        </is>
+      </c>
+      <c r="B82" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.03</v>
+      </c>
+      <c r="C82" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D82" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E82" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>119.97</v>
+      </c>
+      <c r="F82" s="3">
+        <f>SUM(B82:E82)</f>
+        <v>228.0</v>
+      </c>
+      <c r="G82" s="3">
+        <f>F82/4</f>
         <v>57.0</v>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="7" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Retail</t>
         </is>
       </c>
-      <c r="B80" s="6">
-        <f>SUM(B65:B79)</f>
+      <c r="B83" s="6">
+        <f>SUM(B68:B82)</f>
         <v>815.42</v>
       </c>
-      <c r="C80" s="6">
-        <f>SUM(C65:C79)</f>
+      <c r="C83" s="6">
+        <f>SUM(C68:C82)</f>
         <v>1150.18</v>
       </c>
-      <c r="D80" s="6">
-        <f>SUM(D65:D79)</f>
+      <c r="D83" s="6">
+        <f>SUM(D68:D82)</f>
         <v>2380.47</v>
       </c>
-      <c r="E80" s="6">
-        <f>SUM(E65:E79)</f>
+      <c r="E83" s="6">
+        <f>SUM(E68:E82)</f>
         <v>333.11</v>
       </c>
-      <c r="F80" s="6">
-        <f>SUM(F65:F79)</f>
+      <c r="F83" s="6">
+        <f>SUM(F68:F82)</f>
         <v>4679.18</v>
       </c>
-      <c r="G80" s="6">
-        <f>SUM(G65:G79)</f>
+      <c r="G83" s="6">
+        <f>F83/4</f>
         <v>1169.8</v>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="5" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Home</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="12" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
-      <c r="B83" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B86" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>60.0</v>
       </c>
-      <c r="C83" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C86" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>100.0</v>
       </c>
-      <c r="D83" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D86" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>220.0</v>
       </c>
-      <c r="E83" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E86" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>120.0</v>
       </c>
-      <c r="F83" s="3">
-        <f>SUM(B83:E83)</f>
+      <c r="F86" s="3">
+        <f>SUM(B86:E86)</f>
         <v>500.0</v>
       </c>
-      <c r="G83" s="3">
-        <f>F83/4</f>
+      <c r="G86" s="3">
+        <f>F86/4</f>
         <v>125.0</v>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="12" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
         </is>
       </c>
-      <c r="B84" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B87" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C84" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C87" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>242.05</v>
       </c>
-      <c r="D84" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D87" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>536.6</v>
       </c>
-      <c r="E84" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E87" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F84" s="3">
-        <f>SUM(B84:E84)</f>
+      <c r="F87" s="3">
+        <f>SUM(B87:E87)</f>
         <v>778.65</v>
       </c>
-      <c r="G84" s="3">
-        <f>F84/4</f>
+      <c r="G87" s="3">
+        <f>F87/4</f>
         <v>194.66</v>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" s="7" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Home</t>
         </is>
       </c>
-      <c r="B85" s="6">
-        <f>SUM(B83:B84)</f>
+      <c r="B88" s="6">
+        <f>SUM(B86:B87)</f>
         <v>60.0</v>
       </c>
-      <c r="C85" s="6">
-        <f>SUM(C83:C84)</f>
+      <c r="C88" s="6">
+        <f>SUM(C86:C87)</f>
         <v>342.05</v>
       </c>
-      <c r="D85" s="6">
-        <f>SUM(D83:D84)</f>
+      <c r="D88" s="6">
+        <f>SUM(D86:D87)</f>
         <v>756.6</v>
       </c>
-      <c r="E85" s="6">
-        <f>SUM(E83:E84)</f>
+      <c r="E88" s="6">
+        <f>SUM(E86:E87)</f>
         <v>120.0</v>
       </c>
-      <c r="F85" s="6">
-        <f>SUM(F83:F84)</f>
+      <c r="F88" s="6">
+        <f>SUM(F86:F87)</f>
         <v>1278.65</v>
       </c>
-      <c r="G85" s="6">
-        <f>SUM(G83:G84)</f>
+      <c r="G88" s="6">
+        <f>F88/4</f>
         <v>319.66</v>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" s="5" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel</t>
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" s="12" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel (Lyft, Hotel)</t>
         </is>
       </c>
-      <c r="B88" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B91" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>102.65</v>
       </c>
-      <c r="C88" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C91" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D88" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D91" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E88" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E91" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F88" s="3">
-        <f>SUM(B88:E88)</f>
+      <c r="F91" s="3">
+        <f>SUM(B91:E91)</f>
         <v>102.65</v>
       </c>
-      <c r="G88" s="3">
-        <f>F88/4</f>
+      <c r="G91" s="3">
+        <f>F91/4</f>
         <v>25.66</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="7" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Travel</t>
         </is>
       </c>
-      <c r="B89" s="6">
-        <f>SUM(B88:B88)</f>
+      <c r="B92" s="6">
+        <f>SUM(B91:B91)</f>
         <v>102.65</v>
       </c>
-      <c r="C89" s="6">
-        <f>SUM(C88:C88)</f>
+      <c r="C92" s="6">
+        <f>SUM(C91:C91)</f>
         <v>0</v>
       </c>
-      <c r="D89" s="6">
-        <f>SUM(D88:D88)</f>
+      <c r="D92" s="6">
+        <f>SUM(D91:D91)</f>
         <v>0</v>
       </c>
-      <c r="E89" s="6">
-        <f>SUM(E88:E88)</f>
+      <c r="E92" s="6">
+        <f>SUM(E91:E91)</f>
         <v>0</v>
       </c>
-      <c r="F89" s="6">
-        <f>SUM(F88:F88)</f>
+      <c r="F92" s="6">
+        <f>SUM(F91:F91)</f>
         <v>102.65</v>
       </c>
-      <c r="G89" s="6">
-        <f>SUM(G88:G88)</f>
+      <c r="G92" s="6">
+        <f>F92/4</f>
         <v>25.66</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="5" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Recreation</t>
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="12" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">St. James Marina</t>
         </is>
       </c>
-      <c r="B92" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B95" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C92" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C95" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>33.54</v>
       </c>
-      <c r="D92" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D95" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E92" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E95" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F92" s="3">
-        <f>SUM(B92:E92)</f>
+      <c r="F95" s="3">
+        <f>SUM(B95:E95)</f>
         <v>33.54</v>
       </c>
-      <c r="G92" s="3">
-        <f>F92/4</f>
+      <c r="G95" s="3">
+        <f>F95/4</f>
         <v>8.38</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="12" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Entertainment &amp; Events</t>
         </is>
       </c>
-      <c r="B93" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B96" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C93" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C96" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>400.0</v>
       </c>
-      <c r="D93" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D96" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>13.5</v>
       </c>
-      <c r="E93" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E96" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F93" s="3">
-        <f>SUM(B93:E93)</f>
+      <c r="F96" s="3">
+        <f>SUM(B96:E96)</f>
         <v>413.5</v>
       </c>
-      <c r="G93" s="3">
-        <f>F93/4</f>
+      <c r="G96" s="3">
+        <f>F96/4</f>
         <v>103.38</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="7" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Recreation</t>
         </is>
       </c>
-      <c r="B94" s="6">
-        <f>SUM(B92:B93)</f>
+      <c r="B97" s="6">
+        <f>SUM(B95:B96)</f>
         <v>0</v>
       </c>
-      <c r="C94" s="6">
-        <f>SUM(C92:C93)</f>
+      <c r="C97" s="6">
+        <f>SUM(C95:C96)</f>
         <v>433.54</v>
       </c>
-      <c r="D94" s="6">
-        <f>SUM(D92:D93)</f>
+      <c r="D97" s="6">
+        <f>SUM(D95:D96)</f>
         <v>13.5</v>
       </c>
-      <c r="E94" s="6">
-        <f>SUM(E92:E93)</f>
+      <c r="E97" s="6">
+        <f>SUM(E95:E96)</f>
         <v>0</v>
       </c>
-      <c r="F94" s="6">
-        <f>SUM(F92:F93)</f>
+      <c r="F97" s="6">
+        <f>SUM(F95:F96)</f>
         <v>447.04</v>
       </c>
-      <c r="G94" s="6">
-        <f>SUM(G92:G93)</f>
+      <c r="G97" s="6">
+        <f>F97/4</f>
         <v>111.76</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="5" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="12" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
         </is>
       </c>
-      <c r="B97" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A97,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B100" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>75.0</v>
       </c>
-      <c r="C97" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A97,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C100" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>764.05</v>
       </c>
-      <c r="D97" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A97,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D100" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>331.5</v>
       </c>
-      <c r="E97" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A97,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E100" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>130.0</v>
       </c>
-      <c r="F97" s="3">
-        <f>SUM(B97:E97)</f>
+      <c r="F100" s="3">
+        <f>SUM(B100:E100)</f>
         <v>1300.55</v>
       </c>
-      <c r="G97" s="3">
-        <f>F97/4</f>
+      <c r="G100" s="3">
+        <f>F100/4</f>
         <v>325.14</v>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="7" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Transfers</t>
         </is>
       </c>
-      <c r="B98" s="6">
-        <f>SUM(B97:B97)</f>
+      <c r="B101" s="6">
+        <f>SUM(B100:B100)</f>
         <v>75.0</v>
       </c>
-      <c r="C98" s="6">
-        <f>SUM(C97:C97)</f>
+      <c r="C101" s="6">
+        <f>SUM(C100:C100)</f>
         <v>764.05</v>
       </c>
-      <c r="D98" s="6">
-        <f>SUM(D97:D97)</f>
+      <c r="D101" s="6">
+        <f>SUM(D100:D100)</f>
         <v>331.5</v>
       </c>
-      <c r="E98" s="6">
-        <f>SUM(E97:E97)</f>
+      <c r="E101" s="6">
+        <f>SUM(E100:E100)</f>
         <v>130.0</v>
       </c>
-      <c r="F98" s="6">
-        <f>SUM(F97:F97)</f>
+      <c r="F101" s="6">
+        <f>SUM(F100:F100)</f>
         <v>1300.55</v>
       </c>
-      <c r="G98" s="6">
-        <f>SUM(G97:G97)</f>
+      <c r="G101" s="6">
+        <f>F101/4</f>
         <v>325.14</v>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="5" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Other</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="12" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Donations &amp; Clubs (Kiwanis)</t>
         </is>
       </c>
-      <c r="B101" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A101,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B104" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C101" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A101,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C104" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D101" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A101,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D104" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E101" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A101,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E104" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>200.0</v>
       </c>
-      <c r="F101" s="3">
-        <f>SUM(B101:E101)</f>
+      <c r="F104" s="3">
+        <f>SUM(B104:E104)</f>
         <v>200.0</v>
       </c>
-      <c r="G101" s="3">
-        <f>F101/4</f>
+      <c r="G104" s="3">
+        <f>F104/4</f>
         <v>50.0</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="12" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
         </is>
       </c>
-      <c r="B102" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B105" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C102" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C105" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D102" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D105" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E102" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E105" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>147.0</v>
       </c>
-      <c r="F102" s="3">
-        <f>SUM(B102:E102)</f>
+      <c r="F105" s="3">
+        <f>SUM(B105:E105)</f>
         <v>147.0</v>
       </c>
-      <c r="G102" s="3">
-        <f>F102/4</f>
+      <c r="G105" s="3">
+        <f>F105/4</f>
         <v>36.75</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="7" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Other</t>
         </is>
       </c>
-      <c r="B103" s="6">
-        <f>SUM(B101:B102)</f>
+      <c r="B106" s="6">
+        <f>SUM(B104:B105)</f>
         <v>0</v>
       </c>
-      <c r="C103" s="6">
-        <f>SUM(C101:C102)</f>
+      <c r="C106" s="6">
+        <f>SUM(C104:C105)</f>
         <v>0</v>
       </c>
-      <c r="D103" s="6">
-        <f>SUM(D101:D102)</f>
+      <c r="D106" s="6">
+        <f>SUM(D104:D105)</f>
         <v>0</v>
       </c>
-      <c r="E103" s="6">
-        <f>SUM(E101:E102)</f>
+      <c r="E106" s="6">
+        <f>SUM(E104:E105)</f>
         <v>347.0</v>
       </c>
-      <c r="F103" s="6">
-        <f>SUM(F101:F102)</f>
+      <c r="F106" s="6">
+        <f>SUM(F104:F105)</f>
         <v>347.0</v>
       </c>
-      <c r="G103" s="6">
-        <f>SUM(G101:G102)</f>
+      <c r="G106" s="6">
+        <f>F106/4</f>
         <v>86.75</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="8" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL SPENDING</t>
         </is>
       </c>
-      <c r="B105" s="9">
-        <f>B10+B18+B25+B29+B34+B39+B50+B54+B58+B62+B80+B85+B89+B94+B98+B103</f>
+      <c r="B108" s="9">
+        <f>B10+B18+B23+B28+B32+B37+B42+B53+B57+B61+B65+B83+B88+B92+B97+B101+B106</f>
         <v>12135.81</v>
       </c>
-      <c r="C105" s="9">
-        <f>C10+C18+C25+C29+C34+C39+C50+C54+C58+C62+C80+C85+C89+C94+C98+C103</f>
+      <c r="C108" s="9">
+        <f>C10+C18+C23+C28+C32+C37+C42+C53+C57+C61+C65+C83+C88+C92+C97+C101+C106</f>
         <v>12663.24</v>
       </c>
-      <c r="D105" s="9">
-        <f>D10+D18+D25+D29+D34+D39+D50+D54+D58+D62+D80+D85+D89+D94+D98+D103</f>
+      <c r="D108" s="9">
+        <f>D10+D18+D23+D28+D32+D37+D42+D53+D57+D61+D65+D83+D88+D92+D97+D101+D106</f>
         <v>15086.64</v>
       </c>
-      <c r="E105" s="9">
-        <f>E10+E18+E25+E29+E34+E39+E50+E54+E58+E62+E80+E85+E89+E94+E98+E103</f>
+      <c r="E108" s="9">
+        <f>E10+E18+E23+E28+E32+E37+E42+E53+E57+E61+E65+E83+E88+E92+E97+E101+E106</f>
         <v>11515.63</v>
       </c>
-      <c r="F105" s="9">
-        <f>F10+F18+F25+F29+F34+F39+F50+F54+F58+F62+F80+F85+F89+F94+F98+F103</f>
+      <c r="F108" s="9">
+        <f>F10+F18+F23+F28+F32+F37+F42+F53+F57+F61+F65+F83+F88+F92+F97+F101+F106</f>
         <v>51401.32</v>
       </c>
-      <c r="G105" s="9">
-        <f>G10+G18+G25+G29+G34+G39+G50+G54+G58+G62+G80+G85+G89+G94+G98+G103</f>
-        <v>12850.35</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="5" t="inlineStr">
+      <c r="G108" s="9">
+        <f>F108/4</f>
+        <v>12850.33</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Not counted as spending</t>
         </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
-        </is>
-      </c>
-      <c r="B108" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="C108" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="D108" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="E108" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="F108" s="3">
-        <f>SUM(B108:E108)</f>
-        <v>10304.0</v>
-      </c>
-      <c r="G108" s="3">
-        <f>F108/4</f>
-        <v>2576.0</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
-        </is>
-      </c>
-      <c r="B109" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C109" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>7227.09</v>
-      </c>
-      <c r="D109" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>4593.08</v>
-      </c>
-      <c r="E109" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>4738.51</v>
-      </c>
-      <c r="F109" s="3">
-        <f>SUM(B109:E109)</f>
-        <v>16558.68</v>
-      </c>
-      <c r="G109" s="3">
-        <f>F109/4</f>
-        <v>4139.67</v>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sloane Realty</t>
-        </is>
-      </c>
-      <c r="B110" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A110,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C110" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A110,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2891.98</v>
-      </c>
-      <c r="D110" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A110,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E110" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A110,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F110" s="3">
-        <f>SUM(B110:E110)</f>
-        <v>2891.98</v>
-      </c>
-      <c r="G110" s="3">
-        <f>F110/4</f>
-        <v>723.0</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checks Written (payee not shown)</t>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
         </is>
       </c>
       <c r="B111" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2630.0</v>
+        <v>2576.0</v>
       </c>
       <c r="C111" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>2576.0</v>
       </c>
       <c r="D111" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>728.0</v>
+        <v>2576.0</v>
       </c>
       <c r="E111" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>2576.0</v>
       </c>
       <c r="F111" s="3">
         <f>SUM(B111:E111)</f>
-        <v>3358.0</v>
+        <v>10304.0</v>
       </c>
       <c r="G111" s="3">
         <f>F111/4</f>
-        <v>839.5</v>
+        <v>2576.0</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="B112" s="3">
@@ -2611,707 +2556,831 @@
       </c>
       <c r="C112" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3.26</v>
+        <v>7227.09</v>
       </c>
       <c r="D112" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>4593.08</v>
       </c>
       <c r="E112" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>4738.51</v>
       </c>
       <c r="F112" s="3">
         <f>SUM(B112:E112)</f>
-        <v>3.26</v>
+        <v>16558.68</v>
       </c>
       <c r="G112" s="3">
         <f>F112/4</f>
-        <v>0.81</v>
+        <v>4139.67</v>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total not counted as spending</t>
-        </is>
-      </c>
-      <c r="B113" s="6">
-        <f>SUM(B108:B112)</f>
-        <v>5206.0</v>
-      </c>
-      <c r="C113" s="6">
-        <f>SUM(C108:C112)</f>
-        <v>12698.33</v>
-      </c>
-      <c r="D113" s="6">
-        <f>SUM(D108:D112)</f>
-        <v>7897.08</v>
-      </c>
-      <c r="E113" s="6">
-        <f>SUM(E108:E112)</f>
-        <v>7314.51</v>
-      </c>
-      <c r="F113" s="6">
-        <f>SUM(F108:F112)</f>
-        <v>33115.92</v>
-      </c>
-      <c r="G113" s="6">
-        <f>SUM(G108:G112)</f>
-        <v>8278.98</v>
+      <c r="A113" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sloane Realty</t>
+        </is>
+      </c>
+      <c r="B113" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C113" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>2891.98</v>
+      </c>
+      <c r="D113" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E113" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F113" s="3">
+        <f>SUM(B113:E113)</f>
+        <v>2891.98</v>
+      </c>
+      <c r="G113" s="3">
+        <f>F113/4</f>
+        <v>723.0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Checks Written (payee not shown)</t>
+        </is>
+      </c>
+      <c r="B114" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>2630.0</v>
+      </c>
+      <c r="C114" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D114" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>728.0</v>
+      </c>
+      <c r="E114" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F114" s="3">
+        <f>SUM(B114:E114)</f>
+        <v>3358.0</v>
+      </c>
+      <c r="G114" s="3">
+        <f>F114/4</f>
+        <v>839.5</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
+        </is>
+      </c>
+      <c r="B115" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A115,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C115" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A115,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>3.26</v>
+      </c>
+      <c r="D115" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A115,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E115" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A115,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F115" s="3">
+        <f>SUM(B115:E115)</f>
+        <v>3.26</v>
+      </c>
+      <c r="G115" s="3">
+        <f>F115/4</f>
+        <v>0.81</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total not counted as spending</t>
+        </is>
+      </c>
+      <c r="B116" s="6">
+        <f>SUM(B111:B115)</f>
+        <v>5206.0</v>
+      </c>
+      <c r="C116" s="6">
+        <f>SUM(C111:C115)</f>
+        <v>12698.33</v>
+      </c>
+      <c r="D116" s="6">
+        <f>SUM(D111:D115)</f>
+        <v>7897.08</v>
+      </c>
+      <c r="E116" s="6">
+        <f>SUM(E111:E115)</f>
+        <v>7314.51</v>
+      </c>
+      <c r="F116" s="6">
+        <f>SUM(F111:F115)</f>
+        <v>33115.92</v>
+      </c>
+      <c r="G116" s="6">
+        <f>F116/4</f>
+        <v>8278.98</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Check: spending + not-counted items</t>
         </is>
       </c>
-      <c r="B115" s="3">
-        <f>B105+B113</f>
+      <c r="B118" s="3">
+        <f>B108+B116</f>
         <v>17341.81</v>
       </c>
-      <c r="C115" s="3">
-        <f>C105+C113</f>
+      <c r="C118" s="3">
+        <f>C108+C116</f>
         <v>25361.57</v>
       </c>
-      <c r="D115" s="3">
-        <f>D105+D113</f>
+      <c r="D118" s="3">
+        <f>D108+D116</f>
         <v>22983.72</v>
       </c>
-      <c r="E115" s="3">
-        <f>E105+E113</f>
+      <c r="E118" s="3">
+        <f>E108+E116</f>
         <v>18830.14</v>
       </c>
-      <c r="F115" s="3">
-        <f>F105+F113</f>
+      <c r="F118" s="3">
+        <f>F108+F116</f>
         <v>84517.24</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="12" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
         </is>
       </c>
-      <c r="B116" s="13">
+      <c r="B119" s="13">
         <v>17341.81</v>
       </c>
-      <c r="C116" s="13">
+      <c r="C119" s="13">
         <v>25361.57</v>
       </c>
-      <c r="D116" s="13">
+      <c r="D119" s="13">
         <v>22983.72</v>
       </c>
-      <c r="E116" s="13">
+      <c r="E119" s="13">
         <v>18830.14</v>
       </c>
-      <c r="F116" s="3">
-        <f>SUM(B116:E116)</f>
+      <c r="F119" s="3">
+        <f>SUM(B119:E119)</f>
         <v>84517.24</v>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="12" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Difference (should be $0 = every dollar accounted for)</t>
         </is>
       </c>
-      <c r="B117" s="3">
-        <f>B115-B116</f>
+      <c r="B120" s="3">
+        <f>B118-B119</f>
         <v>0.0</v>
       </c>
-      <c r="C117" s="3">
-        <f>C115-C116</f>
+      <c r="C120" s="3">
+        <f>C118-C119</f>
         <v>0.0</v>
       </c>
-      <c r="D117" s="3">
-        <f>D115-D116</f>
+      <c r="D120" s="3">
+        <f>D118-D119</f>
         <v>0.0</v>
       </c>
-      <c r="E117" s="3">
-        <f>E115-E116</f>
+      <c r="E120" s="3">
+        <f>E118-E119</f>
         <v>0.0</v>
       </c>
-      <c r="F117" s="3">
-        <f>F115-F116</f>
+      <c r="F120" s="3">
+        <f>F118-F119</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="5" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Key Bills at a Glance</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="15" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Bill</t>
         </is>
       </c>
-      <c r="B120" s="1" t="inlineStr">
+      <c r="B123" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">June 2026</t>
         </is>
       </c>
-      <c r="C120" s="1" t="inlineStr">
+      <c r="C123" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">July 2026</t>
         </is>
       </c>
-      <c r="D120" s="1" t="inlineStr">
+      <c r="D123" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">August 2026</t>
         </is>
       </c>
-      <c r="E120" s="1" t="inlineStr">
+      <c r="E123" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">September 2026</t>
         </is>
       </c>
-      <c r="F120" s="1" t="inlineStr">
+      <c r="F123" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">4-Month Total</t>
         </is>
       </c>
-      <c r="G120" s="1" t="inlineStr">
+      <c r="G123" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Monthly Avg</t>
         </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A&amp;D Mortgage</t>
-        </is>
-      </c>
-      <c r="B121" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="C121" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="D121" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="E121" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="F121" s="3">
-        <f>SUM(B121:E121)</f>
-        <v>13644.4</v>
-      </c>
-      <c r="G121" s="3">
-        <f>F121/4</f>
-        <v>3411.1</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">St. James Membership (Club)</t>
-        </is>
-      </c>
-      <c r="B122" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1591.78</v>
-      </c>
-      <c r="C122" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>1601.56</v>
-      </c>
-      <c r="D122" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1492.11</v>
-      </c>
-      <c r="E122" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>1767.0</v>
-      </c>
-      <c r="F122" s="3">
-        <f>SUM(B122:E122)</f>
-        <v>6452.45</v>
-      </c>
-      <c r="G122" s="3">
-        <f>F122/4</f>
-        <v>1613.11</v>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">St. James Plantation POA Dues</t>
-        </is>
-      </c>
-      <c r="B123" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>692.95</v>
-      </c>
-      <c r="C123" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D123" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E123" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F123" s="3">
-        <f>SUM(B123:E123)</f>
-        <v>692.95</v>
-      </c>
-      <c r="G123" s="3">
-        <f>F123/4</f>
-        <v>173.24</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">A&amp;D Mortgage</t>
         </is>
       </c>
       <c r="B124" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>360.42</v>
+        <v>3411.1</v>
       </c>
       <c r="C124" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>360.42</v>
+        <v>3411.1</v>
       </c>
       <c r="D124" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>475.42</v>
+        <v>3411.1</v>
       </c>
       <c r="E124" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>354.17</v>
+        <v>3411.1</v>
       </c>
       <c r="F124" s="3">
         <f>SUM(B124:E124)</f>
-        <v>1550.43</v>
+        <v>13644.4</v>
       </c>
       <c r="G124" s="3">
         <f>F124/4</f>
-        <v>387.61</v>
+        <v>3411.1</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">St. James Membership (Club)</t>
         </is>
       </c>
       <c r="B125" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A125,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>79.21</v>
+        <v>1591.78</v>
       </c>
       <c r="C125" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A125,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>73.61</v>
+        <v>1601.56</v>
       </c>
       <c r="D125" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A125,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>73.61</v>
+        <v>1492.11</v>
       </c>
       <c r="E125" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A125,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>73.61</v>
+        <v>1767.0</v>
       </c>
       <c r="F125" s="3">
         <f>SUM(B125:E125)</f>
-        <v>300.04</v>
+        <v>6452.45</v>
       </c>
       <c r="G125" s="3">
         <f>F125/4</f>
-        <v>75.01</v>
+        <v>1613.11</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Banner Life Insurance</t>
+          <t xml:space="preserve">St. James Plantation POA Dues</t>
         </is>
       </c>
       <c r="B126" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>710.06</v>
+        <v>692.95</v>
       </c>
       <c r="C126" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>710.06</v>
+        <v>0</v>
       </c>
       <c r="D126" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>710.06</v>
+        <v>0</v>
       </c>
       <c r="E126" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>710.06</v>
+        <v>0</v>
       </c>
       <c r="F126" s="3">
         <f>SUM(B126:E126)</f>
-        <v>2840.24</v>
+        <v>692.95</v>
       </c>
       <c r="G126" s="3">
         <f>F126/4</f>
-        <v>710.06</v>
+        <v>173.24</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="B127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>360.42</v>
       </c>
       <c r="C127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>360.42</v>
       </c>
       <c r="D127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>475.42</v>
       </c>
       <c r="E127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>354.17</v>
       </c>
       <c r="F127" s="3">
         <f>SUM(B127:E127)</f>
-        <v>1412.24</v>
+        <v>1550.43</v>
       </c>
       <c r="G127" s="3">
         <f>F127/4</f>
-        <v>353.06</v>
+        <v>387.61</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="B128" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>79.21</v>
       </c>
       <c r="C128" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>73.61</v>
       </c>
       <c r="D128" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>73.61</v>
       </c>
       <c r="E128" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>73.61</v>
       </c>
       <c r="F128" s="3">
         <f>SUM(B128:E128)</f>
-        <v>1162.97</v>
+        <v>300.04</v>
       </c>
       <c r="G128" s="3">
         <f>F128/4</f>
-        <v>290.74</v>
+        <v>75.01</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Banner Life Insurance</t>
         </is>
       </c>
       <c r="B129" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A129,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>710.06</v>
       </c>
       <c r="C129" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A129,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>710.06</v>
       </c>
       <c r="D129" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A129,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>710.06</v>
       </c>
       <c r="E129" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A129,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>710.06</v>
       </c>
       <c r="F129" s="3">
         <f>SUM(B129:E129)</f>
-        <v>342.43</v>
+        <v>2840.24</v>
       </c>
       <c r="G129" s="3">
         <f>F129/4</f>
-        <v>85.61</v>
+        <v>710.06</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B130" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A130,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
+        <v>294.57</v>
       </c>
       <c r="C130" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A130,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>294.8</v>
       </c>
       <c r="D130" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A130,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
+        <v>436.02</v>
       </c>
       <c r="E130" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A130,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
+        <v>386.85</v>
       </c>
       <c r="F130" s="3">
         <f>SUM(B130:E130)</f>
-        <v>323.16</v>
+        <v>1412.24</v>
       </c>
       <c r="G130" s="3">
         <f>F130/4</f>
-        <v>80.79</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B131" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <v>0</v>
       </c>
       <c r="C131" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>935.1</v>
+        <v>336.35</v>
       </c>
       <c r="D131" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <v>406.96</v>
       </c>
       <c r="E131" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>872.56</v>
+        <v>419.66</v>
       </c>
       <c r="F131" s="3">
         <f>SUM(B131:E131)</f>
-        <v>3789.73</v>
+        <v>1162.97</v>
       </c>
       <c r="G131" s="3">
         <f>F131/4</f>
-        <v>947.43</v>
+        <v>290.74</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
         </is>
       </c>
       <c r="B132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>78.84</v>
       </c>
       <c r="C132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>0</v>
       </c>
       <c r="D132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>179.33</v>
       </c>
       <c r="E132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>84.26</v>
       </c>
       <c r="F132" s="3">
         <f>SUM(B132:E132)</f>
-        <v>792.99</v>
+        <v>342.43</v>
       </c>
       <c r="G132" s="3">
         <f>F132/4</f>
-        <v>198.25</v>
+        <v>85.61</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Groceries</t>
+          <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
       <c r="B133" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1529.75</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
       </c>
       <c r="C133" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>1279.24</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>336.35</v>
       </c>
       <c r="D133" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1190.12</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>586.29</v>
       </c>
       <c r="E133" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>1202.5</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>503.92</v>
       </c>
       <c r="F133" s="3">
         <f>SUM(B133:E133)</f>
-        <v>5201.61</v>
+        <v>1505.4</v>
       </c>
       <c r="G133" s="3">
         <f>F133/4</f>
-        <v>1300.4</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
+        </is>
+      </c>
+      <c r="B134" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>80.79</v>
+      </c>
+      <c r="C134" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D134" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>161.58</v>
+      </c>
+      <c r="E134" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>80.79</v>
+      </c>
+      <c r="F134" s="3">
+        <f>SUM(B134:E134)</f>
+        <v>323.16</v>
+      </c>
+      <c r="G134" s="3">
+        <f>F134/4</f>
+        <v>80.79</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+        </is>
+      </c>
+      <c r="B135" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>1019.45</v>
+      </c>
+      <c r="C135" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>935.1</v>
+      </c>
+      <c r="D135" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>962.62</v>
+      </c>
+      <c r="E135" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>872.56</v>
+      </c>
+      <c r="F135" s="3">
+        <f>SUM(B135:E135)</f>
+        <v>3789.73</v>
+      </c>
+      <c r="G135" s="3">
+        <f>F135/4</f>
+        <v>947.43</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B136" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C136" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D136" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E136" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F136" s="3">
+        <f>SUM(B136:E136)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G136" s="3">
+        <f>F136/4</f>
+        <v>198.25</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Groceries</t>
+        </is>
+      </c>
+      <c r="B137" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>1529.75</v>
+      </c>
+      <c r="C137" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>1279.24</v>
+      </c>
+      <c r="D137" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>1190.12</v>
+      </c>
+      <c r="E137" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>1202.5</v>
+      </c>
+      <c r="F137" s="3">
+        <f>SUM(B137:E137)</f>
+        <v>5201.61</v>
+      </c>
+      <c r="G137" s="3">
+        <f>F137/4</f>
+        <v>1300.4</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B134" s="3">
+      <c r="B138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C134" s="3">
+      <c r="C138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D134" s="3">
+      <c r="D138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E134" s="3">
+      <c r="E138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>333.11</v>
       </c>
-      <c r="F134" s="3">
-        <f>SUM(B134:E134)</f>
+      <c r="F138" s="3">
+        <f>SUM(B138:E138)</f>
         <v>4679.18</v>
       </c>
-      <c r="G134" s="3">
-        <f>F134/4</f>
+      <c r="G138" s="3">
+        <f>F138/4</f>
         <v>1169.8</v>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="12" t="inlineStr">
+    <row r="139">
+      <c r="A139" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B135" s="3">
+      <c r="B139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C135" s="3">
+      <c r="C139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D135" s="3">
+      <c r="D139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E135" s="3">
+      <c r="E139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F135" s="3">
-        <f>SUM(B135:E135)</f>
+      <c r="F139" s="3">
+        <f>SUM(B139:E139)</f>
         <v>737.73</v>
       </c>
-      <c r="G135" s="3">
-        <f>F135/4</f>
+      <c r="G139" s="3">
+        <f>F139/4</f>
         <v>184.43</v>
       </c>
     </row>
-    <row r="137">
-      <c r="A137" s="5" t="inlineStr">
+    <row r="141">
+      <c r="A141" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="27" customHeight="1">
-      <c r="A138" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="27" customHeight="1">
-      <c r="A139" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="27" customHeight="1">
-      <c r="A140" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="27" customHeight="1">
-      <c r="A141" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="142" ht="27" customHeight="1">
       <c r="A142" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities identified: BEMC = Brunswick Electric Membership Corp (electric); OPC*Brunswick CO U = Brunswick County Utilities (water/sewer) + $2.95 online-payment fee; Focus Broadband (internet). Verizon Wireless shown separately.</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="143" ht="27" customHeight="1">
       <c r="A143" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="144" ht="27" customHeight="1">
       <c r="A144" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="27" customHeight="1">
+      <c r="A145" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="27" customHeight="1">
+      <c r="A146" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="27" customHeight="1">
+      <c r="A147" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="27" customHeight="1">
+      <c r="A148" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Small hospital-cafeteria charges (Granville Med, Duke) are counted as Restaurants.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A138:G138"/>
-    <mergeCell ref="A139:G139"/>
-    <mergeCell ref="A140:G140"/>
-    <mergeCell ref="A141:G141"/>
     <mergeCell ref="A142:G142"/>
     <mergeCell ref="A143:G143"/>
     <mergeCell ref="A144:G144"/>
+    <mergeCell ref="A145:G145"/>
+    <mergeCell ref="A146:G146"/>
+    <mergeCell ref="A147:G147"/>
+    <mergeCell ref="A148:G148"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -4008,7 +4077,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="H23" s="3">
@@ -4678,12 +4747,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="E45" s="3">
@@ -6316,7 +6385,7 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="E116" s="3">
@@ -9441,7 +9510,7 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="E118" s="3">
@@ -10140,12 +10209,12 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="E16" s="3">
@@ -10409,7 +10478,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="H24" s="3">
@@ -11470,12 +11539,12 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="E63" s="3">
@@ -12464,7 +12533,7 @@
       </c>
       <c r="D106" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="E106" s="3">
@@ -13349,7 +13418,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="H25" s="3">
@@ -13928,12 +13997,12 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="E45" s="3">
@@ -14692,7 +14761,7 @@
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="E78" s="3">
@@ -16183,12 +16252,12 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="F46" s="3">
@@ -18176,7 +18245,7 @@
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="F117" s="3">
@@ -21480,7 +21549,7 @@
       </c>
       <c r="E235" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="F235" s="3">
@@ -22091,12 +22160,12 @@
       </c>
       <c r="D257" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="E257" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="F257" s="3">
@@ -23407,12 +23476,12 @@
       </c>
       <c r="D304" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="F304" s="3">
@@ -24616,7 +24685,7 @@
       </c>
       <c r="E347" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="F347" s="3">
@@ -25899,12 +25968,12 @@
       </c>
       <c r="D393" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Internet (Focus Broadband)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="E393" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="F393" s="3">
@@ -26828,7 +26897,7 @@
       </c>
       <c r="E426" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities</t>
+          <t xml:space="preserve">Phone &amp; Internet</t>
         </is>
       </c>
       <c r="F426" s="3">

</xml_diff>

<commit_message>
Add Haircuts – The Color Bar line item
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -1606,7 +1606,7 @@
     <row r="70">
       <c r="A70" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="B70" s="3">
@@ -1623,130 +1623,130 @@
       </c>
       <c r="E70" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>114.5</v>
+        <v>32.5</v>
       </c>
       <c r="F70" s="3">
         <f>SUM(B70:E70)</f>
-        <v>479.5</v>
+        <v>397.5</v>
       </c>
       <c r="G70" s="3">
         <f>F70/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Personal Care – Simple Beauty</t>
+        </is>
+      </c>
+      <c r="B71" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C71" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D71" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E71" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>82.0</v>
+      </c>
+      <c r="F71" s="3">
+        <f>SUM(B71:E71)</f>
+        <v>82.0</v>
+      </c>
+      <c r="G71" s="3">
+        <f>F71/4</f>
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Personal</t>
+        </is>
+      </c>
+      <c r="B72" s="6">
+        <f>SUM(B70:B71)</f>
+        <v>182.5</v>
+      </c>
+      <c r="C72" s="6">
+        <f>SUM(C70:C71)</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="6">
+        <f>SUM(D70:D71)</f>
+        <v>182.5</v>
+      </c>
+      <c r="E72" s="6">
+        <f>SUM(E70:E71)</f>
+        <v>114.5</v>
+      </c>
+      <c r="F72" s="6">
+        <f>SUM(F70:F71)</f>
+        <v>479.5</v>
+      </c>
+      <c r="G72" s="6">
+        <f>F72/4</f>
         <v>119.875</v>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Personal</t>
-        </is>
-      </c>
-      <c r="B71" s="6">
-        <f>SUM(B70:B70)</f>
-        <v>182.5</v>
-      </c>
-      <c r="C71" s="6">
-        <f>SUM(C70:C70)</f>
-        <v>0</v>
-      </c>
-      <c r="D71" s="6">
-        <f>SUM(D70:D70)</f>
-        <v>182.5</v>
-      </c>
-      <c r="E71" s="6">
-        <f>SUM(E70:E70)</f>
-        <v>114.5</v>
-      </c>
-      <c r="F71" s="6">
-        <f>SUM(F70:F70)</f>
-        <v>479.5</v>
-      </c>
-      <c r="G71" s="6">
-        <f>F71/4</f>
-        <v>119.875</v>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="5" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Retail</t>
         </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Walmart</t>
-        </is>
-      </c>
-      <c r="B74" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C74" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>132.66</v>
-      </c>
-      <c r="D74" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1732.6</v>
-      </c>
-      <c r="E74" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.63</v>
-      </c>
-      <c r="F74" s="3">
-        <f>SUM(B74:E74)</f>
-        <v>1897.89</v>
-      </c>
-      <c r="G74" s="3">
-        <f>F74/4</f>
-        <v>474.4725</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Belk (store card payments)</t>
+          <t xml:space="preserve">Retail – Walmart</t>
         </is>
       </c>
       <c r="B75" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>386.69</v>
+        <v>0</v>
       </c>
       <c r="C75" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>948.04</v>
+        <v>132.66</v>
       </c>
       <c r="D75" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1732.6</v>
       </c>
       <c r="E75" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>32.63</v>
       </c>
       <c r="F75" s="3">
         <f>SUM(B75:E75)</f>
-        <v>1334.73</v>
+        <v>1897.89</v>
       </c>
       <c r="G75" s="3">
         <f>F75/4</f>
-        <v>333.6825</v>
+        <v>474.4725</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Marshalls</t>
+          <t xml:space="preserve">Retail – Belk (store card payments)</t>
         </is>
       </c>
       <c r="B76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>386.69</v>
       </c>
       <c r="C76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>948.04</v>
       </c>
       <c r="D76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,D$4)</f>
@@ -1754,26 +1754,26 @@
       </c>
       <c r="E76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>41.59</v>
+        <v>0</v>
       </c>
       <c r="F76" s="3">
         <f>SUM(B76:E76)</f>
-        <v>41.59</v>
+        <v>1334.73</v>
       </c>
       <c r="G76" s="3">
         <f>F76/4</f>
-        <v>10.3975</v>
+        <v>333.6825</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ross</t>
+          <t xml:space="preserve">Retail – Marshalls</t>
         </is>
       </c>
       <c r="B77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>48.03</v>
+        <v>0</v>
       </c>
       <c r="C77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1785,26 +1785,26 @@
       </c>
       <c r="E77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>16.32</v>
+        <v>41.59</v>
       </c>
       <c r="F77" s="3">
         <f>SUM(B77:E77)</f>
-        <v>64.35</v>
+        <v>41.59</v>
       </c>
       <c r="G77" s="3">
         <f>F77/4</f>
-        <v>16.0875</v>
+        <v>10.3975</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dillard's</t>
+          <t xml:space="preserve">Retail – Ross</t>
         </is>
       </c>
       <c r="B78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>48.03</v>
       </c>
       <c r="C78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1812,30 +1812,30 @@
       </c>
       <c r="D78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>174.74</v>
+        <v>0</v>
       </c>
       <c r="E78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>16.32</v>
       </c>
       <c r="F78" s="3">
         <f>SUM(B78:E78)</f>
-        <v>174.74</v>
+        <v>64.35</v>
       </c>
       <c r="G78" s="3">
         <f>F78/4</f>
-        <v>43.685</v>
+        <v>16.0875</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Target</t>
+          <t xml:space="preserve">Retail – Dillard's</t>
         </is>
       </c>
       <c r="B79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>58.98</v>
+        <v>0</v>
       </c>
       <c r="C79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="D79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>174.74</v>
       </c>
       <c r="E79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1851,22 +1851,22 @@
       </c>
       <c r="F79" s="3">
         <f>SUM(B79:E79)</f>
-        <v>58.98</v>
+        <v>174.74</v>
       </c>
       <c r="G79" s="3">
         <f>F79/4</f>
-        <v>14.745</v>
+        <v>43.685</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – HomeSense</t>
+          <t xml:space="preserve">Retail – Target</t>
         </is>
       </c>
       <c r="B80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>58.98</v>
       </c>
       <c r="C80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="D80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>88.7</v>
+        <v>0</v>
       </c>
       <c r="E80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1882,17 +1882,17 @@
       </c>
       <c r="F80" s="3">
         <f>SUM(B80:E80)</f>
-        <v>88.7</v>
+        <v>58.98</v>
       </c>
       <c r="G80" s="3">
         <f>F80/4</f>
-        <v>22.175</v>
+        <v>14.745</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Hobby Lobby</t>
+          <t xml:space="preserve">Retail – HomeSense</t>
         </is>
       </c>
       <c r="B81" s="3">
@@ -1905,30 +1905,30 @@
       </c>
       <c r="D81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>165.67</v>
+        <v>88.7</v>
       </c>
       <c r="E81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>37.33</v>
+        <v>0</v>
       </c>
       <c r="F81" s="3">
         <f>SUM(B81:E81)</f>
-        <v>203.0</v>
+        <v>88.7</v>
       </c>
       <c r="G81" s="3">
         <f>F81/4</f>
-        <v>50.75</v>
+        <v>22.175</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
+          <t xml:space="preserve">Retail – Hobby Lobby</t>
         </is>
       </c>
       <c r="B82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>27.67</v>
+        <v>0</v>
       </c>
       <c r="C82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1936,30 +1936,30 @@
       </c>
       <c r="D82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>171.55</v>
+        <v>165.67</v>
       </c>
       <c r="E82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>85.27</v>
+        <v>37.33</v>
       </c>
       <c r="F82" s="3">
         <f>SUM(B82:E82)</f>
-        <v>284.49</v>
+        <v>203.0</v>
       </c>
       <c r="G82" s="3">
         <f>F82/4</f>
-        <v>71.1225</v>
+        <v>50.75</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Tractor Supply</t>
+          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
         </is>
       </c>
       <c r="B83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>27.67</v>
       </c>
       <c r="C83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1967,25 +1967,25 @@
       </c>
       <c r="D83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>29.86</v>
+        <v>171.55</v>
       </c>
       <c r="E83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>85.27</v>
       </c>
       <c r="F83" s="3">
         <f>SUM(B83:E83)</f>
-        <v>29.86</v>
+        <v>284.49</v>
       </c>
       <c r="G83" s="3">
         <f>F83/4</f>
-        <v>7.465</v>
+        <v>71.1225</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
+          <t xml:space="preserve">Retail – Tractor Supply</t>
         </is>
       </c>
       <c r="B84" s="3">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="C84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>63.61</v>
+        <v>0</v>
       </c>
       <c r="D84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>29.86</v>
       </c>
       <c r="E84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2006,26 +2006,26 @@
       </c>
       <c r="F84" s="3">
         <f>SUM(B84:E84)</f>
-        <v>63.61</v>
+        <v>29.86</v>
       </c>
       <c r="G84" s="3">
         <f>F84/4</f>
-        <v>15.9025</v>
+        <v>7.465</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ulta Beauty</t>
+          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
         </is>
       </c>
       <c r="B85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>134.71</v>
+        <v>0</v>
       </c>
       <c r="C85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>63.61</v>
       </c>
       <c r="D85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,D$4)</f>
@@ -2037,22 +2037,22 @@
       </c>
       <c r="F85" s="3">
         <f>SUM(B85:E85)</f>
-        <v>134.71</v>
+        <v>63.61</v>
       </c>
       <c r="G85" s="3">
         <f>F85/4</f>
-        <v>33.6775</v>
+        <v>15.9025</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
+          <t xml:space="preserve">Retail – Ulta Beauty</t>
         </is>
       </c>
       <c r="B86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>51.31</v>
+        <v>134.71</v>
       </c>
       <c r="C86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -2068,30 +2068,30 @@
       </c>
       <c r="F86" s="3">
         <f>SUM(B86:E86)</f>
-        <v>51.31</v>
+        <v>134.71</v>
       </c>
       <c r="G86" s="3">
         <f>F86/4</f>
-        <v>12.8275</v>
+        <v>33.6775</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
         </is>
       </c>
       <c r="B87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>51.31</v>
       </c>
       <c r="C87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>5.87</v>
+        <v>0</v>
       </c>
       <c r="D87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>17.35</v>
+        <v>0</v>
       </c>
       <c r="E87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2099,286 +2099,286 @@
       </c>
       <c r="F87" s="3">
         <f>SUM(B87:E87)</f>
-        <v>23.22</v>
+        <v>51.31</v>
       </c>
       <c r="G87" s="3">
         <f>F87/4</f>
-        <v>5.805</v>
+        <v>12.8275</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
         </is>
       </c>
       <c r="B88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.03</v>
+        <v>0</v>
       </c>
       <c r="C88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>5.87</v>
       </c>
       <c r="D88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>17.35</v>
       </c>
       <c r="E88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>119.97</v>
+        <v>0</v>
       </c>
       <c r="F88" s="3">
         <f>SUM(B88:E88)</f>
-        <v>228.0</v>
+        <v>23.22</v>
       </c>
       <c r="G88" s="3">
         <f>F88/4</f>
+        <v>5.805</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+        </is>
+      </c>
+      <c r="B89" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.03</v>
+      </c>
+      <c r="C89" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D89" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E89" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>119.97</v>
+      </c>
+      <c r="F89" s="3">
+        <f>SUM(B89:E89)</f>
+        <v>228.0</v>
+      </c>
+      <c r="G89" s="3">
+        <f>F89/4</f>
         <v>57.0</v>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="7" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Retail</t>
         </is>
       </c>
-      <c r="B89" s="6">
-        <f>SUM(B74:B88)</f>
+      <c r="B90" s="6">
+        <f>SUM(B75:B89)</f>
         <v>815.42</v>
       </c>
-      <c r="C89" s="6">
-        <f>SUM(C74:C88)</f>
+      <c r="C90" s="6">
+        <f>SUM(C75:C89)</f>
         <v>1150.18</v>
       </c>
-      <c r="D89" s="6">
-        <f>SUM(D74:D88)</f>
+      <c r="D90" s="6">
+        <f>SUM(D75:D89)</f>
         <v>2380.47</v>
       </c>
-      <c r="E89" s="6">
-        <f>SUM(E74:E88)</f>
+      <c r="E90" s="6">
+        <f>SUM(E75:E89)</f>
         <v>333.11</v>
       </c>
-      <c r="F89" s="6">
-        <f>SUM(F74:F88)</f>
+      <c r="F90" s="6">
+        <f>SUM(F75:F89)</f>
         <v>4679.18</v>
       </c>
-      <c r="G89" s="6">
-        <f>F89/4</f>
+      <c r="G90" s="6">
+        <f>F90/4</f>
         <v>1169.795</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="5" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Home</t>
         </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yard Company (NextGen)</t>
-        </is>
-      </c>
-      <c r="B92" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>60.0</v>
-      </c>
-      <c r="C92" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.0</v>
-      </c>
-      <c r="D92" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>220.0</v>
-      </c>
-      <c r="E92" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>120.0</v>
-      </c>
-      <c r="F92" s="3">
-        <f>SUM(B92:E92)</f>
-        <v>500.0</v>
-      </c>
-      <c r="G92" s="3">
-        <f>F92/4</f>
-        <v>125.0</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
       <c r="B93" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>60.0</v>
       </c>
       <c r="C93" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>242.05</v>
+        <v>100.0</v>
       </c>
       <c r="D93" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>536.6</v>
+        <v>220.0</v>
       </c>
       <c r="E93" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>120.0</v>
       </c>
       <c r="F93" s="3">
         <f>SUM(B93:E93)</f>
-        <v>778.65</v>
+        <v>500.0</v>
       </c>
       <c r="G93" s="3">
         <f>F93/4</f>
+        <v>125.0</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+        </is>
+      </c>
+      <c r="B94" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C94" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>242.05</v>
+      </c>
+      <c r="D94" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>536.6</v>
+      </c>
+      <c r="E94" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F94" s="3">
+        <f>SUM(B94:E94)</f>
+        <v>778.65</v>
+      </c>
+      <c r="G94" s="3">
+        <f>F94/4</f>
         <v>194.6625</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="7" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Home</t>
         </is>
       </c>
-      <c r="B94" s="6">
-        <f>SUM(B92:B93)</f>
+      <c r="B95" s="6">
+        <f>SUM(B93:B94)</f>
         <v>60.0</v>
       </c>
-      <c r="C94" s="6">
-        <f>SUM(C92:C93)</f>
+      <c r="C95" s="6">
+        <f>SUM(C93:C94)</f>
         <v>342.05</v>
       </c>
-      <c r="D94" s="6">
-        <f>SUM(D92:D93)</f>
+      <c r="D95" s="6">
+        <f>SUM(D93:D94)</f>
         <v>756.6</v>
       </c>
-      <c r="E94" s="6">
-        <f>SUM(E92:E93)</f>
+      <c r="E95" s="6">
+        <f>SUM(E93:E94)</f>
         <v>120.0</v>
       </c>
-      <c r="F94" s="6">
-        <f>SUM(F92:F93)</f>
+      <c r="F95" s="6">
+        <f>SUM(F93:F94)</f>
         <v>1278.65</v>
       </c>
-      <c r="G94" s="6">
-        <f>F94/4</f>
+      <c r="G95" s="6">
+        <f>F95/4</f>
         <v>319.6625</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="5" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="12" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel (Lyft, Hotel)</t>
         </is>
       </c>
-      <c r="B97" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A97,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B98" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>102.65</v>
       </c>
-      <c r="C97" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A97,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C98" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D97" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A97,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D98" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E97" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A97,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E98" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F97" s="3">
-        <f>SUM(B97:E97)</f>
+      <c r="F98" s="3">
+        <f>SUM(B98:E98)</f>
         <v>102.65</v>
       </c>
-      <c r="G97" s="3">
-        <f>F97/4</f>
-        <v>25.6625</v>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Travel</t>
-        </is>
-      </c>
-      <c r="B98" s="6">
-        <f>SUM(B97:B97)</f>
-        <v>102.65</v>
-      </c>
-      <c r="C98" s="6">
-        <f>SUM(C97:C97)</f>
-        <v>0</v>
-      </c>
-      <c r="D98" s="6">
-        <f>SUM(D97:D97)</f>
-        <v>0</v>
-      </c>
-      <c r="E98" s="6">
-        <f>SUM(E97:E97)</f>
-        <v>0</v>
-      </c>
-      <c r="F98" s="6">
-        <f>SUM(F97:F97)</f>
-        <v>102.65</v>
-      </c>
-      <c r="G98" s="6">
+      <c r="G98" s="3">
         <f>F98/4</f>
         <v>25.6625</v>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="5" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Travel</t>
+        </is>
+      </c>
+      <c r="B99" s="6">
+        <f>SUM(B98:B98)</f>
+        <v>102.65</v>
+      </c>
+      <c r="C99" s="6">
+        <f>SUM(C98:C98)</f>
+        <v>0</v>
+      </c>
+      <c r="D99" s="6">
+        <f>SUM(D98:D98)</f>
+        <v>0</v>
+      </c>
+      <c r="E99" s="6">
+        <f>SUM(E98:E98)</f>
+        <v>0</v>
+      </c>
+      <c r="F99" s="6">
+        <f>SUM(F98:F98)</f>
+        <v>102.65</v>
+      </c>
+      <c r="G99" s="6">
+        <f>F99/4</f>
+        <v>25.6625</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Recreation</t>
         </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">St. James Marina</t>
-        </is>
-      </c>
-      <c r="B101" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A101,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C101" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A101,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>33.54</v>
-      </c>
-      <c r="D101" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A101,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E101" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A101,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F101" s="3">
-        <f>SUM(B101:E101)</f>
-        <v>33.54</v>
-      </c>
-      <c r="G101" s="3">
-        <f>F101/4</f>
-        <v>8.385</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">St. James Marina</t>
         </is>
       </c>
       <c r="B102" s="3">
@@ -2387,11 +2387,11 @@
       </c>
       <c r="C102" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>400.0</v>
+        <v>33.54</v>
       </c>
       <c r="D102" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>13.5</v>
+        <v>0</v>
       </c>
       <c r="E102" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2399,155 +2399,155 @@
       </c>
       <c r="F102" s="3">
         <f>SUM(B102:E102)</f>
-        <v>413.5</v>
+        <v>33.54</v>
       </c>
       <c r="G102" s="3">
         <f>F102/4</f>
+        <v>8.385</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entertainment &amp; Events</t>
+        </is>
+      </c>
+      <c r="B103" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C103" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>400.0</v>
+      </c>
+      <c r="D103" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>13.5</v>
+      </c>
+      <c r="E103" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F103" s="3">
+        <f>SUM(B103:E103)</f>
+        <v>413.5</v>
+      </c>
+      <c r="G103" s="3">
+        <f>F103/4</f>
         <v>103.375</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="7" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Recreation</t>
         </is>
       </c>
-      <c r="B103" s="6">
-        <f>SUM(B101:B102)</f>
+      <c r="B104" s="6">
+        <f>SUM(B102:B103)</f>
         <v>0</v>
       </c>
-      <c r="C103" s="6">
-        <f>SUM(C101:C102)</f>
+      <c r="C104" s="6">
+        <f>SUM(C102:C103)</f>
         <v>433.54</v>
       </c>
-      <c r="D103" s="6">
-        <f>SUM(D101:D102)</f>
+      <c r="D104" s="6">
+        <f>SUM(D102:D103)</f>
         <v>13.5</v>
       </c>
-      <c r="E103" s="6">
-        <f>SUM(E101:E102)</f>
+      <c r="E104" s="6">
+        <f>SUM(E102:E103)</f>
         <v>0</v>
       </c>
-      <c r="F103" s="6">
-        <f>SUM(F101:F102)</f>
+      <c r="F104" s="6">
+        <f>SUM(F102:F103)</f>
         <v>447.04</v>
       </c>
-      <c r="G103" s="6">
-        <f>F103/4</f>
+      <c r="G104" s="6">
+        <f>F104/4</f>
         <v>111.76</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="12" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
         </is>
       </c>
-      <c r="B106" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A106,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B107" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>75.0</v>
       </c>
-      <c r="C106" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A106,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C107" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>764.05</v>
       </c>
-      <c r="D106" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A106,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D107" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>331.5</v>
       </c>
-      <c r="E106" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A106,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E107" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>130.0</v>
       </c>
-      <c r="F106" s="3">
-        <f>SUM(B106:E106)</f>
+      <c r="F107" s="3">
+        <f>SUM(B107:E107)</f>
         <v>1300.55</v>
       </c>
-      <c r="G106" s="3">
-        <f>F106/4</f>
-        <v>325.1375</v>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Transfers</t>
-        </is>
-      </c>
-      <c r="B107" s="6">
-        <f>SUM(B106:B106)</f>
-        <v>75.0</v>
-      </c>
-      <c r="C107" s="6">
-        <f>SUM(C106:C106)</f>
-        <v>764.05</v>
-      </c>
-      <c r="D107" s="6">
-        <f>SUM(D106:D106)</f>
-        <v>331.5</v>
-      </c>
-      <c r="E107" s="6">
-        <f>SUM(E106:E106)</f>
-        <v>130.0</v>
-      </c>
-      <c r="F107" s="6">
-        <f>SUM(F106:F106)</f>
-        <v>1300.55</v>
-      </c>
-      <c r="G107" s="6">
+      <c r="G107" s="3">
         <f>F107/4</f>
         <v>325.1375</v>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="5" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Transfers</t>
+        </is>
+      </c>
+      <c r="B108" s="6">
+        <f>SUM(B107:B107)</f>
+        <v>75.0</v>
+      </c>
+      <c r="C108" s="6">
+        <f>SUM(C107:C107)</f>
+        <v>764.05</v>
+      </c>
+      <c r="D108" s="6">
+        <f>SUM(D107:D107)</f>
+        <v>331.5</v>
+      </c>
+      <c r="E108" s="6">
+        <f>SUM(E107:E107)</f>
+        <v>130.0</v>
+      </c>
+      <c r="F108" s="6">
+        <f>SUM(F107:F107)</f>
+        <v>1300.55</v>
+      </c>
+      <c r="G108" s="6">
+        <f>F108/4</f>
+        <v>325.1375</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Other</t>
         </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Donations &amp; Clubs (Kiwanis)</t>
-        </is>
-      </c>
-      <c r="B110" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A110,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C110" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A110,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D110" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A110,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E110" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A110,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>200.0</v>
-      </c>
-      <c r="F110" s="3">
-        <f>SUM(B110:E110)</f>
-        <v>200.0</v>
-      </c>
-      <c r="G110" s="3">
-        <f>F110/4</f>
-        <v>50.0</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
+          <t xml:space="preserve">Donations &amp; Clubs (Kiwanis)</t>
         </is>
       </c>
       <c r="B111" s="3">
@@ -2564,152 +2564,152 @@
       </c>
       <c r="E111" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>147.0</v>
+        <v>200.0</v>
       </c>
       <c r="F111" s="3">
         <f>SUM(B111:E111)</f>
-        <v>147.0</v>
+        <v>200.0</v>
       </c>
       <c r="G111" s="3">
         <f>F111/4</f>
+        <v>50.0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
+        </is>
+      </c>
+      <c r="B112" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C112" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D112" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E112" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>147.0</v>
+      </c>
+      <c r="F112" s="3">
+        <f>SUM(B112:E112)</f>
+        <v>147.0</v>
+      </c>
+      <c r="G112" s="3">
+        <f>F112/4</f>
         <v>36.75</v>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="7" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Other</t>
         </is>
       </c>
-      <c r="B112" s="6">
-        <f>SUM(B110:B111)</f>
+      <c r="B113" s="6">
+        <f>SUM(B111:B112)</f>
         <v>0</v>
       </c>
-      <c r="C112" s="6">
-        <f>SUM(C110:C111)</f>
+      <c r="C113" s="6">
+        <f>SUM(C111:C112)</f>
         <v>0</v>
       </c>
-      <c r="D112" s="6">
-        <f>SUM(D110:D111)</f>
+      <c r="D113" s="6">
+        <f>SUM(D111:D112)</f>
         <v>0</v>
       </c>
-      <c r="E112" s="6">
-        <f>SUM(E110:E111)</f>
+      <c r="E113" s="6">
+        <f>SUM(E111:E112)</f>
         <v>347.0</v>
       </c>
-      <c r="F112" s="6">
-        <f>SUM(F110:F111)</f>
+      <c r="F113" s="6">
+        <f>SUM(F111:F112)</f>
         <v>347.0</v>
       </c>
-      <c r="G112" s="6">
-        <f>F112/4</f>
+      <c r="G113" s="6">
+        <f>F113/4</f>
         <v>86.75</v>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="8" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL SPENDING</t>
         </is>
       </c>
-      <c r="B114" s="9">
-        <f>B10+B18+B23+B28+B32+B38+B43+B48+B59+B63+B67+B71+B89+B94+B98+B103+B107+B112</f>
+      <c r="B115" s="9">
+        <f>B10+B18+B23+B28+B32+B38+B43+B48+B59+B63+B67+B72+B90+B95+B99+B104+B108+B113</f>
         <v>12135.81</v>
       </c>
-      <c r="C114" s="9">
-        <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C67+C71+C89+C94+C98+C103+C107+C112</f>
+      <c r="C115" s="9">
+        <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C67+C72+C90+C95+C99+C104+C108+C113</f>
         <v>12663.24</v>
       </c>
-      <c r="D114" s="9">
-        <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D67+D71+D89+D94+D98+D103+D107+D112</f>
+      <c r="D115" s="9">
+        <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D67+D72+D90+D95+D99+D104+D108+D113</f>
         <v>15086.64</v>
       </c>
-      <c r="E114" s="9">
-        <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E67+E71+E89+E94+E98+E103+E107+E112</f>
+      <c r="E115" s="9">
+        <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E67+E72+E90+E95+E99+E104+E108+E113</f>
         <v>11515.63</v>
       </c>
-      <c r="F114" s="9">
-        <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F67+F71+F89+F94+F98+F103+F107+F112</f>
+      <c r="F115" s="9">
+        <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F67+F72+F90+F95+F99+F104+F108+F113</f>
         <v>51401.32</v>
       </c>
-      <c r="G114" s="9">
-        <f>F114/4</f>
+      <c r="G115" s="9">
+        <f>F115/4</f>
         <v>12850.33</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="5" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Not counted as spending</t>
         </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
-        </is>
-      </c>
-      <c r="B117" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A117,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="C117" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A117,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="D117" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A117,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="E117" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A117,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="F117" s="3">
-        <f>SUM(B117:E117)</f>
-        <v>10304.0</v>
-      </c>
-      <c r="G117" s="3">
-        <f>F117/4</f>
-        <v>2576.0</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
         </is>
       </c>
       <c r="B118" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A118,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>2576.0</v>
       </c>
       <c r="C118" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A118,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>7227.09</v>
+        <v>2576.0</v>
       </c>
       <c r="D118" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A118,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>4593.08</v>
+        <v>2576.0</v>
       </c>
       <c r="E118" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A118,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>4738.51</v>
+        <v>2576.0</v>
       </c>
       <c r="F118" s="3">
         <f>SUM(B118:E118)</f>
-        <v>16558.68</v>
+        <v>10304.0</v>
       </c>
       <c r="G118" s="3">
         <f>F118/4</f>
-        <v>4139.67</v>
+        <v>2576.0</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sloane Realty</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="B119" s="3">
@@ -2718,42 +2718,42 @@
       </c>
       <c r="C119" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2891.98</v>
+        <v>7227.09</v>
       </c>
       <c r="D119" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>4593.08</v>
       </c>
       <c r="E119" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>4738.51</v>
       </c>
       <c r="F119" s="3">
         <f>SUM(B119:E119)</f>
-        <v>2891.98</v>
+        <v>16558.68</v>
       </c>
       <c r="G119" s="3">
         <f>F119/4</f>
-        <v>722.995</v>
+        <v>4139.67</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checks Written (payee not shown)</t>
+          <t xml:space="preserve">Sloane Realty</t>
         </is>
       </c>
       <c r="B120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2630.0</v>
+        <v>0</v>
       </c>
       <c r="C120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>2891.98</v>
       </c>
       <c r="D120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>728.0</v>
+        <v>0</v>
       </c>
       <c r="E120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2761,30 +2761,30 @@
       </c>
       <c r="F120" s="3">
         <f>SUM(B120:E120)</f>
-        <v>3358.0</v>
+        <v>2891.98</v>
       </c>
       <c r="G120" s="3">
         <f>F120/4</f>
-        <v>839.5</v>
+        <v>722.995</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Checks Written (payee not shown)</t>
         </is>
       </c>
       <c r="B121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>2630.0</v>
       </c>
       <c r="C121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3.26</v>
+        <v>0</v>
       </c>
       <c r="D121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>728.0</v>
       </c>
       <c r="E121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2792,726 +2792,788 @@
       </c>
       <c r="F121" s="3">
         <f>SUM(B121:E121)</f>
-        <v>3.26</v>
+        <v>3358.0</v>
       </c>
       <c r="G121" s="3">
         <f>F121/4</f>
+        <v>839.5</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
+        </is>
+      </c>
+      <c r="B122" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C122" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>3.26</v>
+      </c>
+      <c r="D122" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E122" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F122" s="3">
+        <f>SUM(B122:E122)</f>
+        <v>3.26</v>
+      </c>
+      <c r="G122" s="3">
+        <f>F122/4</f>
         <v>0.815</v>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="7" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total not counted as spending</t>
         </is>
       </c>
-      <c r="B122" s="6">
-        <f>SUM(B117:B121)</f>
+      <c r="B123" s="6">
+        <f>SUM(B118:B122)</f>
         <v>5206.0</v>
       </c>
-      <c r="C122" s="6">
-        <f>SUM(C117:C121)</f>
+      <c r="C123" s="6">
+        <f>SUM(C118:C122)</f>
         <v>12698.33</v>
       </c>
-      <c r="D122" s="6">
-        <f>SUM(D117:D121)</f>
+      <c r="D123" s="6">
+        <f>SUM(D118:D122)</f>
         <v>7897.08</v>
       </c>
-      <c r="E122" s="6">
-        <f>SUM(E117:E121)</f>
+      <c r="E123" s="6">
+        <f>SUM(E118:E122)</f>
         <v>7314.51</v>
       </c>
-      <c r="F122" s="6">
-        <f>SUM(F117:F121)</f>
+      <c r="F123" s="6">
+        <f>SUM(F118:F122)</f>
         <v>33115.92</v>
       </c>
-      <c r="G122" s="6">
-        <f>F122/4</f>
+      <c r="G123" s="6">
+        <f>F123/4</f>
         <v>8278.98</v>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Check: spending + not-counted items</t>
-        </is>
-      </c>
-      <c r="B124" s="3">
-        <f>B114+B122</f>
-        <v>17341.81</v>
-      </c>
-      <c r="C124" s="3">
-        <f>C114+C122</f>
-        <v>25361.57</v>
-      </c>
-      <c r="D124" s="3">
-        <f>D114+D122</f>
-        <v>22983.72</v>
-      </c>
-      <c r="E124" s="3">
-        <f>E114+E122</f>
-        <v>18830.14</v>
-      </c>
-      <c r="F124" s="3">
-        <f>F114+F122</f>
-        <v>84517.24</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
-        </is>
-      </c>
-      <c r="B125" s="13">
+          <t xml:space="preserve">Check: spending + not-counted items</t>
+        </is>
+      </c>
+      <c r="B125" s="3">
+        <f>B115+B123</f>
         <v>17341.81</v>
       </c>
-      <c r="C125" s="13">
+      <c r="C125" s="3">
+        <f>C115+C123</f>
         <v>25361.57</v>
       </c>
-      <c r="D125" s="13">
+      <c r="D125" s="3">
+        <f>D115+D123</f>
         <v>22983.72</v>
       </c>
-      <c r="E125" s="13">
+      <c r="E125" s="3">
+        <f>E115+E123</f>
         <v>18830.14</v>
       </c>
       <c r="F125" s="3">
-        <f>SUM(B125:E125)</f>
+        <f>F115+F123</f>
         <v>84517.24</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
+        </is>
+      </c>
+      <c r="B126" s="13">
+        <v>17341.81</v>
+      </c>
+      <c r="C126" s="13">
+        <v>25361.57</v>
+      </c>
+      <c r="D126" s="13">
+        <v>22983.72</v>
+      </c>
+      <c r="E126" s="13">
+        <v>18830.14</v>
+      </c>
+      <c r="F126" s="3">
+        <f>SUM(B126:E126)</f>
+        <v>84517.24</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Difference (should be $0 = every dollar accounted for)</t>
         </is>
       </c>
-      <c r="B126" s="3">
-        <f>B124-B125</f>
+      <c r="B127" s="3">
+        <f>B125-B126</f>
         <v>0.0</v>
       </c>
-      <c r="C126" s="3">
-        <f>C124-C125</f>
+      <c r="C127" s="3">
+        <f>C125-C126</f>
         <v>0.0</v>
       </c>
-      <c r="D126" s="3">
-        <f>D124-D125</f>
+      <c r="D127" s="3">
+        <f>D125-D126</f>
         <v>0.0</v>
       </c>
-      <c r="E126" s="3">
-        <f>E124-E125</f>
+      <c r="E127" s="3">
+        <f>E125-E126</f>
         <v>0.0</v>
       </c>
-      <c r="F126" s="3">
-        <f>F124-F125</f>
+      <c r="F127" s="3">
+        <f>F125-F126</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="5" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Key Bills at a Glance</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="15" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Bill</t>
         </is>
       </c>
-      <c r="B129" s="1" t="inlineStr">
+      <c r="B130" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">June 2026</t>
         </is>
       </c>
-      <c r="C129" s="1" t="inlineStr">
+      <c r="C130" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">July 2026</t>
         </is>
       </c>
-      <c r="D129" s="1" t="inlineStr">
+      <c r="D130" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">August 2026</t>
         </is>
       </c>
-      <c r="E129" s="1" t="inlineStr">
+      <c r="E130" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">September 2026</t>
         </is>
       </c>
-      <c r="F129" s="1" t="inlineStr">
+      <c r="F130" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">4-Month Total</t>
         </is>
       </c>
-      <c r="G129" s="1" t="inlineStr">
+      <c r="G130" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Monthly Avg</t>
         </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A&amp;D Mortgage</t>
-        </is>
-      </c>
-      <c r="B130" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A130,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="C130" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A130,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="D130" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A130,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="E130" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A130,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="F130" s="3">
-        <f>SUM(B130:E130)</f>
-        <v>13644.4</v>
-      </c>
-      <c r="G130" s="3">
-        <f>F130/4</f>
-        <v>3411.1</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Membership (Club)</t>
+          <t xml:space="preserve">A&amp;D Mortgage</t>
         </is>
       </c>
       <c r="B131" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1591.78</v>
+        <v>3411.1</v>
       </c>
       <c r="C131" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>1601.56</v>
+        <v>3411.1</v>
       </c>
       <c r="D131" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1492.11</v>
+        <v>3411.1</v>
       </c>
       <c r="E131" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>1767.0</v>
+        <v>3411.1</v>
       </c>
       <c r="F131" s="3">
         <f>SUM(B131:E131)</f>
-        <v>6452.45</v>
+        <v>13644.4</v>
       </c>
       <c r="G131" s="3">
         <f>F131/4</f>
-        <v>1613.1125</v>
+        <v>3411.1</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Plantation POA Dues</t>
+          <t xml:space="preserve">St. James Membership (Club)</t>
         </is>
       </c>
       <c r="B132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>692.95</v>
+        <v>1591.78</v>
       </c>
       <c r="C132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>1601.56</v>
       </c>
       <c r="D132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1492.11</v>
       </c>
       <c r="E132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>1767.0</v>
       </c>
       <c r="F132" s="3">
         <f>SUM(B132:E132)</f>
-        <v>692.95</v>
+        <v>6452.45</v>
       </c>
       <c r="G132" s="3">
         <f>F132/4</f>
-        <v>173.2375</v>
+        <v>1613.1125</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">St. James Plantation POA Dues</t>
         </is>
       </c>
       <c r="B133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>360.42</v>
+        <v>692.95</v>
       </c>
       <c r="C133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>360.42</v>
+        <v>0</v>
       </c>
       <c r="D133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>475.42</v>
+        <v>0</v>
       </c>
       <c r="E133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>354.17</v>
+        <v>0</v>
       </c>
       <c r="F133" s="3">
         <f>SUM(B133:E133)</f>
-        <v>1550.43</v>
+        <v>692.95</v>
       </c>
       <c r="G133" s="3">
         <f>F133/4</f>
-        <v>387.6075</v>
+        <v>173.2375</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="B134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>79.21</v>
+        <v>360.42</v>
       </c>
       <c r="C134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>73.61</v>
+        <v>360.42</v>
       </c>
       <c r="D134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>73.61</v>
+        <v>475.42</v>
       </c>
       <c r="E134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>73.61</v>
+        <v>354.17</v>
       </c>
       <c r="F134" s="3">
         <f>SUM(B134:E134)</f>
-        <v>300.04</v>
+        <v>1550.43</v>
       </c>
       <c r="G134" s="3">
         <f>F134/4</f>
-        <v>75.01</v>
+        <v>387.6075</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Banner Life Insurance</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="B135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>710.06</v>
+        <v>79.21</v>
       </c>
       <c r="C135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="D135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="E135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="F135" s="3">
         <f>SUM(B135:E135)</f>
-        <v>2840.24</v>
+        <v>300.04</v>
       </c>
       <c r="G135" s="3">
         <f>F135/4</f>
-        <v>710.06</v>
+        <v>75.01</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Banner Life Insurance</t>
         </is>
       </c>
       <c r="B136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>710.06</v>
       </c>
       <c r="C136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>710.06</v>
       </c>
       <c r="D136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>710.06</v>
       </c>
       <c r="E136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>710.06</v>
       </c>
       <c r="F136" s="3">
         <f>SUM(B136:E136)</f>
-        <v>1412.24</v>
+        <v>2840.24</v>
       </c>
       <c r="G136" s="3">
         <f>F136/4</f>
-        <v>353.06</v>
+        <v>710.06</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>294.57</v>
       </c>
       <c r="C137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>294.8</v>
       </c>
       <c r="D137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>436.02</v>
       </c>
       <c r="E137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>386.85</v>
       </c>
       <c r="F137" s="3">
         <f>SUM(B137:E137)</f>
-        <v>1162.97</v>
+        <v>1412.24</v>
       </c>
       <c r="G137" s="3">
         <f>F137/4</f>
-        <v>290.7425</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>0</v>
       </c>
       <c r="C138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>336.35</v>
       </c>
       <c r="D138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>406.96</v>
       </c>
       <c r="E138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>419.66</v>
       </c>
       <c r="F138" s="3">
         <f>SUM(B138:E138)</f>
-        <v>342.43</v>
+        <v>1162.97</v>
       </c>
       <c r="G138" s="3">
         <f>F138/4</f>
-        <v>85.6075</v>
+        <v>290.7425</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+        </is>
+      </c>
+      <c r="B139" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C139" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D139" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>179.33</v>
+      </c>
+      <c r="E139" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>84.26</v>
+      </c>
+      <c r="F139" s="3">
+        <f>SUM(B139:E139)</f>
+        <v>342.43</v>
+      </c>
+      <c r="G139" s="3">
+        <f>F139/4</f>
+        <v>85.6075</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
-      <c r="B139" s="3">
+      <c r="B140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>78.84</v>
       </c>
-      <c r="C139" s="3">
+      <c r="C140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
-      <c r="D139" s="3">
+      <c r="D140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>586.29</v>
       </c>
-      <c r="E139" s="3">
+      <c r="E140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>503.92</v>
       </c>
-      <c r="F139" s="3">
-        <f>SUM(B139:E139)</f>
-        <v>1505.4</v>
-      </c>
-      <c r="G139" s="3">
-        <f>F139/4</f>
-        <v>376.35</v>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
-        </is>
-      </c>
-      <c r="B140" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="C140" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D140" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
-      </c>
-      <c r="E140" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
-      </c>
       <c r="F140" s="3">
         <f>SUM(B140:E140)</f>
-        <v>323.16</v>
+        <v>1505.4</v>
       </c>
       <c r="G140" s="3">
         <f>F140/4</f>
-        <v>80.79</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="B141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <v>80.79</v>
       </c>
       <c r="C141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>935.1</v>
+        <v>0</v>
       </c>
       <c r="D141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <v>161.58</v>
       </c>
       <c r="E141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>872.56</v>
+        <v>80.79</v>
       </c>
       <c r="F141" s="3">
         <f>SUM(B141:E141)</f>
-        <v>3789.73</v>
+        <v>323.16</v>
       </c>
       <c r="G141" s="3">
         <f>F141/4</f>
-        <v>947.4325</v>
+        <v>80.79</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
         </is>
       </c>
       <c r="B142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>1019.45</v>
       </c>
       <c r="C142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>935.1</v>
       </c>
       <c r="D142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>962.62</v>
       </c>
       <c r="E142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>872.56</v>
       </c>
       <c r="F142" s="3">
         <f>SUM(B142:E142)</f>
-        <v>792.99</v>
+        <v>3789.73</v>
       </c>
       <c r="G142" s="3">
         <f>F142/4</f>
-        <v>198.2475</v>
+        <v>947.4325</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B143" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C143" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D143" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E143" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F143" s="3">
+        <f>SUM(B143:E143)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G143" s="3">
+        <f>F143/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B143" s="3">
+      <c r="B144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C143" s="3">
+      <c r="C144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D143" s="3">
+      <c r="D144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E143" s="3">
+      <c r="E144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F143" s="3">
-        <f>SUM(B143:E143)</f>
+      <c r="F144" s="3">
+        <f>SUM(B144:E144)</f>
         <v>4932.41</v>
       </c>
-      <c r="G143" s="3">
-        <f>F143/4</f>
+      <c r="G144" s="3">
+        <f>F144/4</f>
         <v>1233.1025</v>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" s="12" t="inlineStr">
+    <row r="145">
+      <c r="A145" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
+        </is>
+      </c>
+      <c r="B145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="C145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="E145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>32.5</v>
+      </c>
+      <c r="F145" s="3">
+        <f>SUM(B145:E145)</f>
+        <v>397.5</v>
+      </c>
+      <c r="G145" s="3">
+        <f>F145/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B144" s="3">
+      <c r="B146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C144" s="3">
+      <c r="C146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D144" s="3">
+      <c r="D146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E144" s="3">
+      <c r="E146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>333.11</v>
       </c>
-      <c r="F144" s="3">
-        <f>SUM(B144:E144)</f>
+      <c r="F146" s="3">
+        <f>SUM(B146:E146)</f>
         <v>4679.18</v>
       </c>
-      <c r="G144" s="3">
-        <f>F144/4</f>
+      <c r="G146" s="3">
+        <f>F146/4</f>
         <v>1169.795</v>
       </c>
     </row>
-    <row r="145">
-      <c r="A145" s="12" t="inlineStr">
+    <row r="147">
+      <c r="A147" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B145" s="3">
+      <c r="B147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C145" s="3">
+      <c r="C147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D145" s="3">
+      <c r="D147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E145" s="3">
+      <c r="E147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F145" s="3">
-        <f>SUM(B145:E145)</f>
+      <c r="F147" s="3">
+        <f>SUM(B147:E147)</f>
         <v>737.73</v>
       </c>
-      <c r="G145" s="3">
-        <f>F145/4</f>
+      <c r="G147" s="3">
+        <f>F147/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" s="5" t="inlineStr">
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="148" ht="27" customHeight="1">
-      <c r="A148" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="27" customHeight="1">
-      <c r="A149" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="150" ht="27" customHeight="1">
       <c r="A150" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="151" ht="27" customHeight="1">
       <c r="A151" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="152" ht="27" customHeight="1">
       <c r="A152" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="153" ht="27" customHeight="1">
       <c r="A153" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="154" ht="27" customHeight="1">
       <c r="A154" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="27" customHeight="1">
+      <c r="A155" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="27" customHeight="1">
+      <c r="A156" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Small hospital-cafeteria charges (Granville Med, Duke) are counted as Restaurants.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A148:G148"/>
-    <mergeCell ref="A149:G149"/>
     <mergeCell ref="A150:G150"/>
     <mergeCell ref="A151:G151"/>
     <mergeCell ref="A152:G152"/>
     <mergeCell ref="A153:G153"/>
     <mergeCell ref="A154:G154"/>
+    <mergeCell ref="A155:G155"/>
+    <mergeCell ref="A156:G156"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -3952,7 +4014,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="H15" s="3">
@@ -4515,7 +4577,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -6598,7 +6660,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -10312,7 +10374,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -10485,7 +10547,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="H19" s="3">
@@ -12561,7 +12623,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -13548,12 +13610,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
         </is>
       </c>
       <c r="H23" s="3">
         <f>SUMIF($C$4:$C$88,G23,$E$4:$E$88)</f>
-        <v>114.5</v>
+        <v>85.27</v>
       </c>
     </row>
     <row r="24">
@@ -13580,12 +13642,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
         </is>
       </c>
       <c r="H24" s="3">
         <f>SUMIF($C$4:$C$88,G24,$E$4:$E$88)</f>
-        <v>85.27</v>
+        <v>84.26</v>
       </c>
     </row>
     <row r="25">
@@ -13599,7 +13661,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Personal Care – Simple Beauty</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -13612,12 +13674,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Personal Care – Simple Beauty</t>
         </is>
       </c>
       <c r="H25" s="3">
         <f>SUMIF($C$4:$C$88,G25,$E$4:$E$88)</f>
-        <v>84.26</v>
+        <v>82.0</v>
       </c>
     </row>
     <row r="26">
@@ -13695,7 +13757,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -13868,12 +13930,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Frndly TV</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="H33" s="3">
         <f>SUMIF($C$4:$C$88,G33,$E$4:$E$88)</f>
-        <v>22.41</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="34">
@@ -13900,12 +13962,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
+          <t xml:space="preserve">Streaming – Frndly TV</t>
         </is>
       </c>
       <c r="H34" s="3">
         <f>SUMIF($C$4:$C$88,G34,$E$4:$E$88)</f>
-        <v>20.27</v>
+        <v>22.41</v>
       </c>
     </row>
     <row r="35">
@@ -13932,12 +13994,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ross</t>
+          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
         </is>
       </c>
       <c r="H35" s="3">
         <f>SUMIF($C$4:$C$88,G35,$E$4:$E$88)</f>
-        <v>16.32</v>
+        <v>20.27</v>
       </c>
     </row>
     <row r="36">
@@ -13964,12 +14026,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+          <t xml:space="preserve">Retail – Ross</t>
         </is>
       </c>
       <c r="H36" s="3">
         <f>SUMIF($C$4:$C$88,G36,$E$4:$E$88)</f>
-        <v>13.87</v>
+        <v>16.32</v>
       </c>
     </row>
     <row r="37">
@@ -13994,14 +14056,14 @@
       <c r="E37" s="3">
         <v>69.36</v>
       </c>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total spending</t>
-        </is>
-      </c>
-      <c r="H37" s="9">
-        <f>SUM(H4:H36)</f>
-        <v>11515.63</v>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+        </is>
+      </c>
+      <c r="H37" s="3">
+        <f>SUMIF($C$4:$C$88,G37,$E$4:$E$88)</f>
+        <v>13.87</v>
       </c>
     </row>
     <row r="38">
@@ -14026,6 +14088,15 @@
       <c r="E38" s="3">
         <v>710.06</v>
       </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total spending</t>
+        </is>
+      </c>
+      <c r="H38" s="9">
+        <f>SUM(H4:H37)</f>
+        <v>11515.63</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="4">
@@ -14049,12 +14120,6 @@
       <c r="E39" s="3">
         <v>221.77</v>
       </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not counted as spending</t>
-        </is>
-      </c>
-      <c r="H39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="4">
@@ -14078,15 +14143,12 @@
       <c r="E40" s="3">
         <v>2576.0</v>
       </c>
-      <c r="G40" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
-        </is>
-      </c>
-      <c r="H40" s="3">
-        <f>SUMIF($C$4:$C$88,G40,$E$4:$E$88)</f>
-        <v>4738.51</v>
-      </c>
+      <c r="G40" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not counted as spending</t>
+        </is>
+      </c>
+      <c r="H40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="4">
@@ -14112,12 +14174,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="H41" s="3">
         <f>SUMIF($C$4:$C$88,G41,$E$4:$E$88)</f>
-        <v>2576.0</v>
+        <v>4738.51</v>
       </c>
     </row>
     <row r="42">
@@ -14141,6 +14203,15 @@
       </c>
       <c r="E42" s="3">
         <v>216.25</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+        </is>
+      </c>
+      <c r="H42" s="3">
+        <f>SUMIF($C$4:$C$88,G42,$E$4:$E$88)</f>
+        <v>2576.0</v>
       </c>
     </row>
     <row r="43">
@@ -16119,7 +16190,7 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
@@ -18527,7 +18598,7 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -22307,7 +22378,7 @@
       </c>
       <c r="D255" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="E255" s="2" t="inlineStr">
@@ -24687,7 +24758,7 @@
       </c>
       <c r="D340" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="E340" s="2" t="inlineStr">
@@ -25611,7 +25682,7 @@
       </c>
       <c r="D373" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Personal Care – Simple Beauty</t>
         </is>
       </c>
       <c r="E373" s="2" t="inlineStr">
@@ -25695,7 +25766,7 @@
       </c>
       <c r="D376" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care (Hair Salon, Beauty)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="E376" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Move Cat on a Whisk to Retail
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -1030,15 +1030,15 @@
       </c>
       <c r="E42" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A42,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>872.56</v>
+        <v>848.05</v>
       </c>
       <c r="F42" s="3">
         <f>SUM(B42:E42)</f>
-        <v>3789.73</v>
+        <v>3765.22</v>
       </c>
       <c r="G42" s="3">
         <f>F42/4</f>
-        <v>947.4325</v>
+        <v>941.305</v>
       </c>
     </row>
     <row r="43">
@@ -1061,15 +1061,15 @@
       </c>
       <c r="E43" s="6">
         <f>SUM(E41:E42)</f>
-        <v>872.56</v>
+        <v>848.05</v>
       </c>
       <c r="F43" s="6">
         <f>SUM(F41:F42)</f>
-        <v>4058.93</v>
+        <v>4034.42</v>
       </c>
       <c r="G43" s="6">
         <f>F43/4</f>
-        <v>1014.7325</v>
+        <v>1008.605</v>
       </c>
     </row>
     <row r="45">
@@ -1985,7 +1985,7 @@
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Tractor Supply</t>
+          <t xml:space="preserve">Retail – Cat on a Whisk</t>
         </is>
       </c>
       <c r="B84" s="3">
@@ -1998,25 +1998,25 @@
       </c>
       <c r="D84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>29.86</v>
+        <v>0</v>
       </c>
       <c r="E84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>24.51</v>
       </c>
       <c r="F84" s="3">
         <f>SUM(B84:E84)</f>
-        <v>29.86</v>
+        <v>24.51</v>
       </c>
       <c r="G84" s="3">
         <f>F84/4</f>
-        <v>7.465</v>
+        <v>6.1275</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
+          <t xml:space="preserve">Retail – Tractor Supply</t>
         </is>
       </c>
       <c r="B85" s="3">
@@ -2025,11 +2025,11 @@
       </c>
       <c r="C85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>63.61</v>
+        <v>0</v>
       </c>
       <c r="D85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>29.86</v>
       </c>
       <c r="E85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2037,26 +2037,26 @@
       </c>
       <c r="F85" s="3">
         <f>SUM(B85:E85)</f>
-        <v>63.61</v>
+        <v>29.86</v>
       </c>
       <c r="G85" s="3">
         <f>F85/4</f>
-        <v>15.9025</v>
+        <v>7.465</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ulta Beauty</t>
+          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
         </is>
       </c>
       <c r="B86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>134.71</v>
+        <v>0</v>
       </c>
       <c r="C86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>63.61</v>
       </c>
       <c r="D86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,D$4)</f>
@@ -2068,22 +2068,22 @@
       </c>
       <c r="F86" s="3">
         <f>SUM(B86:E86)</f>
-        <v>134.71</v>
+        <v>63.61</v>
       </c>
       <c r="G86" s="3">
         <f>F86/4</f>
-        <v>33.6775</v>
+        <v>15.9025</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
+          <t xml:space="preserve">Retail – Ulta Beauty</t>
         </is>
       </c>
       <c r="B87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>51.31</v>
+        <v>134.71</v>
       </c>
       <c r="C87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -2099,30 +2099,30 @@
       </c>
       <c r="F87" s="3">
         <f>SUM(B87:E87)</f>
-        <v>51.31</v>
+        <v>134.71</v>
       </c>
       <c r="G87" s="3">
         <f>F87/4</f>
-        <v>12.8275</v>
+        <v>33.6775</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
         </is>
       </c>
       <c r="B88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>51.31</v>
       </c>
       <c r="C88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>5.87</v>
+        <v>0</v>
       </c>
       <c r="D88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>17.35</v>
+        <v>0</v>
       </c>
       <c r="E88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2130,286 +2130,286 @@
       </c>
       <c r="F88" s="3">
         <f>SUM(B88:E88)</f>
-        <v>23.22</v>
+        <v>51.31</v>
       </c>
       <c r="G88" s="3">
         <f>F88/4</f>
-        <v>5.805</v>
+        <v>12.8275</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
         </is>
       </c>
       <c r="B89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.03</v>
+        <v>0</v>
       </c>
       <c r="C89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>5.87</v>
       </c>
       <c r="D89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>17.35</v>
       </c>
       <c r="E89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>119.97</v>
+        <v>0</v>
       </c>
       <c r="F89" s="3">
         <f>SUM(B89:E89)</f>
-        <v>228.0</v>
+        <v>23.22</v>
       </c>
       <c r="G89" s="3">
         <f>F89/4</f>
+        <v>5.805</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+        </is>
+      </c>
+      <c r="B90" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.03</v>
+      </c>
+      <c r="C90" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D90" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E90" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>119.97</v>
+      </c>
+      <c r="F90" s="3">
+        <f>SUM(B90:E90)</f>
+        <v>228.0</v>
+      </c>
+      <c r="G90" s="3">
+        <f>F90/4</f>
         <v>57.0</v>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="7" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Retail</t>
         </is>
       </c>
-      <c r="B90" s="6">
-        <f>SUM(B75:B89)</f>
+      <c r="B91" s="6">
+        <f>SUM(B75:B90)</f>
         <v>815.42</v>
       </c>
-      <c r="C90" s="6">
-        <f>SUM(C75:C89)</f>
+      <c r="C91" s="6">
+        <f>SUM(C75:C90)</f>
         <v>1150.18</v>
       </c>
-      <c r="D90" s="6">
-        <f>SUM(D75:D89)</f>
+      <c r="D91" s="6">
+        <f>SUM(D75:D90)</f>
         <v>2380.47</v>
       </c>
-      <c r="E90" s="6">
-        <f>SUM(E75:E89)</f>
-        <v>333.11</v>
-      </c>
-      <c r="F90" s="6">
-        <f>SUM(F75:F89)</f>
-        <v>4679.18</v>
-      </c>
-      <c r="G90" s="6">
-        <f>F90/4</f>
-        <v>1169.795</v>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="5" t="inlineStr">
+      <c r="E91" s="6">
+        <f>SUM(E75:E90)</f>
+        <v>357.62</v>
+      </c>
+      <c r="F91" s="6">
+        <f>SUM(F75:F90)</f>
+        <v>4703.69</v>
+      </c>
+      <c r="G91" s="6">
+        <f>F91/4</f>
+        <v>1175.9225</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Home</t>
         </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yard Company (NextGen)</t>
-        </is>
-      </c>
-      <c r="B93" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>60.0</v>
-      </c>
-      <c r="C93" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.0</v>
-      </c>
-      <c r="D93" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>220.0</v>
-      </c>
-      <c r="E93" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>120.0</v>
-      </c>
-      <c r="F93" s="3">
-        <f>SUM(B93:E93)</f>
-        <v>500.0</v>
-      </c>
-      <c r="G93" s="3">
-        <f>F93/4</f>
-        <v>125.0</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
       <c r="B94" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>60.0</v>
       </c>
       <c r="C94" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>242.05</v>
+        <v>100.0</v>
       </c>
       <c r="D94" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>536.6</v>
+        <v>220.0</v>
       </c>
       <c r="E94" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>120.0</v>
       </c>
       <c r="F94" s="3">
         <f>SUM(B94:E94)</f>
-        <v>778.65</v>
+        <v>500.0</v>
       </c>
       <c r="G94" s="3">
         <f>F94/4</f>
+        <v>125.0</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+        </is>
+      </c>
+      <c r="B95" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C95" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>242.05</v>
+      </c>
+      <c r="D95" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>536.6</v>
+      </c>
+      <c r="E95" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F95" s="3">
+        <f>SUM(B95:E95)</f>
+        <v>778.65</v>
+      </c>
+      <c r="G95" s="3">
+        <f>F95/4</f>
         <v>194.6625</v>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="7" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Home</t>
         </is>
       </c>
-      <c r="B95" s="6">
-        <f>SUM(B93:B94)</f>
+      <c r="B96" s="6">
+        <f>SUM(B94:B95)</f>
         <v>60.0</v>
       </c>
-      <c r="C95" s="6">
-        <f>SUM(C93:C94)</f>
+      <c r="C96" s="6">
+        <f>SUM(C94:C95)</f>
         <v>342.05</v>
       </c>
-      <c r="D95" s="6">
-        <f>SUM(D93:D94)</f>
+      <c r="D96" s="6">
+        <f>SUM(D94:D95)</f>
         <v>756.6</v>
       </c>
-      <c r="E95" s="6">
-        <f>SUM(E93:E94)</f>
+      <c r="E96" s="6">
+        <f>SUM(E94:E95)</f>
         <v>120.0</v>
       </c>
-      <c r="F95" s="6">
-        <f>SUM(F93:F94)</f>
+      <c r="F96" s="6">
+        <f>SUM(F94:F95)</f>
         <v>1278.65</v>
       </c>
-      <c r="G95" s="6">
-        <f>F95/4</f>
+      <c r="G96" s="6">
+        <f>F96/4</f>
         <v>319.6625</v>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="5" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel</t>
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="12" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel (Lyft, Hotel)</t>
         </is>
       </c>
-      <c r="B98" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B99" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>102.65</v>
       </c>
-      <c r="C98" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C99" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D98" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D99" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E98" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E99" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F98" s="3">
-        <f>SUM(B98:E98)</f>
+      <c r="F99" s="3">
+        <f>SUM(B99:E99)</f>
         <v>102.65</v>
       </c>
-      <c r="G98" s="3">
-        <f>F98/4</f>
-        <v>25.6625</v>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Travel</t>
-        </is>
-      </c>
-      <c r="B99" s="6">
-        <f>SUM(B98:B98)</f>
-        <v>102.65</v>
-      </c>
-      <c r="C99" s="6">
-        <f>SUM(C98:C98)</f>
-        <v>0</v>
-      </c>
-      <c r="D99" s="6">
-        <f>SUM(D98:D98)</f>
-        <v>0</v>
-      </c>
-      <c r="E99" s="6">
-        <f>SUM(E98:E98)</f>
-        <v>0</v>
-      </c>
-      <c r="F99" s="6">
-        <f>SUM(F98:F98)</f>
-        <v>102.65</v>
-      </c>
-      <c r="G99" s="6">
+      <c r="G99" s="3">
         <f>F99/4</f>
         <v>25.6625</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="5" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Travel</t>
+        </is>
+      </c>
+      <c r="B100" s="6">
+        <f>SUM(B99:B99)</f>
+        <v>102.65</v>
+      </c>
+      <c r="C100" s="6">
+        <f>SUM(C99:C99)</f>
+        <v>0</v>
+      </c>
+      <c r="D100" s="6">
+        <f>SUM(D99:D99)</f>
+        <v>0</v>
+      </c>
+      <c r="E100" s="6">
+        <f>SUM(E99:E99)</f>
+        <v>0</v>
+      </c>
+      <c r="F100" s="6">
+        <f>SUM(F99:F99)</f>
+        <v>102.65</v>
+      </c>
+      <c r="G100" s="6">
+        <f>F100/4</f>
+        <v>25.6625</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Recreation</t>
         </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">St. James Marina</t>
-        </is>
-      </c>
-      <c r="B102" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C102" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>33.54</v>
-      </c>
-      <c r="D102" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E102" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A102,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F102" s="3">
-        <f>SUM(B102:E102)</f>
-        <v>33.54</v>
-      </c>
-      <c r="G102" s="3">
-        <f>F102/4</f>
-        <v>8.385</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">St. James Marina</t>
         </is>
       </c>
       <c r="B103" s="3">
@@ -2418,11 +2418,11 @@
       </c>
       <c r="C103" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>400.0</v>
+        <v>33.54</v>
       </c>
       <c r="D103" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>13.5</v>
+        <v>0</v>
       </c>
       <c r="E103" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2430,155 +2430,155 @@
       </c>
       <c r="F103" s="3">
         <f>SUM(B103:E103)</f>
-        <v>413.5</v>
+        <v>33.54</v>
       </c>
       <c r="G103" s="3">
         <f>F103/4</f>
+        <v>8.385</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entertainment &amp; Events</t>
+        </is>
+      </c>
+      <c r="B104" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C104" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>400.0</v>
+      </c>
+      <c r="D104" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>13.5</v>
+      </c>
+      <c r="E104" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F104" s="3">
+        <f>SUM(B104:E104)</f>
+        <v>413.5</v>
+      </c>
+      <c r="G104" s="3">
+        <f>F104/4</f>
         <v>103.375</v>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="7" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Recreation</t>
         </is>
       </c>
-      <c r="B104" s="6">
-        <f>SUM(B102:B103)</f>
+      <c r="B105" s="6">
+        <f>SUM(B103:B104)</f>
         <v>0</v>
       </c>
-      <c r="C104" s="6">
-        <f>SUM(C102:C103)</f>
+      <c r="C105" s="6">
+        <f>SUM(C103:C104)</f>
         <v>433.54</v>
       </c>
-      <c r="D104" s="6">
-        <f>SUM(D102:D103)</f>
+      <c r="D105" s="6">
+        <f>SUM(D103:D104)</f>
         <v>13.5</v>
       </c>
-      <c r="E104" s="6">
-        <f>SUM(E102:E103)</f>
+      <c r="E105" s="6">
+        <f>SUM(E103:E104)</f>
         <v>0</v>
       </c>
-      <c r="F104" s="6">
-        <f>SUM(F102:F103)</f>
+      <c r="F105" s="6">
+        <f>SUM(F103:F104)</f>
         <v>447.04</v>
       </c>
-      <c r="G104" s="6">
-        <f>F104/4</f>
+      <c r="G105" s="6">
+        <f>F105/4</f>
         <v>111.76</v>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="5" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="12" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
         </is>
       </c>
-      <c r="B107" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B108" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>75.0</v>
       </c>
-      <c r="C107" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C108" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>764.05</v>
       </c>
-      <c r="D107" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D108" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>331.5</v>
       </c>
-      <c r="E107" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E108" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>130.0</v>
       </c>
-      <c r="F107" s="3">
-        <f>SUM(B107:E107)</f>
+      <c r="F108" s="3">
+        <f>SUM(B108:E108)</f>
         <v>1300.55</v>
       </c>
-      <c r="G107" s="3">
-        <f>F107/4</f>
-        <v>325.1375</v>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Transfers</t>
-        </is>
-      </c>
-      <c r="B108" s="6">
-        <f>SUM(B107:B107)</f>
-        <v>75.0</v>
-      </c>
-      <c r="C108" s="6">
-        <f>SUM(C107:C107)</f>
-        <v>764.05</v>
-      </c>
-      <c r="D108" s="6">
-        <f>SUM(D107:D107)</f>
-        <v>331.5</v>
-      </c>
-      <c r="E108" s="6">
-        <f>SUM(E107:E107)</f>
-        <v>130.0</v>
-      </c>
-      <c r="F108" s="6">
-        <f>SUM(F107:F107)</f>
-        <v>1300.55</v>
-      </c>
-      <c r="G108" s="6">
+      <c r="G108" s="3">
         <f>F108/4</f>
         <v>325.1375</v>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="5" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Transfers</t>
+        </is>
+      </c>
+      <c r="B109" s="6">
+        <f>SUM(B108:B108)</f>
+        <v>75.0</v>
+      </c>
+      <c r="C109" s="6">
+        <f>SUM(C108:C108)</f>
+        <v>764.05</v>
+      </c>
+      <c r="D109" s="6">
+        <f>SUM(D108:D108)</f>
+        <v>331.5</v>
+      </c>
+      <c r="E109" s="6">
+        <f>SUM(E108:E108)</f>
+        <v>130.0</v>
+      </c>
+      <c r="F109" s="6">
+        <f>SUM(F108:F108)</f>
+        <v>1300.55</v>
+      </c>
+      <c r="G109" s="6">
+        <f>F109/4</f>
+        <v>325.1375</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Other</t>
         </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Donations &amp; Clubs (Kiwanis)</t>
-        </is>
-      </c>
-      <c r="B111" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C111" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D111" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E111" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A111,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>200.0</v>
-      </c>
-      <c r="F111" s="3">
-        <f>SUM(B111:E111)</f>
-        <v>200.0</v>
-      </c>
-      <c r="G111" s="3">
-        <f>F111/4</f>
-        <v>50.0</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
+          <t xml:space="preserve">Donations &amp; Clubs (Kiwanis)</t>
         </is>
       </c>
       <c r="B112" s="3">
@@ -2595,152 +2595,152 @@
       </c>
       <c r="E112" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>147.0</v>
+        <v>200.0</v>
       </c>
       <c r="F112" s="3">
         <f>SUM(B112:E112)</f>
-        <v>147.0</v>
+        <v>200.0</v>
       </c>
       <c r="G112" s="3">
         <f>F112/4</f>
+        <v>50.0</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
+        </is>
+      </c>
+      <c r="B113" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C113" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D113" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E113" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>147.0</v>
+      </c>
+      <c r="F113" s="3">
+        <f>SUM(B113:E113)</f>
+        <v>147.0</v>
+      </c>
+      <c r="G113" s="3">
+        <f>F113/4</f>
         <v>36.75</v>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="7" t="inlineStr">
+    <row r="114">
+      <c r="A114" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Other</t>
         </is>
       </c>
-      <c r="B113" s="6">
-        <f>SUM(B111:B112)</f>
+      <c r="B114" s="6">
+        <f>SUM(B112:B113)</f>
         <v>0</v>
       </c>
-      <c r="C113" s="6">
-        <f>SUM(C111:C112)</f>
+      <c r="C114" s="6">
+        <f>SUM(C112:C113)</f>
         <v>0</v>
       </c>
-      <c r="D113" s="6">
-        <f>SUM(D111:D112)</f>
+      <c r="D114" s="6">
+        <f>SUM(D112:D113)</f>
         <v>0</v>
       </c>
-      <c r="E113" s="6">
-        <f>SUM(E111:E112)</f>
+      <c r="E114" s="6">
+        <f>SUM(E112:E113)</f>
         <v>347.0</v>
       </c>
-      <c r="F113" s="6">
-        <f>SUM(F111:F112)</f>
+      <c r="F114" s="6">
+        <f>SUM(F112:F113)</f>
         <v>347.0</v>
       </c>
-      <c r="G113" s="6">
-        <f>F113/4</f>
+      <c r="G114" s="6">
+        <f>F114/4</f>
         <v>86.75</v>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="8" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL SPENDING</t>
         </is>
       </c>
-      <c r="B115" s="9">
-        <f>B10+B18+B23+B28+B32+B38+B43+B48+B59+B63+B67+B72+B90+B95+B99+B104+B108+B113</f>
+      <c r="B116" s="9">
+        <f>B10+B18+B23+B28+B32+B38+B43+B48+B59+B63+B67+B72+B91+B96+B100+B105+B109+B114</f>
         <v>12135.81</v>
       </c>
-      <c r="C115" s="9">
-        <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C67+C72+C90+C95+C99+C104+C108+C113</f>
+      <c r="C116" s="9">
+        <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C67+C72+C91+C96+C100+C105+C109+C114</f>
         <v>12663.24</v>
       </c>
-      <c r="D115" s="9">
-        <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D67+D72+D90+D95+D99+D104+D108+D113</f>
+      <c r="D116" s="9">
+        <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D67+D72+D91+D96+D100+D105+D109+D114</f>
         <v>15086.64</v>
       </c>
-      <c r="E115" s="9">
-        <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E67+E72+E90+E95+E99+E104+E108+E113</f>
+      <c r="E116" s="9">
+        <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E67+E72+E91+E96+E100+E105+E109+E114</f>
         <v>11515.63</v>
       </c>
-      <c r="F115" s="9">
-        <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F67+F72+F90+F95+F99+F104+F108+F113</f>
+      <c r="F116" s="9">
+        <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F67+F72+F91+F96+F100+F105+F109+F114</f>
         <v>51401.32</v>
       </c>
-      <c r="G115" s="9">
-        <f>F115/4</f>
+      <c r="G116" s="9">
+        <f>F116/4</f>
         <v>12850.33</v>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="5" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Not counted as spending</t>
         </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
-        </is>
-      </c>
-      <c r="B118" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A118,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="C118" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A118,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="D118" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A118,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="E118" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A118,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="F118" s="3">
-        <f>SUM(B118:E118)</f>
-        <v>10304.0</v>
-      </c>
-      <c r="G118" s="3">
-        <f>F118/4</f>
-        <v>2576.0</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
         </is>
       </c>
       <c r="B119" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>2576.0</v>
       </c>
       <c r="C119" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>7227.09</v>
+        <v>2576.0</v>
       </c>
       <c r="D119" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>4593.08</v>
+        <v>2576.0</v>
       </c>
       <c r="E119" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>4738.51</v>
+        <v>2576.0</v>
       </c>
       <c r="F119" s="3">
         <f>SUM(B119:E119)</f>
-        <v>16558.68</v>
+        <v>10304.0</v>
       </c>
       <c r="G119" s="3">
         <f>F119/4</f>
-        <v>4139.67</v>
+        <v>2576.0</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sloane Realty</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="B120" s="3">
@@ -2749,42 +2749,42 @@
       </c>
       <c r="C120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2891.98</v>
+        <v>7227.09</v>
       </c>
       <c r="D120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>4593.08</v>
       </c>
       <c r="E120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>4738.51</v>
       </c>
       <c r="F120" s="3">
         <f>SUM(B120:E120)</f>
-        <v>2891.98</v>
+        <v>16558.68</v>
       </c>
       <c r="G120" s="3">
         <f>F120/4</f>
-        <v>722.995</v>
+        <v>4139.67</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checks Written (payee not shown)</t>
+          <t xml:space="preserve">Sloane Realty</t>
         </is>
       </c>
       <c r="B121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2630.0</v>
+        <v>0</v>
       </c>
       <c r="C121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>2891.98</v>
       </c>
       <c r="D121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>728.0</v>
+        <v>0</v>
       </c>
       <c r="E121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2792,30 +2792,30 @@
       </c>
       <c r="F121" s="3">
         <f>SUM(B121:E121)</f>
-        <v>3358.0</v>
+        <v>2891.98</v>
       </c>
       <c r="G121" s="3">
         <f>F121/4</f>
-        <v>839.5</v>
+        <v>722.995</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Checks Written (payee not shown)</t>
         </is>
       </c>
       <c r="B122" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>2630.0</v>
       </c>
       <c r="C122" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3.26</v>
+        <v>0</v>
       </c>
       <c r="D122" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>728.0</v>
       </c>
       <c r="E122" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2823,757 +2823,788 @@
       </c>
       <c r="F122" s="3">
         <f>SUM(B122:E122)</f>
-        <v>3.26</v>
+        <v>3358.0</v>
       </c>
       <c r="G122" s="3">
         <f>F122/4</f>
+        <v>839.5</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
+        </is>
+      </c>
+      <c r="B123" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C123" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>3.26</v>
+      </c>
+      <c r="D123" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E123" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F123" s="3">
+        <f>SUM(B123:E123)</f>
+        <v>3.26</v>
+      </c>
+      <c r="G123" s="3">
+        <f>F123/4</f>
         <v>0.815</v>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="7" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total not counted as spending</t>
         </is>
       </c>
-      <c r="B123" s="6">
-        <f>SUM(B118:B122)</f>
+      <c r="B124" s="6">
+        <f>SUM(B119:B123)</f>
         <v>5206.0</v>
       </c>
-      <c r="C123" s="6">
-        <f>SUM(C118:C122)</f>
+      <c r="C124" s="6">
+        <f>SUM(C119:C123)</f>
         <v>12698.33</v>
       </c>
-      <c r="D123" s="6">
-        <f>SUM(D118:D122)</f>
+      <c r="D124" s="6">
+        <f>SUM(D119:D123)</f>
         <v>7897.08</v>
       </c>
-      <c r="E123" s="6">
-        <f>SUM(E118:E122)</f>
+      <c r="E124" s="6">
+        <f>SUM(E119:E123)</f>
         <v>7314.51</v>
       </c>
-      <c r="F123" s="6">
-        <f>SUM(F118:F122)</f>
+      <c r="F124" s="6">
+        <f>SUM(F119:F123)</f>
         <v>33115.92</v>
       </c>
-      <c r="G123" s="6">
-        <f>F123/4</f>
+      <c r="G124" s="6">
+        <f>F124/4</f>
         <v>8278.98</v>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Check: spending + not-counted items</t>
-        </is>
-      </c>
-      <c r="B125" s="3">
-        <f>B115+B123</f>
-        <v>17341.81</v>
-      </c>
-      <c r="C125" s="3">
-        <f>C115+C123</f>
-        <v>25361.57</v>
-      </c>
-      <c r="D125" s="3">
-        <f>D115+D123</f>
-        <v>22983.72</v>
-      </c>
-      <c r="E125" s="3">
-        <f>E115+E123</f>
-        <v>18830.14</v>
-      </c>
-      <c r="F125" s="3">
-        <f>F115+F123</f>
-        <v>84517.24</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
-        </is>
-      </c>
-      <c r="B126" s="13">
+          <t xml:space="preserve">Check: spending + not-counted items</t>
+        </is>
+      </c>
+      <c r="B126" s="3">
+        <f>B116+B124</f>
         <v>17341.81</v>
       </c>
-      <c r="C126" s="13">
+      <c r="C126" s="3">
+        <f>C116+C124</f>
         <v>25361.57</v>
       </c>
-      <c r="D126" s="13">
+      <c r="D126" s="3">
+        <f>D116+D124</f>
         <v>22983.72</v>
       </c>
-      <c r="E126" s="13">
+      <c r="E126" s="3">
+        <f>E116+E124</f>
         <v>18830.14</v>
       </c>
       <c r="F126" s="3">
-        <f>SUM(B126:E126)</f>
+        <f>F116+F124</f>
         <v>84517.24</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
+        </is>
+      </c>
+      <c r="B127" s="13">
+        <v>17341.81</v>
+      </c>
+      <c r="C127" s="13">
+        <v>25361.57</v>
+      </c>
+      <c r="D127" s="13">
+        <v>22983.72</v>
+      </c>
+      <c r="E127" s="13">
+        <v>18830.14</v>
+      </c>
+      <c r="F127" s="3">
+        <f>SUM(B127:E127)</f>
+        <v>84517.24</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Difference (should be $0 = every dollar accounted for)</t>
         </is>
       </c>
-      <c r="B127" s="3">
-        <f>B125-B126</f>
+      <c r="B128" s="3">
+        <f>B126-B127</f>
         <v>0.0</v>
       </c>
-      <c r="C127" s="3">
-        <f>C125-C126</f>
+      <c r="C128" s="3">
+        <f>C126-C127</f>
         <v>0.0</v>
       </c>
-      <c r="D127" s="3">
-        <f>D125-D126</f>
+      <c r="D128" s="3">
+        <f>D126-D127</f>
         <v>0.0</v>
       </c>
-      <c r="E127" s="3">
-        <f>E125-E126</f>
+      <c r="E128" s="3">
+        <f>E126-E127</f>
         <v>0.0</v>
       </c>
-      <c r="F127" s="3">
-        <f>F125-F126</f>
+      <c r="F128" s="3">
+        <f>F126-F127</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="5" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Key Bills at a Glance</t>
         </is>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="15" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Bill</t>
         </is>
       </c>
-      <c r="B130" s="1" t="inlineStr">
+      <c r="B131" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">June 2026</t>
         </is>
       </c>
-      <c r="C130" s="1" t="inlineStr">
+      <c r="C131" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">July 2026</t>
         </is>
       </c>
-      <c r="D130" s="1" t="inlineStr">
+      <c r="D131" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">August 2026</t>
         </is>
       </c>
-      <c r="E130" s="1" t="inlineStr">
+      <c r="E131" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">September 2026</t>
         </is>
       </c>
-      <c r="F130" s="1" t="inlineStr">
+      <c r="F131" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">4-Month Total</t>
         </is>
       </c>
-      <c r="G130" s="1" t="inlineStr">
+      <c r="G131" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Monthly Avg</t>
         </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A&amp;D Mortgage</t>
-        </is>
-      </c>
-      <c r="B131" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="C131" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="D131" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="E131" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A131,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="F131" s="3">
-        <f>SUM(B131:E131)</f>
-        <v>13644.4</v>
-      </c>
-      <c r="G131" s="3">
-        <f>F131/4</f>
-        <v>3411.1</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Membership (Club)</t>
+          <t xml:space="preserve">A&amp;D Mortgage</t>
         </is>
       </c>
       <c r="B132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1591.78</v>
+        <v>3411.1</v>
       </c>
       <c r="C132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>1601.56</v>
+        <v>3411.1</v>
       </c>
       <c r="D132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1492.11</v>
+        <v>3411.1</v>
       </c>
       <c r="E132" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>1767.0</v>
+        <v>3411.1</v>
       </c>
       <c r="F132" s="3">
         <f>SUM(B132:E132)</f>
-        <v>6452.45</v>
+        <v>13644.4</v>
       </c>
       <c r="G132" s="3">
         <f>F132/4</f>
-        <v>1613.1125</v>
+        <v>3411.1</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Plantation POA Dues</t>
+          <t xml:space="preserve">St. James Membership (Club)</t>
         </is>
       </c>
       <c r="B133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>692.95</v>
+        <v>1591.78</v>
       </c>
       <c r="C133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>1601.56</v>
       </c>
       <c r="D133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1492.11</v>
       </c>
       <c r="E133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>1767.0</v>
       </c>
       <c r="F133" s="3">
         <f>SUM(B133:E133)</f>
-        <v>692.95</v>
+        <v>6452.45</v>
       </c>
       <c r="G133" s="3">
         <f>F133/4</f>
-        <v>173.2375</v>
+        <v>1613.1125</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">St. James Plantation POA Dues</t>
         </is>
       </c>
       <c r="B134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>360.42</v>
+        <v>692.95</v>
       </c>
       <c r="C134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>360.42</v>
+        <v>0</v>
       </c>
       <c r="D134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>475.42</v>
+        <v>0</v>
       </c>
       <c r="E134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>354.17</v>
+        <v>0</v>
       </c>
       <c r="F134" s="3">
         <f>SUM(B134:E134)</f>
-        <v>1550.43</v>
+        <v>692.95</v>
       </c>
       <c r="G134" s="3">
         <f>F134/4</f>
-        <v>387.6075</v>
+        <v>173.2375</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="B135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>79.21</v>
+        <v>360.42</v>
       </c>
       <c r="C135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>73.61</v>
+        <v>360.42</v>
       </c>
       <c r="D135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>73.61</v>
+        <v>475.42</v>
       </c>
       <c r="E135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>73.61</v>
+        <v>354.17</v>
       </c>
       <c r="F135" s="3">
         <f>SUM(B135:E135)</f>
-        <v>300.04</v>
+        <v>1550.43</v>
       </c>
       <c r="G135" s="3">
         <f>F135/4</f>
-        <v>75.01</v>
+        <v>387.6075</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Banner Life Insurance</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="B136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>710.06</v>
+        <v>79.21</v>
       </c>
       <c r="C136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="D136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="E136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="F136" s="3">
         <f>SUM(B136:E136)</f>
-        <v>2840.24</v>
+        <v>300.04</v>
       </c>
       <c r="G136" s="3">
         <f>F136/4</f>
-        <v>710.06</v>
+        <v>75.01</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Banner Life Insurance</t>
         </is>
       </c>
       <c r="B137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>710.06</v>
       </c>
       <c r="C137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>710.06</v>
       </c>
       <c r="D137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>710.06</v>
       </c>
       <c r="E137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>710.06</v>
       </c>
       <c r="F137" s="3">
         <f>SUM(B137:E137)</f>
-        <v>1412.24</v>
+        <v>2840.24</v>
       </c>
       <c r="G137" s="3">
         <f>F137/4</f>
-        <v>353.06</v>
+        <v>710.06</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>294.57</v>
       </c>
       <c r="C138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>294.8</v>
       </c>
       <c r="D138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>436.02</v>
       </c>
       <c r="E138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>386.85</v>
       </c>
       <c r="F138" s="3">
         <f>SUM(B138:E138)</f>
-        <v>1162.97</v>
+        <v>1412.24</v>
       </c>
       <c r="G138" s="3">
         <f>F138/4</f>
-        <v>290.7425</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>0</v>
       </c>
       <c r="C139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>336.35</v>
       </c>
       <c r="D139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>406.96</v>
       </c>
       <c r="E139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>419.66</v>
       </c>
       <c r="F139" s="3">
         <f>SUM(B139:E139)</f>
-        <v>342.43</v>
+        <v>1162.97</v>
       </c>
       <c r="G139" s="3">
         <f>F139/4</f>
-        <v>85.6075</v>
+        <v>290.7425</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+        </is>
+      </c>
+      <c r="B140" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C140" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D140" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>179.33</v>
+      </c>
+      <c r="E140" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>84.26</v>
+      </c>
+      <c r="F140" s="3">
+        <f>SUM(B140:E140)</f>
+        <v>342.43</v>
+      </c>
+      <c r="G140" s="3">
+        <f>F140/4</f>
+        <v>85.6075</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
-      <c r="B140" s="3">
+      <c r="B141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>78.84</v>
       </c>
-      <c r="C140" s="3">
+      <c r="C141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
-      <c r="D140" s="3">
+      <c r="D141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>586.29</v>
       </c>
-      <c r="E140" s="3">
+      <c r="E141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>503.92</v>
       </c>
-      <c r="F140" s="3">
-        <f>SUM(B140:E140)</f>
-        <v>1505.4</v>
-      </c>
-      <c r="G140" s="3">
-        <f>F140/4</f>
-        <v>376.35</v>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
-        </is>
-      </c>
-      <c r="B141" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="C141" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D141" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
-      </c>
-      <c r="E141" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
-      </c>
       <c r="F141" s="3">
         <f>SUM(B141:E141)</f>
-        <v>323.16</v>
+        <v>1505.4</v>
       </c>
       <c r="G141" s="3">
         <f>F141/4</f>
-        <v>80.79</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="B142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <v>80.79</v>
       </c>
       <c r="C142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>935.1</v>
+        <v>0</v>
       </c>
       <c r="D142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <v>161.58</v>
       </c>
       <c r="E142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>872.56</v>
+        <v>80.79</v>
       </c>
       <c r="F142" s="3">
         <f>SUM(B142:E142)</f>
-        <v>3789.73</v>
+        <v>323.16</v>
       </c>
       <c r="G142" s="3">
         <f>F142/4</f>
-        <v>947.4325</v>
+        <v>80.79</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
         </is>
       </c>
       <c r="B143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>1019.45</v>
       </c>
       <c r="C143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>935.1</v>
       </c>
       <c r="D143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>962.62</v>
       </c>
       <c r="E143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>848.05</v>
       </c>
       <c r="F143" s="3">
         <f>SUM(B143:E143)</f>
-        <v>792.99</v>
+        <v>3765.22</v>
       </c>
       <c r="G143" s="3">
         <f>F143/4</f>
-        <v>198.2475</v>
+        <v>941.305</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B144" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C144" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D144" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E144" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F144" s="3">
+        <f>SUM(B144:E144)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G144" s="3">
+        <f>F144/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B144" s="3">
+      <c r="B145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C144" s="3">
+      <c r="C145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D144" s="3">
+      <c r="D145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E144" s="3">
+      <c r="E145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F144" s="3">
-        <f>SUM(B144:E144)</f>
-        <v>4932.41</v>
-      </c>
-      <c r="G144" s="3">
-        <f>F144/4</f>
-        <v>1233.1025</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
-        </is>
-      </c>
-      <c r="B145" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="C145" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D145" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="E145" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.5</v>
-      </c>
       <c r="F145" s="3">
         <f>SUM(B145:E145)</f>
-        <v>397.5</v>
+        <v>4932.41</v>
       </c>
       <c r="G145" s="3">
         <f>F145/4</f>
-        <v>99.375</v>
+        <v>1233.1025</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
+        </is>
+      </c>
+      <c r="B146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="C146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="E146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>32.5</v>
+      </c>
+      <c r="F146" s="3">
+        <f>SUM(B146:E146)</f>
+        <v>397.5</v>
+      </c>
+      <c r="G146" s="3">
+        <f>F146/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B146" s="3">
+      <c r="B147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C146" s="3">
+      <c r="C147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D146" s="3">
+      <c r="D147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E146" s="3">
+      <c r="E147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>333.11</v>
-      </c>
-      <c r="F146" s="3">
-        <f>SUM(B146:E146)</f>
-        <v>4679.18</v>
-      </c>
-      <c r="G146" s="3">
-        <f>F146/4</f>
-        <v>1169.795</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="12" t="inlineStr">
+        <v>357.62</v>
+      </c>
+      <c r="F147" s="3">
+        <f>SUM(B147:E147)</f>
+        <v>4703.69</v>
+      </c>
+      <c r="G147" s="3">
+        <f>F147/4</f>
+        <v>1175.9225</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B147" s="3">
+      <c r="B148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C147" s="3">
+      <c r="C148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D147" s="3">
+      <c r="D148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E147" s="3">
+      <c r="E148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F147" s="3">
-        <f>SUM(B147:E147)</f>
+      <c r="F148" s="3">
+        <f>SUM(B148:E148)</f>
         <v>737.73</v>
       </c>
-      <c r="G147" s="3">
-        <f>F147/4</f>
+      <c r="G148" s="3">
+        <f>F148/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" s="5" t="inlineStr">
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="27" customHeight="1">
-      <c r="A150" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="151" ht="27" customHeight="1">
       <c r="A151" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="152" ht="27" customHeight="1">
       <c r="A152" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="153" ht="27" customHeight="1">
       <c r="A153" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="154" ht="27" customHeight="1">
       <c r="A154" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="155" ht="27" customHeight="1">
       <c r="A155" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
         </is>
       </c>
     </row>
     <row r="156" ht="27" customHeight="1">
       <c r="A156" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="27" customHeight="1">
+      <c r="A157" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Small hospital-cafeteria charges (Granville Med, Duke) are counted as Restaurants.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A150:G150"/>
     <mergeCell ref="A151:G151"/>
     <mergeCell ref="A152:G152"/>
     <mergeCell ref="A153:G153"/>
     <mergeCell ref="A154:G154"/>
     <mergeCell ref="A155:G155"/>
     <mergeCell ref="A156:G156"/>
+    <mergeCell ref="A157:G157"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -13021,12 +13052,12 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Retail – Cat on a Whisk</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Retail</t>
         </is>
       </c>
       <c r="E5" s="3">
@@ -13071,7 +13102,7 @@
       </c>
       <c r="H6" s="3">
         <f>SUMIF($C$4:$C$88,G6,$E$4:$E$88)</f>
-        <v>872.56</v>
+        <v>848.05</v>
       </c>
     </row>
     <row r="7">
@@ -13962,12 +13993,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Frndly TV</t>
+          <t xml:space="preserve">Retail – Cat on a Whisk</t>
         </is>
       </c>
       <c r="H34" s="3">
         <f>SUMIF($C$4:$C$88,G34,$E$4:$E$88)</f>
-        <v>22.41</v>
+        <v>24.51</v>
       </c>
     </row>
     <row r="35">
@@ -13994,12 +14025,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
+          <t xml:space="preserve">Streaming – Frndly TV</t>
         </is>
       </c>
       <c r="H35" s="3">
         <f>SUMIF($C$4:$C$88,G35,$E$4:$E$88)</f>
-        <v>20.27</v>
+        <v>22.41</v>
       </c>
     </row>
     <row r="36">
@@ -14026,12 +14057,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ross</t>
+          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
         </is>
       </c>
       <c r="H36" s="3">
         <f>SUMIF($C$4:$C$88,G36,$E$4:$E$88)</f>
-        <v>16.32</v>
+        <v>20.27</v>
       </c>
     </row>
     <row r="37">
@@ -14058,12 +14089,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+          <t xml:space="preserve">Retail – Ross</t>
         </is>
       </c>
       <c r="H37" s="3">
         <f>SUMIF($C$4:$C$88,G37,$E$4:$E$88)</f>
-        <v>13.87</v>
+        <v>16.32</v>
       </c>
     </row>
     <row r="38">
@@ -14088,14 +14119,14 @@
       <c r="E38" s="3">
         <v>710.06</v>
       </c>
-      <c r="G38" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total spending</t>
-        </is>
-      </c>
-      <c r="H38" s="9">
-        <f>SUM(H4:H37)</f>
-        <v>11515.63</v>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+        </is>
+      </c>
+      <c r="H38" s="3">
+        <f>SUMIF($C$4:$C$88,G38,$E$4:$E$88)</f>
+        <v>13.87</v>
       </c>
     </row>
     <row r="39">
@@ -14120,6 +14151,15 @@
       <c r="E39" s="3">
         <v>221.77</v>
       </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total spending</t>
+        </is>
+      </c>
+      <c r="H39" s="9">
+        <f>SUM(H4:H38)</f>
+        <v>11515.63</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4">
@@ -14143,12 +14183,6 @@
       <c r="E40" s="3">
         <v>2576.0</v>
       </c>
-      <c r="G40" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not counted as spending</t>
-        </is>
-      </c>
-      <c r="H40" s="7"/>
     </row>
     <row r="41">
       <c r="A41" s="4">
@@ -14172,15 +14206,12 @@
       <c r="E41" s="3">
         <v>68.24</v>
       </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
-        </is>
-      </c>
-      <c r="H41" s="3">
-        <f>SUMIF($C$4:$C$88,G41,$E$4:$E$88)</f>
-        <v>4738.51</v>
-      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not counted as spending</t>
+        </is>
+      </c>
+      <c r="H41" s="7"/>
     </row>
     <row r="42">
       <c r="A42" s="4">
@@ -14206,12 +14237,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="H42" s="3">
         <f>SUMIF($C$4:$C$88,G42,$E$4:$E$88)</f>
-        <v>2576.0</v>
+        <v>4738.51</v>
       </c>
     </row>
     <row r="43">
@@ -14235,6 +14266,15 @@
       </c>
       <c r="E43" s="3">
         <v>100.28</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+        </is>
+      </c>
+      <c r="H43" s="3">
+        <f>SUMIF($C$4:$C$88,G43,$E$4:$E$88)</f>
+        <v>2576.0</v>
       </c>
     </row>
     <row r="44">
@@ -25122,12 +25162,12 @@
       </c>
       <c r="D353" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Retail – Cat on a Whisk</t>
         </is>
       </c>
       <c r="E353" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Retail</t>
         </is>
       </c>
       <c r="F353" s="3">

</xml_diff>

<commit_message>
Show student loan as its own group and in Key Bills
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -775,7 +775,7 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Total Debt Payments</t>
+          <t xml:space="preserve">Total Student Loan</t>
         </is>
       </c>
       <c r="B32" s="6">
@@ -3233,378 +3233,409 @@
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="B139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>160.37</v>
       </c>
       <c r="C139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>160.37</v>
       </c>
       <c r="D139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>160.37</v>
       </c>
       <c r="E139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>160.37</v>
       </c>
       <c r="F139" s="3">
         <f>SUM(B139:E139)</f>
-        <v>1162.97</v>
+        <v>641.48</v>
       </c>
       <c r="G139" s="3">
         <f>F139/4</f>
-        <v>290.7425</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>0</v>
       </c>
       <c r="C140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>336.35</v>
       </c>
       <c r="D140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>406.96</v>
       </c>
       <c r="E140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>419.66</v>
       </c>
       <c r="F140" s="3">
         <f>SUM(B140:E140)</f>
-        <v>342.43</v>
+        <v>1162.97</v>
       </c>
       <c r="G140" s="3">
         <f>F140/4</f>
-        <v>85.6075</v>
+        <v>290.7425</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+        </is>
+      </c>
+      <c r="B141" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C141" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D141" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>179.33</v>
+      </c>
+      <c r="E141" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>84.26</v>
+      </c>
+      <c r="F141" s="3">
+        <f>SUM(B141:E141)</f>
+        <v>342.43</v>
+      </c>
+      <c r="G141" s="3">
+        <f>F141/4</f>
+        <v>85.6075</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
-      <c r="B141" s="3">
+      <c r="B142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>78.84</v>
       </c>
-      <c r="C141" s="3">
+      <c r="C142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
-      <c r="D141" s="3">
+      <c r="D142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>586.29</v>
       </c>
-      <c r="E141" s="3">
+      <c r="E142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>503.92</v>
       </c>
-      <c r="F141" s="3">
-        <f>SUM(B141:E141)</f>
-        <v>1505.4</v>
-      </c>
-      <c r="G141" s="3">
-        <f>F141/4</f>
-        <v>376.35</v>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
-        </is>
-      </c>
-      <c r="B142" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="C142" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D142" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
-      </c>
-      <c r="E142" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
-      </c>
       <c r="F142" s="3">
         <f>SUM(B142:E142)</f>
-        <v>323.16</v>
+        <v>1505.4</v>
       </c>
       <c r="G142" s="3">
         <f>F142/4</f>
-        <v>80.79</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="B143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <v>80.79</v>
       </c>
       <c r="C143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>935.1</v>
+        <v>0</v>
       </c>
       <c r="D143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <v>161.58</v>
       </c>
       <c r="E143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>848.05</v>
+        <v>80.79</v>
       </c>
       <c r="F143" s="3">
         <f>SUM(B143:E143)</f>
-        <v>3765.22</v>
+        <v>323.16</v>
       </c>
       <c r="G143" s="3">
         <f>F143/4</f>
-        <v>941.305</v>
+        <v>80.79</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
         </is>
       </c>
       <c r="B144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>1019.45</v>
       </c>
       <c r="C144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>935.1</v>
       </c>
       <c r="D144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>962.62</v>
       </c>
       <c r="E144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>848.05</v>
       </c>
       <c r="F144" s="3">
         <f>SUM(B144:E144)</f>
-        <v>792.99</v>
+        <v>3765.22</v>
       </c>
       <c r="G144" s="3">
         <f>F144/4</f>
-        <v>198.2475</v>
+        <v>941.305</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F145" s="3">
+        <f>SUM(B145:E145)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G145" s="3">
+        <f>F145/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B145" s="3">
+      <c r="B146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C145" s="3">
+      <c r="C146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D145" s="3">
+      <c r="D146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E145" s="3">
+      <c r="E146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F145" s="3">
-        <f>SUM(B145:E145)</f>
-        <v>4932.41</v>
-      </c>
-      <c r="G145" s="3">
-        <f>F145/4</f>
-        <v>1233.1025</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
-        </is>
-      </c>
-      <c r="B146" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="C146" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D146" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="E146" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.5</v>
-      </c>
       <c r="F146" s="3">
         <f>SUM(B146:E146)</f>
-        <v>397.5</v>
+        <v>4932.41</v>
       </c>
       <c r="G146" s="3">
         <f>F146/4</f>
-        <v>99.375</v>
+        <v>1233.1025</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
+        </is>
+      </c>
+      <c r="B147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="C147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="E147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>32.5</v>
+      </c>
+      <c r="F147" s="3">
+        <f>SUM(B147:E147)</f>
+        <v>397.5</v>
+      </c>
+      <c r="G147" s="3">
+        <f>F147/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B147" s="3">
+      <c r="B148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C147" s="3">
+      <c r="C148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D147" s="3">
+      <c r="D148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E147" s="3">
+      <c r="E148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>357.62</v>
       </c>
-      <c r="F147" s="3">
-        <f>SUM(B147:E147)</f>
+      <c r="F148" s="3">
+        <f>SUM(B148:E148)</f>
         <v>4703.69</v>
       </c>
-      <c r="G147" s="3">
-        <f>F147/4</f>
+      <c r="G148" s="3">
+        <f>F148/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="12" t="inlineStr">
+    <row r="149">
+      <c r="A149" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B148" s="3">
+      <c r="B149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C148" s="3">
+      <c r="C149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D148" s="3">
+      <c r="D149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E148" s="3">
+      <c r="E149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F148" s="3">
-        <f>SUM(B148:E148)</f>
+      <c r="F149" s="3">
+        <f>SUM(B149:E149)</f>
         <v>737.73</v>
       </c>
-      <c r="G148" s="3">
-        <f>F148/4</f>
+      <c r="G149" s="3">
+        <f>F149/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="5" t="inlineStr">
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="27" customHeight="1">
-      <c r="A151" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="152" ht="27" customHeight="1">
       <c r="A152" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="153" ht="27" customHeight="1">
       <c r="A153" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="154" ht="27" customHeight="1">
       <c r="A154" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="155" ht="27" customHeight="1">
       <c r="A155" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="156" ht="27" customHeight="1">
       <c r="A156" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
         </is>
       </c>
     </row>
     <row r="157" ht="27" customHeight="1">
       <c r="A157" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="27" customHeight="1">
+      <c r="A158" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Small hospital-cafeteria charges (Granville Med, Duke) are counted as Restaurants.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A151:G151"/>
     <mergeCell ref="A152:G152"/>
     <mergeCell ref="A153:G153"/>
     <mergeCell ref="A154:G154"/>
     <mergeCell ref="A155:G155"/>
     <mergeCell ref="A156:G156"/>
     <mergeCell ref="A157:G157"/>
+    <mergeCell ref="A158:G158"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>

</xml_diff>

<commit_message>
Add CVS Pharmacy line item
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -1537,7 +1537,7 @@
     <row r="66">
       <c r="A66" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="B66" s="3">
@@ -1550,99 +1550,99 @@
       </c>
       <c r="D66" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A66,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>850.9</v>
+        <v>383.24</v>
       </c>
       <c r="E66" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A66,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>160.28</v>
+        <v>0</v>
       </c>
       <c r="F66" s="3">
         <f>SUM(B66:E66)</f>
-        <v>1272.18</v>
+        <v>644.24</v>
       </c>
       <c r="G66" s="3">
         <f>F66/4</f>
+        <v>161.06</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+        </is>
+      </c>
+      <c r="B67" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C67" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D67" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>467.66</v>
+      </c>
+      <c r="E67" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>160.28</v>
+      </c>
+      <c r="F67" s="3">
+        <f>SUM(B67:E67)</f>
+        <v>627.94</v>
+      </c>
+      <c r="G67" s="3">
+        <f>F67/4</f>
+        <v>156.985</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Health</t>
+        </is>
+      </c>
+      <c r="B68" s="6">
+        <f>SUM(B66:B67)</f>
+        <v>160.07</v>
+      </c>
+      <c r="C68" s="6">
+        <f>SUM(C66:C67)</f>
+        <v>100.93</v>
+      </c>
+      <c r="D68" s="6">
+        <f>SUM(D66:D67)</f>
+        <v>850.9</v>
+      </c>
+      <c r="E68" s="6">
+        <f>SUM(E66:E67)</f>
+        <v>160.28</v>
+      </c>
+      <c r="F68" s="6">
+        <f>SUM(F66:F67)</f>
+        <v>1272.18</v>
+      </c>
+      <c r="G68" s="6">
+        <f>F68/4</f>
         <v>318.045</v>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Health</t>
-        </is>
-      </c>
-      <c r="B67" s="6">
-        <f>SUM(B66:B66)</f>
-        <v>160.07</v>
-      </c>
-      <c r="C67" s="6">
-        <f>SUM(C66:C66)</f>
-        <v>100.93</v>
-      </c>
-      <c r="D67" s="6">
-        <f>SUM(D66:D66)</f>
-        <v>850.9</v>
-      </c>
-      <c r="E67" s="6">
-        <f>SUM(E66:E66)</f>
-        <v>160.28</v>
-      </c>
-      <c r="F67" s="6">
-        <f>SUM(F66:F66)</f>
-        <v>1272.18</v>
-      </c>
-      <c r="G67" s="6">
-        <f>F67/4</f>
-        <v>318.045</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="5" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Personal</t>
         </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
-        </is>
-      </c>
-      <c r="B70" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="C70" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D70" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="E70" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.5</v>
-      </c>
-      <c r="F70" s="3">
-        <f>SUM(B70:E70)</f>
-        <v>397.5</v>
-      </c>
-      <c r="G70" s="3">
-        <f>F70/4</f>
-        <v>99.375</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Personal Care – Simple Beauty</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="B71" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>182.5</v>
       </c>
       <c r="C71" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1650,134 +1650,134 @@
       </c>
       <c r="D71" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>182.5</v>
       </c>
       <c r="E71" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>82.0</v>
+        <v>32.5</v>
       </c>
       <c r="F71" s="3">
         <f>SUM(B71:E71)</f>
-        <v>82.0</v>
+        <v>397.5</v>
       </c>
       <c r="G71" s="3">
         <f>F71/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Personal Care – Simple Beauty</t>
+        </is>
+      </c>
+      <c r="B72" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C72" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D72" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E72" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>82.0</v>
+      </c>
+      <c r="F72" s="3">
+        <f>SUM(B72:E72)</f>
+        <v>82.0</v>
+      </c>
+      <c r="G72" s="3">
+        <f>F72/4</f>
         <v>20.5</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="7" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Personal</t>
         </is>
       </c>
-      <c r="B72" s="6">
-        <f>SUM(B70:B71)</f>
+      <c r="B73" s="6">
+        <f>SUM(B71:B72)</f>
         <v>182.5</v>
       </c>
-      <c r="C72" s="6">
-        <f>SUM(C70:C71)</f>
+      <c r="C73" s="6">
+        <f>SUM(C71:C72)</f>
         <v>0</v>
       </c>
-      <c r="D72" s="6">
-        <f>SUM(D70:D71)</f>
+      <c r="D73" s="6">
+        <f>SUM(D71:D72)</f>
         <v>182.5</v>
       </c>
-      <c r="E72" s="6">
-        <f>SUM(E70:E71)</f>
+      <c r="E73" s="6">
+        <f>SUM(E71:E72)</f>
         <v>114.5</v>
       </c>
-      <c r="F72" s="6">
-        <f>SUM(F70:F71)</f>
+      <c r="F73" s="6">
+        <f>SUM(F71:F72)</f>
         <v>479.5</v>
       </c>
-      <c r="G72" s="6">
-        <f>F72/4</f>
+      <c r="G73" s="6">
+        <f>F73/4</f>
         <v>119.875</v>
       </c>
     </row>
-    <row r="74">
-      <c r="A74" s="5" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Retail</t>
         </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Walmart</t>
-        </is>
-      </c>
-      <c r="B75" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C75" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>132.66</v>
-      </c>
-      <c r="D75" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1732.6</v>
-      </c>
-      <c r="E75" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.63</v>
-      </c>
-      <c r="F75" s="3">
-        <f>SUM(B75:E75)</f>
-        <v>1897.89</v>
-      </c>
-      <c r="G75" s="3">
-        <f>F75/4</f>
-        <v>474.4725</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Belk (store card payments)</t>
+          <t xml:space="preserve">Retail – Walmart</t>
         </is>
       </c>
       <c r="B76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>386.69</v>
+        <v>0</v>
       </c>
       <c r="C76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>948.04</v>
+        <v>132.66</v>
       </c>
       <c r="D76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1732.6</v>
       </c>
       <c r="E76" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>32.63</v>
       </c>
       <c r="F76" s="3">
         <f>SUM(B76:E76)</f>
-        <v>1334.73</v>
+        <v>1897.89</v>
       </c>
       <c r="G76" s="3">
         <f>F76/4</f>
-        <v>333.6825</v>
+        <v>474.4725</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Marshalls</t>
+          <t xml:space="preserve">Retail – Belk (store card payments)</t>
         </is>
       </c>
       <c r="B77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>386.69</v>
       </c>
       <c r="C77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>948.04</v>
       </c>
       <c r="D77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,D$4)</f>
@@ -1785,26 +1785,26 @@
       </c>
       <c r="E77" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>41.59</v>
+        <v>0</v>
       </c>
       <c r="F77" s="3">
         <f>SUM(B77:E77)</f>
-        <v>41.59</v>
+        <v>1334.73</v>
       </c>
       <c r="G77" s="3">
         <f>F77/4</f>
-        <v>10.3975</v>
+        <v>333.6825</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ross</t>
+          <t xml:space="preserve">Retail – Marshalls</t>
         </is>
       </c>
       <c r="B78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>48.03</v>
+        <v>0</v>
       </c>
       <c r="C78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1816,26 +1816,26 @@
       </c>
       <c r="E78" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>16.32</v>
+        <v>41.59</v>
       </c>
       <c r="F78" s="3">
         <f>SUM(B78:E78)</f>
-        <v>64.35</v>
+        <v>41.59</v>
       </c>
       <c r="G78" s="3">
         <f>F78/4</f>
-        <v>16.0875</v>
+        <v>10.3975</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dillard's</t>
+          <t xml:space="preserve">Retail – Ross</t>
         </is>
       </c>
       <c r="B79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>48.03</v>
       </c>
       <c r="C79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1843,30 +1843,30 @@
       </c>
       <c r="D79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>174.74</v>
+        <v>0</v>
       </c>
       <c r="E79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>16.32</v>
       </c>
       <c r="F79" s="3">
         <f>SUM(B79:E79)</f>
-        <v>174.74</v>
+        <v>64.35</v>
       </c>
       <c r="G79" s="3">
         <f>F79/4</f>
-        <v>43.685</v>
+        <v>16.0875</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Target</t>
+          <t xml:space="preserve">Retail – Dillard's</t>
         </is>
       </c>
       <c r="B80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>58.98</v>
+        <v>0</v>
       </c>
       <c r="C80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="D80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>174.74</v>
       </c>
       <c r="E80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1882,22 +1882,22 @@
       </c>
       <c r="F80" s="3">
         <f>SUM(B80:E80)</f>
-        <v>58.98</v>
+        <v>174.74</v>
       </c>
       <c r="G80" s="3">
         <f>F80/4</f>
-        <v>14.745</v>
+        <v>43.685</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – HomeSense</t>
+          <t xml:space="preserve">Retail – Target</t>
         </is>
       </c>
       <c r="B81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>58.98</v>
       </c>
       <c r="C81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="D81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>88.7</v>
+        <v>0</v>
       </c>
       <c r="E81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1913,17 +1913,17 @@
       </c>
       <c r="F81" s="3">
         <f>SUM(B81:E81)</f>
-        <v>88.7</v>
+        <v>58.98</v>
       </c>
       <c r="G81" s="3">
         <f>F81/4</f>
-        <v>22.175</v>
+        <v>14.745</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Hobby Lobby</t>
+          <t xml:space="preserve">Retail – HomeSense</t>
         </is>
       </c>
       <c r="B82" s="3">
@@ -1936,30 +1936,30 @@
       </c>
       <c r="D82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>165.67</v>
+        <v>88.7</v>
       </c>
       <c r="E82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>37.33</v>
+        <v>0</v>
       </c>
       <c r="F82" s="3">
         <f>SUM(B82:E82)</f>
-        <v>203.0</v>
+        <v>88.7</v>
       </c>
       <c r="G82" s="3">
         <f>F82/4</f>
-        <v>50.75</v>
+        <v>22.175</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
+          <t xml:space="preserve">Retail – Hobby Lobby</t>
         </is>
       </c>
       <c r="B83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>27.67</v>
+        <v>0</v>
       </c>
       <c r="C83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1967,30 +1967,30 @@
       </c>
       <c r="D83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>171.55</v>
+        <v>165.67</v>
       </c>
       <c r="E83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>85.27</v>
+        <v>37.33</v>
       </c>
       <c r="F83" s="3">
         <f>SUM(B83:E83)</f>
-        <v>284.49</v>
+        <v>203.0</v>
       </c>
       <c r="G83" s="3">
         <f>F83/4</f>
-        <v>71.1225</v>
+        <v>50.75</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Cat on a Whisk</t>
+          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
         </is>
       </c>
       <c r="B84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>27.67</v>
       </c>
       <c r="C84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1998,25 +1998,25 @@
       </c>
       <c r="D84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>171.55</v>
       </c>
       <c r="E84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>24.51</v>
+        <v>85.27</v>
       </c>
       <c r="F84" s="3">
         <f>SUM(B84:E84)</f>
-        <v>24.51</v>
+        <v>284.49</v>
       </c>
       <c r="G84" s="3">
         <f>F84/4</f>
-        <v>6.1275</v>
+        <v>71.1225</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Tractor Supply</t>
+          <t xml:space="preserve">Retail – Cat on a Whisk</t>
         </is>
       </c>
       <c r="B85" s="3">
@@ -2029,25 +2029,25 @@
       </c>
       <c r="D85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>29.86</v>
+        <v>0</v>
       </c>
       <c r="E85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>24.51</v>
       </c>
       <c r="F85" s="3">
         <f>SUM(B85:E85)</f>
-        <v>29.86</v>
+        <v>24.51</v>
       </c>
       <c r="G85" s="3">
         <f>F85/4</f>
-        <v>7.465</v>
+        <v>6.1275</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
+          <t xml:space="preserve">Retail – Tractor Supply</t>
         </is>
       </c>
       <c r="B86" s="3">
@@ -2056,11 +2056,11 @@
       </c>
       <c r="C86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>63.61</v>
+        <v>0</v>
       </c>
       <c r="D86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>29.86</v>
       </c>
       <c r="E86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2068,26 +2068,26 @@
       </c>
       <c r="F86" s="3">
         <f>SUM(B86:E86)</f>
-        <v>63.61</v>
+        <v>29.86</v>
       </c>
       <c r="G86" s="3">
         <f>F86/4</f>
-        <v>15.9025</v>
+        <v>7.465</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ulta Beauty</t>
+          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
         </is>
       </c>
       <c r="B87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>134.71</v>
+        <v>0</v>
       </c>
       <c r="C87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>63.61</v>
       </c>
       <c r="D87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,D$4)</f>
@@ -2099,22 +2099,22 @@
       </c>
       <c r="F87" s="3">
         <f>SUM(B87:E87)</f>
-        <v>134.71</v>
+        <v>63.61</v>
       </c>
       <c r="G87" s="3">
         <f>F87/4</f>
-        <v>33.6775</v>
+        <v>15.9025</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
+          <t xml:space="preserve">Retail – Ulta Beauty</t>
         </is>
       </c>
       <c r="B88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>51.31</v>
+        <v>134.71</v>
       </c>
       <c r="C88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -2130,30 +2130,30 @@
       </c>
       <c r="F88" s="3">
         <f>SUM(B88:E88)</f>
-        <v>51.31</v>
+        <v>134.71</v>
       </c>
       <c r="G88" s="3">
         <f>F88/4</f>
-        <v>12.8275</v>
+        <v>33.6775</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
         </is>
       </c>
       <c r="B89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>51.31</v>
       </c>
       <c r="C89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>5.87</v>
+        <v>0</v>
       </c>
       <c r="D89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>17.35</v>
+        <v>0</v>
       </c>
       <c r="E89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2161,286 +2161,286 @@
       </c>
       <c r="F89" s="3">
         <f>SUM(B89:E89)</f>
-        <v>23.22</v>
+        <v>51.31</v>
       </c>
       <c r="G89" s="3">
         <f>F89/4</f>
-        <v>5.805</v>
+        <v>12.8275</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
         </is>
       </c>
       <c r="B90" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.03</v>
+        <v>0</v>
       </c>
       <c r="C90" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>5.87</v>
       </c>
       <c r="D90" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>17.35</v>
       </c>
       <c r="E90" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>119.97</v>
+        <v>0</v>
       </c>
       <c r="F90" s="3">
         <f>SUM(B90:E90)</f>
-        <v>228.0</v>
+        <v>23.22</v>
       </c>
       <c r="G90" s="3">
         <f>F90/4</f>
+        <v>5.805</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+        </is>
+      </c>
+      <c r="B91" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.03</v>
+      </c>
+      <c r="C91" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D91" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E91" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>119.97</v>
+      </c>
+      <c r="F91" s="3">
+        <f>SUM(B91:E91)</f>
+        <v>228.0</v>
+      </c>
+      <c r="G91" s="3">
+        <f>F91/4</f>
         <v>57.0</v>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="7" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Retail</t>
         </is>
       </c>
-      <c r="B91" s="6">
-        <f>SUM(B75:B90)</f>
+      <c r="B92" s="6">
+        <f>SUM(B76:B91)</f>
         <v>815.42</v>
       </c>
-      <c r="C91" s="6">
-        <f>SUM(C75:C90)</f>
+      <c r="C92" s="6">
+        <f>SUM(C76:C91)</f>
         <v>1150.18</v>
       </c>
-      <c r="D91" s="6">
-        <f>SUM(D75:D90)</f>
+      <c r="D92" s="6">
+        <f>SUM(D76:D91)</f>
         <v>2380.47</v>
       </c>
-      <c r="E91" s="6">
-        <f>SUM(E75:E90)</f>
+      <c r="E92" s="6">
+        <f>SUM(E76:E91)</f>
         <v>357.62</v>
       </c>
-      <c r="F91" s="6">
-        <f>SUM(F75:F90)</f>
+      <c r="F92" s="6">
+        <f>SUM(F76:F91)</f>
         <v>4703.69</v>
       </c>
-      <c r="G91" s="6">
-        <f>F91/4</f>
+      <c r="G92" s="6">
+        <f>F92/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" s="5" t="inlineStr">
+    <row r="94">
+      <c r="A94" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Home</t>
         </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Yard Company (NextGen)</t>
-        </is>
-      </c>
-      <c r="B94" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>60.0</v>
-      </c>
-      <c r="C94" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.0</v>
-      </c>
-      <c r="D94" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>220.0</v>
-      </c>
-      <c r="E94" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>120.0</v>
-      </c>
-      <c r="F94" s="3">
-        <f>SUM(B94:E94)</f>
-        <v>500.0</v>
-      </c>
-      <c r="G94" s="3">
-        <f>F94/4</f>
-        <v>125.0</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
       <c r="B95" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>60.0</v>
       </c>
       <c r="C95" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>242.05</v>
+        <v>100.0</v>
       </c>
       <c r="D95" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>536.6</v>
+        <v>220.0</v>
       </c>
       <c r="E95" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>120.0</v>
       </c>
       <c r="F95" s="3">
         <f>SUM(B95:E95)</f>
-        <v>778.65</v>
+        <v>500.0</v>
       </c>
       <c r="G95" s="3">
         <f>F95/4</f>
+        <v>125.0</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+        </is>
+      </c>
+      <c r="B96" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C96" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>242.05</v>
+      </c>
+      <c r="D96" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>536.6</v>
+      </c>
+      <c r="E96" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F96" s="3">
+        <f>SUM(B96:E96)</f>
+        <v>778.65</v>
+      </c>
+      <c r="G96" s="3">
+        <f>F96/4</f>
         <v>194.6625</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="7" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Home</t>
         </is>
       </c>
-      <c r="B96" s="6">
-        <f>SUM(B94:B95)</f>
+      <c r="B97" s="6">
+        <f>SUM(B95:B96)</f>
         <v>60.0</v>
       </c>
-      <c r="C96" s="6">
-        <f>SUM(C94:C95)</f>
+      <c r="C97" s="6">
+        <f>SUM(C95:C96)</f>
         <v>342.05</v>
       </c>
-      <c r="D96" s="6">
-        <f>SUM(D94:D95)</f>
+      <c r="D97" s="6">
+        <f>SUM(D95:D96)</f>
         <v>756.6</v>
       </c>
-      <c r="E96" s="6">
-        <f>SUM(E94:E95)</f>
+      <c r="E97" s="6">
+        <f>SUM(E95:E96)</f>
         <v>120.0</v>
       </c>
-      <c r="F96" s="6">
-        <f>SUM(F94:F95)</f>
+      <c r="F97" s="6">
+        <f>SUM(F95:F96)</f>
         <v>1278.65</v>
       </c>
-      <c r="G96" s="6">
-        <f>F96/4</f>
+      <c r="G97" s="6">
+        <f>F97/4</f>
         <v>319.6625</v>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" s="5" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="12" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel (Lyft, Hotel)</t>
         </is>
       </c>
-      <c r="B99" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B100" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>102.65</v>
       </c>
-      <c r="C99" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C100" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D99" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D100" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E99" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E100" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F99" s="3">
-        <f>SUM(B99:E99)</f>
+      <c r="F100" s="3">
+        <f>SUM(B100:E100)</f>
         <v>102.65</v>
       </c>
-      <c r="G99" s="3">
-        <f>F99/4</f>
-        <v>25.6625</v>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Travel</t>
-        </is>
-      </c>
-      <c r="B100" s="6">
-        <f>SUM(B99:B99)</f>
-        <v>102.65</v>
-      </c>
-      <c r="C100" s="6">
-        <f>SUM(C99:C99)</f>
-        <v>0</v>
-      </c>
-      <c r="D100" s="6">
-        <f>SUM(D99:D99)</f>
-        <v>0</v>
-      </c>
-      <c r="E100" s="6">
-        <f>SUM(E99:E99)</f>
-        <v>0</v>
-      </c>
-      <c r="F100" s="6">
-        <f>SUM(F99:F99)</f>
-        <v>102.65</v>
-      </c>
-      <c r="G100" s="6">
+      <c r="G100" s="3">
         <f>F100/4</f>
         <v>25.6625</v>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="5" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Travel</t>
+        </is>
+      </c>
+      <c r="B101" s="6">
+        <f>SUM(B100:B100)</f>
+        <v>102.65</v>
+      </c>
+      <c r="C101" s="6">
+        <f>SUM(C100:C100)</f>
+        <v>0</v>
+      </c>
+      <c r="D101" s="6">
+        <f>SUM(D100:D100)</f>
+        <v>0</v>
+      </c>
+      <c r="E101" s="6">
+        <f>SUM(E100:E100)</f>
+        <v>0</v>
+      </c>
+      <c r="F101" s="6">
+        <f>SUM(F100:F100)</f>
+        <v>102.65</v>
+      </c>
+      <c r="G101" s="6">
+        <f>F101/4</f>
+        <v>25.6625</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Recreation</t>
         </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">St. James Marina</t>
-        </is>
-      </c>
-      <c r="B103" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C103" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>33.54</v>
-      </c>
-      <c r="D103" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E103" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F103" s="3">
-        <f>SUM(B103:E103)</f>
-        <v>33.54</v>
-      </c>
-      <c r="G103" s="3">
-        <f>F103/4</f>
-        <v>8.385</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">St. James Marina</t>
         </is>
       </c>
       <c r="B104" s="3">
@@ -2449,11 +2449,11 @@
       </c>
       <c r="C104" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>400.0</v>
+        <v>33.54</v>
       </c>
       <c r="D104" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>13.5</v>
+        <v>0</v>
       </c>
       <c r="E104" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2461,155 +2461,155 @@
       </c>
       <c r="F104" s="3">
         <f>SUM(B104:E104)</f>
-        <v>413.5</v>
+        <v>33.54</v>
       </c>
       <c r="G104" s="3">
         <f>F104/4</f>
+        <v>8.385</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Entertainment &amp; Events</t>
+        </is>
+      </c>
+      <c r="B105" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C105" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>400.0</v>
+      </c>
+      <c r="D105" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>13.5</v>
+      </c>
+      <c r="E105" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F105" s="3">
+        <f>SUM(B105:E105)</f>
+        <v>413.5</v>
+      </c>
+      <c r="G105" s="3">
+        <f>F105/4</f>
         <v>103.375</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="7" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Recreation</t>
         </is>
       </c>
-      <c r="B105" s="6">
-        <f>SUM(B103:B104)</f>
+      <c r="B106" s="6">
+        <f>SUM(B104:B105)</f>
         <v>0</v>
       </c>
-      <c r="C105" s="6">
-        <f>SUM(C103:C104)</f>
+      <c r="C106" s="6">
+        <f>SUM(C104:C105)</f>
         <v>433.54</v>
       </c>
-      <c r="D105" s="6">
-        <f>SUM(D103:D104)</f>
+      <c r="D106" s="6">
+        <f>SUM(D104:D105)</f>
         <v>13.5</v>
       </c>
-      <c r="E105" s="6">
-        <f>SUM(E103:E104)</f>
+      <c r="E106" s="6">
+        <f>SUM(E104:E105)</f>
         <v>0</v>
       </c>
-      <c r="F105" s="6">
-        <f>SUM(F103:F104)</f>
+      <c r="F106" s="6">
+        <f>SUM(F104:F105)</f>
         <v>447.04</v>
       </c>
-      <c r="G105" s="6">
-        <f>F105/4</f>
+      <c r="G106" s="6">
+        <f>F106/4</f>
         <v>111.76</v>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="5" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="12" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
         </is>
       </c>
-      <c r="B108" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B109" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>75.0</v>
       </c>
-      <c r="C108" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C109" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>764.05</v>
       </c>
-      <c r="D108" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D109" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>331.5</v>
       </c>
-      <c r="E108" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E109" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>130.0</v>
       </c>
-      <c r="F108" s="3">
-        <f>SUM(B108:E108)</f>
+      <c r="F109" s="3">
+        <f>SUM(B109:E109)</f>
         <v>1300.55</v>
       </c>
-      <c r="G108" s="3">
-        <f>F108/4</f>
-        <v>325.1375</v>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total Transfers</t>
-        </is>
-      </c>
-      <c r="B109" s="6">
-        <f>SUM(B108:B108)</f>
-        <v>75.0</v>
-      </c>
-      <c r="C109" s="6">
-        <f>SUM(C108:C108)</f>
-        <v>764.05</v>
-      </c>
-      <c r="D109" s="6">
-        <f>SUM(D108:D108)</f>
-        <v>331.5</v>
-      </c>
-      <c r="E109" s="6">
-        <f>SUM(E108:E108)</f>
-        <v>130.0</v>
-      </c>
-      <c r="F109" s="6">
-        <f>SUM(F108:F108)</f>
-        <v>1300.55</v>
-      </c>
-      <c r="G109" s="6">
+      <c r="G109" s="3">
         <f>F109/4</f>
         <v>325.1375</v>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="5" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total Transfers</t>
+        </is>
+      </c>
+      <c r="B110" s="6">
+        <f>SUM(B109:B109)</f>
+        <v>75.0</v>
+      </c>
+      <c r="C110" s="6">
+        <f>SUM(C109:C109)</f>
+        <v>764.05</v>
+      </c>
+      <c r="D110" s="6">
+        <f>SUM(D109:D109)</f>
+        <v>331.5</v>
+      </c>
+      <c r="E110" s="6">
+        <f>SUM(E109:E109)</f>
+        <v>130.0</v>
+      </c>
+      <c r="F110" s="6">
+        <f>SUM(F109:F109)</f>
+        <v>1300.55</v>
+      </c>
+      <c r="G110" s="6">
+        <f>F110/4</f>
+        <v>325.1375</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Other</t>
         </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Donations &amp; Clubs (Kiwanis)</t>
-        </is>
-      </c>
-      <c r="B112" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C112" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D112" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E112" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>200.0</v>
-      </c>
-      <c r="F112" s="3">
-        <f>SUM(B112:E112)</f>
-        <v>200.0</v>
-      </c>
-      <c r="G112" s="3">
-        <f>F112/4</f>
-        <v>50.0</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
+          <t xml:space="preserve">Donations &amp; Clubs (Kiwanis)</t>
         </is>
       </c>
       <c r="B113" s="3">
@@ -2626,152 +2626,152 @@
       </c>
       <c r="E113" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>147.0</v>
+        <v>200.0</v>
       </c>
       <c r="F113" s="3">
         <f>SUM(B113:E113)</f>
-        <v>147.0</v>
+        <v>200.0</v>
       </c>
       <c r="G113" s="3">
         <f>F113/4</f>
+        <v>50.0</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
+        </is>
+      </c>
+      <c r="B114" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C114" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D114" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E114" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>147.0</v>
+      </c>
+      <c r="F114" s="3">
+        <f>SUM(B114:E114)</f>
+        <v>147.0</v>
+      </c>
+      <c r="G114" s="3">
+        <f>F114/4</f>
         <v>36.75</v>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="7" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Other</t>
         </is>
       </c>
-      <c r="B114" s="6">
-        <f>SUM(B112:B113)</f>
+      <c r="B115" s="6">
+        <f>SUM(B113:B114)</f>
         <v>0</v>
       </c>
-      <c r="C114" s="6">
-        <f>SUM(C112:C113)</f>
+      <c r="C115" s="6">
+        <f>SUM(C113:C114)</f>
         <v>0</v>
       </c>
-      <c r="D114" s="6">
-        <f>SUM(D112:D113)</f>
+      <c r="D115" s="6">
+        <f>SUM(D113:D114)</f>
         <v>0</v>
       </c>
-      <c r="E114" s="6">
-        <f>SUM(E112:E113)</f>
+      <c r="E115" s="6">
+        <f>SUM(E113:E114)</f>
         <v>347.0</v>
       </c>
-      <c r="F114" s="6">
-        <f>SUM(F112:F113)</f>
+      <c r="F115" s="6">
+        <f>SUM(F113:F114)</f>
         <v>347.0</v>
       </c>
-      <c r="G114" s="6">
-        <f>F114/4</f>
+      <c r="G115" s="6">
+        <f>F115/4</f>
         <v>86.75</v>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="8" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL SPENDING</t>
         </is>
       </c>
-      <c r="B116" s="9">
-        <f>B10+B18+B23+B28+B32+B38+B43+B48+B59+B63+B67+B72+B91+B96+B100+B105+B109+B114</f>
+      <c r="B117" s="9">
+        <f>B10+B18+B23+B28+B32+B38+B43+B48+B59+B63+B68+B73+B92+B97+B101+B106+B110+B115</f>
         <v>12135.81</v>
       </c>
-      <c r="C116" s="9">
-        <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C67+C72+C91+C96+C100+C105+C109+C114</f>
+      <c r="C117" s="9">
+        <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C68+C73+C92+C97+C101+C106+C110+C115</f>
         <v>12663.24</v>
       </c>
-      <c r="D116" s="9">
-        <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D67+D72+D91+D96+D100+D105+D109+D114</f>
+      <c r="D117" s="9">
+        <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D68+D73+D92+D97+D101+D106+D110+D115</f>
         <v>15086.64</v>
       </c>
-      <c r="E116" s="9">
-        <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E67+E72+E91+E96+E100+E105+E109+E114</f>
+      <c r="E117" s="9">
+        <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E68+E73+E92+E97+E101+E106+E110+E115</f>
         <v>11515.63</v>
       </c>
-      <c r="F116" s="9">
-        <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F67+F72+F91+F96+F100+F105+F109+F114</f>
+      <c r="F117" s="9">
+        <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F68+F73+F92+F97+F101+F106+F110+F115</f>
         <v>51401.32</v>
       </c>
-      <c r="G116" s="9">
-        <f>F116/4</f>
+      <c r="G117" s="9">
+        <f>F117/4</f>
         <v>12850.33</v>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="5" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Not counted as spending</t>
         </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
-        </is>
-      </c>
-      <c r="B119" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="C119" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="D119" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="E119" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A119,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="F119" s="3">
-        <f>SUM(B119:E119)</f>
-        <v>10304.0</v>
-      </c>
-      <c r="G119" s="3">
-        <f>F119/4</f>
-        <v>2576.0</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
         </is>
       </c>
       <c r="B120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>2576.0</v>
       </c>
       <c r="C120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>7227.09</v>
+        <v>2576.0</v>
       </c>
       <c r="D120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>4593.08</v>
+        <v>2576.0</v>
       </c>
       <c r="E120" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>4738.51</v>
+        <v>2576.0</v>
       </c>
       <c r="F120" s="3">
         <f>SUM(B120:E120)</f>
-        <v>16558.68</v>
+        <v>10304.0</v>
       </c>
       <c r="G120" s="3">
         <f>F120/4</f>
-        <v>4139.67</v>
+        <v>2576.0</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sloane Realty</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="B121" s="3">
@@ -2780,42 +2780,42 @@
       </c>
       <c r="C121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2891.98</v>
+        <v>7227.09</v>
       </c>
       <c r="D121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>4593.08</v>
       </c>
       <c r="E121" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>4738.51</v>
       </c>
       <c r="F121" s="3">
         <f>SUM(B121:E121)</f>
-        <v>2891.98</v>
+        <v>16558.68</v>
       </c>
       <c r="G121" s="3">
         <f>F121/4</f>
-        <v>722.995</v>
+        <v>4139.67</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checks Written (payee not shown)</t>
+          <t xml:space="preserve">Sloane Realty</t>
         </is>
       </c>
       <c r="B122" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2630.0</v>
+        <v>0</v>
       </c>
       <c r="C122" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>2891.98</v>
       </c>
       <c r="D122" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>728.0</v>
+        <v>0</v>
       </c>
       <c r="E122" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2823,30 +2823,30 @@
       </c>
       <c r="F122" s="3">
         <f>SUM(B122:E122)</f>
-        <v>3358.0</v>
+        <v>2891.98</v>
       </c>
       <c r="G122" s="3">
         <f>F122/4</f>
-        <v>839.5</v>
+        <v>722.995</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Checks Written (payee not shown)</t>
         </is>
       </c>
       <c r="B123" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>2630.0</v>
       </c>
       <c r="C123" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3.26</v>
+        <v>0</v>
       </c>
       <c r="D123" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>728.0</v>
       </c>
       <c r="E123" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2854,515 +2854,515 @@
       </c>
       <c r="F123" s="3">
         <f>SUM(B123:E123)</f>
-        <v>3.26</v>
+        <v>3358.0</v>
       </c>
       <c r="G123" s="3">
         <f>F123/4</f>
+        <v>839.5</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
+        </is>
+      </c>
+      <c r="B124" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C124" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>3.26</v>
+      </c>
+      <c r="D124" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E124" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F124" s="3">
+        <f>SUM(B124:E124)</f>
+        <v>3.26</v>
+      </c>
+      <c r="G124" s="3">
+        <f>F124/4</f>
         <v>0.815</v>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="7" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total not counted as spending</t>
         </is>
       </c>
-      <c r="B124" s="6">
-        <f>SUM(B119:B123)</f>
+      <c r="B125" s="6">
+        <f>SUM(B120:B124)</f>
         <v>5206.0</v>
       </c>
-      <c r="C124" s="6">
-        <f>SUM(C119:C123)</f>
+      <c r="C125" s="6">
+        <f>SUM(C120:C124)</f>
         <v>12698.33</v>
       </c>
-      <c r="D124" s="6">
-        <f>SUM(D119:D123)</f>
+      <c r="D125" s="6">
+        <f>SUM(D120:D124)</f>
         <v>7897.08</v>
       </c>
-      <c r="E124" s="6">
-        <f>SUM(E119:E123)</f>
+      <c r="E125" s="6">
+        <f>SUM(E120:E124)</f>
         <v>7314.51</v>
       </c>
-      <c r="F124" s="6">
-        <f>SUM(F119:F123)</f>
+      <c r="F125" s="6">
+        <f>SUM(F120:F124)</f>
         <v>33115.92</v>
       </c>
-      <c r="G124" s="6">
-        <f>F124/4</f>
+      <c r="G125" s="6">
+        <f>F125/4</f>
         <v>8278.98</v>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Check: spending + not-counted items</t>
-        </is>
-      </c>
-      <c r="B126" s="3">
-        <f>B116+B124</f>
-        <v>17341.81</v>
-      </c>
-      <c r="C126" s="3">
-        <f>C116+C124</f>
-        <v>25361.57</v>
-      </c>
-      <c r="D126" s="3">
-        <f>D116+D124</f>
-        <v>22983.72</v>
-      </c>
-      <c r="E126" s="3">
-        <f>E116+E124</f>
-        <v>18830.14</v>
-      </c>
-      <c r="F126" s="3">
-        <f>F116+F124</f>
-        <v>84517.24</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
-        </is>
-      </c>
-      <c r="B127" s="13">
+          <t xml:space="preserve">Check: spending + not-counted items</t>
+        </is>
+      </c>
+      <c r="B127" s="3">
+        <f>B117+B125</f>
         <v>17341.81</v>
       </c>
-      <c r="C127" s="13">
+      <c r="C127" s="3">
+        <f>C117+C125</f>
         <v>25361.57</v>
       </c>
-      <c r="D127" s="13">
+      <c r="D127" s="3">
+        <f>D117+D125</f>
         <v>22983.72</v>
       </c>
-      <c r="E127" s="13">
+      <c r="E127" s="3">
+        <f>E117+E125</f>
         <v>18830.14</v>
       </c>
       <c r="F127" s="3">
-        <f>SUM(B127:E127)</f>
+        <f>F117+F125</f>
         <v>84517.24</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
+        </is>
+      </c>
+      <c r="B128" s="13">
+        <v>17341.81</v>
+      </c>
+      <c r="C128" s="13">
+        <v>25361.57</v>
+      </c>
+      <c r="D128" s="13">
+        <v>22983.72</v>
+      </c>
+      <c r="E128" s="13">
+        <v>18830.14</v>
+      </c>
+      <c r="F128" s="3">
+        <f>SUM(B128:E128)</f>
+        <v>84517.24</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Difference (should be $0 = every dollar accounted for)</t>
         </is>
       </c>
-      <c r="B128" s="3">
-        <f>B126-B127</f>
+      <c r="B129" s="3">
+        <f>B127-B128</f>
         <v>0.0</v>
       </c>
-      <c r="C128" s="3">
-        <f>C126-C127</f>
+      <c r="C129" s="3">
+        <f>C127-C128</f>
         <v>0.0</v>
       </c>
-      <c r="D128" s="3">
-        <f>D126-D127</f>
+      <c r="D129" s="3">
+        <f>D127-D128</f>
         <v>0.0</v>
       </c>
-      <c r="E128" s="3">
-        <f>E126-E127</f>
+      <c r="E129" s="3">
+        <f>E127-E128</f>
         <v>0.0</v>
       </c>
-      <c r="F128" s="3">
-        <f>F126-F127</f>
+      <c r="F129" s="3">
+        <f>F127-F128</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="130">
-      <c r="A130" s="5" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Key Bills at a Glance</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="15" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Bill</t>
         </is>
       </c>
-      <c r="B131" s="1" t="inlineStr">
+      <c r="B132" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">June 2026</t>
         </is>
       </c>
-      <c r="C131" s="1" t="inlineStr">
+      <c r="C132" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">July 2026</t>
         </is>
       </c>
-      <c r="D131" s="1" t="inlineStr">
+      <c r="D132" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">August 2026</t>
         </is>
       </c>
-      <c r="E131" s="1" t="inlineStr">
+      <c r="E132" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">September 2026</t>
         </is>
       </c>
-      <c r="F131" s="1" t="inlineStr">
+      <c r="F132" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">4-Month Total</t>
         </is>
       </c>
-      <c r="G131" s="1" t="inlineStr">
+      <c r="G132" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Monthly Avg</t>
         </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A&amp;D Mortgage</t>
-        </is>
-      </c>
-      <c r="B132" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="C132" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="D132" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="E132" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A132,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="F132" s="3">
-        <f>SUM(B132:E132)</f>
-        <v>13644.4</v>
-      </c>
-      <c r="G132" s="3">
-        <f>F132/4</f>
-        <v>3411.1</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Membership (Club)</t>
+          <t xml:space="preserve">A&amp;D Mortgage</t>
         </is>
       </c>
       <c r="B133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1591.78</v>
+        <v>3411.1</v>
       </c>
       <c r="C133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>1601.56</v>
+        <v>3411.1</v>
       </c>
       <c r="D133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1492.11</v>
+        <v>3411.1</v>
       </c>
       <c r="E133" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>1767.0</v>
+        <v>3411.1</v>
       </c>
       <c r="F133" s="3">
         <f>SUM(B133:E133)</f>
-        <v>6452.45</v>
+        <v>13644.4</v>
       </c>
       <c r="G133" s="3">
         <f>F133/4</f>
-        <v>1613.1125</v>
+        <v>3411.1</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Plantation POA Dues</t>
+          <t xml:space="preserve">St. James Membership (Club)</t>
         </is>
       </c>
       <c r="B134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>692.95</v>
+        <v>1591.78</v>
       </c>
       <c r="C134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>1601.56</v>
       </c>
       <c r="D134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1492.11</v>
       </c>
       <c r="E134" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>1767.0</v>
       </c>
       <c r="F134" s="3">
         <f>SUM(B134:E134)</f>
-        <v>692.95</v>
+        <v>6452.45</v>
       </c>
       <c r="G134" s="3">
         <f>F134/4</f>
-        <v>173.2375</v>
+        <v>1613.1125</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">St. James Plantation POA Dues</t>
         </is>
       </c>
       <c r="B135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>360.42</v>
+        <v>692.95</v>
       </c>
       <c r="C135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>360.42</v>
+        <v>0</v>
       </c>
       <c r="D135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>475.42</v>
+        <v>0</v>
       </c>
       <c r="E135" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>354.17</v>
+        <v>0</v>
       </c>
       <c r="F135" s="3">
         <f>SUM(B135:E135)</f>
-        <v>1550.43</v>
+        <v>692.95</v>
       </c>
       <c r="G135" s="3">
         <f>F135/4</f>
-        <v>387.6075</v>
+        <v>173.2375</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="B136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>79.21</v>
+        <v>360.42</v>
       </c>
       <c r="C136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>73.61</v>
+        <v>360.42</v>
       </c>
       <c r="D136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>73.61</v>
+        <v>475.42</v>
       </c>
       <c r="E136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>73.61</v>
+        <v>354.17</v>
       </c>
       <c r="F136" s="3">
         <f>SUM(B136:E136)</f>
-        <v>300.04</v>
+        <v>1550.43</v>
       </c>
       <c r="G136" s="3">
         <f>F136/4</f>
-        <v>75.01</v>
+        <v>387.6075</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Banner Life Insurance</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="B137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>710.06</v>
+        <v>79.21</v>
       </c>
       <c r="C137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="D137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="E137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="F137" s="3">
         <f>SUM(B137:E137)</f>
-        <v>2840.24</v>
+        <v>300.04</v>
       </c>
       <c r="G137" s="3">
         <f>F137/4</f>
-        <v>710.06</v>
+        <v>75.01</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Banner Life Insurance</t>
         </is>
       </c>
       <c r="B138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>710.06</v>
       </c>
       <c r="C138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>710.06</v>
       </c>
       <c r="D138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>710.06</v>
       </c>
       <c r="E138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>710.06</v>
       </c>
       <c r="F138" s="3">
         <f>SUM(B138:E138)</f>
-        <v>1412.24</v>
+        <v>2840.24</v>
       </c>
       <c r="G138" s="3">
         <f>F138/4</f>
-        <v>353.06</v>
+        <v>710.06</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.37</v>
+        <v>294.57</v>
       </c>
       <c r="C139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>160.37</v>
+        <v>294.8</v>
       </c>
       <c r="D139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>160.37</v>
+        <v>436.02</v>
       </c>
       <c r="E139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>160.37</v>
+        <v>386.85</v>
       </c>
       <c r="F139" s="3">
         <f>SUM(B139:E139)</f>
-        <v>641.48</v>
+        <v>1412.24</v>
       </c>
       <c r="G139" s="3">
         <f>F139/4</f>
-        <v>160.37</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="B140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>160.37</v>
       </c>
       <c r="C140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>160.37</v>
       </c>
       <c r="D140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>160.37</v>
       </c>
       <c r="E140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>160.37</v>
       </c>
       <c r="F140" s="3">
         <f>SUM(B140:E140)</f>
-        <v>1162.97</v>
+        <v>641.48</v>
       </c>
       <c r="G140" s="3">
         <f>F140/4</f>
-        <v>290.7425</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="B141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>160.07</v>
       </c>
       <c r="C141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>100.93</v>
       </c>
       <c r="D141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>383.24</v>
       </c>
       <c r="E141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>0</v>
       </c>
       <c r="F141" s="3">
         <f>SUM(B141:E141)</f>
-        <v>342.43</v>
+        <v>644.24</v>
       </c>
       <c r="G141" s="3">
         <f>F141/4</f>
-        <v>85.6075</v>
+        <v>161.06</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B142" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
       </c>
       <c r="C142" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
       <c r="D142" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>586.29</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>406.96</v>
       </c>
       <c r="E142" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>503.92</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>419.66</v>
       </c>
       <c r="F142" s="3">
         <f>SUM(B142:E142)</f>
-        <v>1505.4</v>
+        <v>1162.97</v>
       </c>
       <c r="G142" s="3">
         <f>F142/4</f>
-        <v>376.35</v>
+        <v>290.7425</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
         </is>
       </c>
       <c r="B143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
+        <v>78.84</v>
       </c>
       <c r="C143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -3370,272 +3370,334 @@
       </c>
       <c r="D143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
+        <v>179.33</v>
       </c>
       <c r="E143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
+        <v>84.26</v>
       </c>
       <c r="F143" s="3">
         <f>SUM(B143:E143)</f>
-        <v>323.16</v>
+        <v>342.43</v>
       </c>
       <c r="G143" s="3">
         <f>F143/4</f>
-        <v>80.79</v>
+        <v>85.6075</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
       <c r="B144" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
       </c>
       <c r="C144" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>935.1</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>336.35</v>
       </c>
       <c r="D144" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>586.29</v>
       </c>
       <c r="E144" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>848.05</v>
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>503.92</v>
       </c>
       <c r="F144" s="3">
         <f>SUM(B144:E144)</f>
-        <v>3765.22</v>
+        <v>1505.4</v>
       </c>
       <c r="G144" s="3">
         <f>F144/4</f>
-        <v>941.305</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="B145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>80.79</v>
       </c>
       <c r="C145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>0</v>
       </c>
       <c r="D145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>161.58</v>
       </c>
       <c r="E145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>80.79</v>
       </c>
       <c r="F145" s="3">
         <f>SUM(B145:E145)</f>
-        <v>792.99</v>
+        <v>323.16</v>
       </c>
       <c r="G145" s="3">
         <f>F145/4</f>
-        <v>198.2475</v>
+        <v>80.79</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+        </is>
+      </c>
+      <c r="B146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>1019.45</v>
+      </c>
+      <c r="C146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>935.1</v>
+      </c>
+      <c r="D146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>962.62</v>
+      </c>
+      <c r="E146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>848.05</v>
+      </c>
+      <c r="F146" s="3">
+        <f>SUM(B146:E146)</f>
+        <v>3765.22</v>
+      </c>
+      <c r="G146" s="3">
+        <f>F146/4</f>
+        <v>941.305</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F147" s="3">
+        <f>SUM(B147:E147)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G147" s="3">
+        <f>F147/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B146" s="3">
+      <c r="B148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C146" s="3">
+      <c r="C148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D146" s="3">
+      <c r="D148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E146" s="3">
+      <c r="E148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F146" s="3">
-        <f>SUM(B146:E146)</f>
+      <c r="F148" s="3">
+        <f>SUM(B148:E148)</f>
         <v>4932.41</v>
       </c>
-      <c r="G146" s="3">
-        <f>F146/4</f>
+      <c r="G148" s="3">
+        <f>F148/4</f>
         <v>1233.1025</v>
       </c>
     </row>
-    <row r="147">
-      <c r="A147" s="12" t="inlineStr">
+    <row r="149">
+      <c r="A149" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
-      <c r="B147" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>182.5</v>
       </c>
-      <c r="C147" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D147" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>182.5</v>
       </c>
-      <c r="E147" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>32.5</v>
       </c>
-      <c r="F147" s="3">
-        <f>SUM(B147:E147)</f>
+      <c r="F149" s="3">
+        <f>SUM(B149:E149)</f>
         <v>397.5</v>
       </c>
-      <c r="G147" s="3">
-        <f>F147/4</f>
+      <c r="G149" s="3">
+        <f>F149/4</f>
         <v>99.375</v>
       </c>
     </row>
-    <row r="148">
-      <c r="A148" s="12" t="inlineStr">
+    <row r="150">
+      <c r="A150" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B148" s="3">
+      <c r="B150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C148" s="3">
+      <c r="C150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D148" s="3">
+      <c r="D150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E148" s="3">
+      <c r="E150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>357.62</v>
       </c>
-      <c r="F148" s="3">
-        <f>SUM(B148:E148)</f>
+      <c r="F150" s="3">
+        <f>SUM(B150:E150)</f>
         <v>4703.69</v>
       </c>
-      <c r="G148" s="3">
-        <f>F148/4</f>
+      <c r="G150" s="3">
+        <f>F150/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" s="12" t="inlineStr">
+    <row r="151">
+      <c r="A151" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B149" s="3">
+      <c r="B151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C149" s="3">
+      <c r="C151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D149" s="3">
+      <c r="D151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E149" s="3">
+      <c r="E151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F149" s="3">
-        <f>SUM(B149:E149)</f>
+      <c r="F151" s="3">
+        <f>SUM(B151:E151)</f>
         <v>737.73</v>
       </c>
-      <c r="G149" s="3">
-        <f>F149/4</f>
+      <c r="G151" s="3">
+        <f>F151/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="5" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="27" customHeight="1">
-      <c r="A152" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="27" customHeight="1">
-      <c r="A153" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="154" ht="27" customHeight="1">
       <c r="A154" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="155" ht="27" customHeight="1">
       <c r="A155" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="156" ht="27" customHeight="1">
       <c r="A156" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="157" ht="27" customHeight="1">
       <c r="A157" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="158" ht="27" customHeight="1">
       <c r="A158" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="27" customHeight="1">
+      <c r="A159" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="27" customHeight="1">
+      <c r="A160" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Small hospital-cafeteria charges (Granville Med, Duke) are counted as Restaurants.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A152:G152"/>
-    <mergeCell ref="A153:G153"/>
     <mergeCell ref="A154:G154"/>
     <mergeCell ref="A155:G155"/>
     <mergeCell ref="A156:G156"/>
     <mergeCell ref="A157:G157"/>
     <mergeCell ref="A158:G158"/>
+    <mergeCell ref="A159:G159"/>
+    <mergeCell ref="A160:G160"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -4140,7 +4202,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="H17" s="3">
@@ -5554,7 +5616,7 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
       <c r="E68" s="3">
@@ -6538,7 +6600,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -6584,7 +6646,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -7424,7 +7486,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="H22" s="3">
@@ -7699,7 +7761,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -8646,7 +8708,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -8904,7 +8966,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
       <c r="E79" s="3">
@@ -9612,7 +9674,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -10257,12 +10319,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Banner Life Insurance</t>
         </is>
       </c>
       <c r="H8" s="3">
         <f>SUMIF($C$4:$C$110,G8,$E$4:$E$110)</f>
-        <v>850.9</v>
+        <v>710.06</v>
       </c>
     </row>
     <row r="9">
@@ -10289,12 +10351,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Banner Life Insurance</t>
+          <t xml:space="preserve">Grocery – Lowes Foods</t>
         </is>
       </c>
       <c r="H9" s="3">
         <f>SUMIF($C$4:$C$110,G9,$E$4:$E$110)</f>
-        <v>710.06</v>
+        <v>584.25</v>
       </c>
     </row>
     <row r="10">
@@ -10321,12 +10383,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grocery – Lowes Foods</t>
+          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
         </is>
       </c>
       <c r="H10" s="3">
         <f>SUMIF($C$4:$C$110,G10,$E$4:$E$110)</f>
-        <v>584.25</v>
+        <v>536.6</v>
       </c>
     </row>
     <row r="11">
@@ -10353,12 +10415,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Grocery – Publix</t>
         </is>
       </c>
       <c r="H11" s="3">
         <f>SUMIF($C$4:$C$110,G11,$E$4:$E$110)</f>
-        <v>536.6</v>
+        <v>522.68</v>
       </c>
     </row>
     <row r="12">
@@ -10385,12 +10447,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grocery – Publix</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="H12" s="3">
         <f>SUMIF($C$4:$C$110,G12,$E$4:$E$110)</f>
-        <v>522.68</v>
+        <v>475.42</v>
       </c>
     </row>
     <row r="13">
@@ -10417,12 +10479,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="H13" s="3">
         <f>SUMIF($C$4:$C$110,G13,$E$4:$E$110)</f>
-        <v>475.42</v>
+        <v>467.66</v>
       </c>
     </row>
     <row r="14">
@@ -10532,7 +10594,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -10545,12 +10607,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="H17" s="3">
         <f>SUMIF($C$4:$C$110,G17,$E$4:$E$110)</f>
-        <v>331.5</v>
+        <v>383.24</v>
       </c>
     </row>
     <row r="18">
@@ -10577,12 +10639,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yard Company (NextGen)</t>
+          <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
         </is>
       </c>
       <c r="H18" s="3">
         <f>SUMIF($C$4:$C$110,G18,$E$4:$E$110)</f>
-        <v>220.0</v>
+        <v>331.5</v>
       </c>
     </row>
     <row r="19">
@@ -10609,12 +10671,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
+          <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
       <c r="H19" s="3">
         <f>SUMIF($C$4:$C$110,G19,$E$4:$E$110)</f>
-        <v>182.5</v>
+        <v>220.0</v>
       </c>
     </row>
     <row r="20">
@@ -10641,12 +10703,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="H20" s="3">
         <f>SUMIF($C$4:$C$110,G20,$E$4:$E$110)</f>
-        <v>179.33</v>
+        <v>182.5</v>
       </c>
     </row>
     <row r="21">
@@ -10673,12 +10735,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dillard's</t>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
         </is>
       </c>
       <c r="H21" s="3">
         <f>SUMIF($C$4:$C$110,G21,$E$4:$E$110)</f>
-        <v>174.74</v>
+        <v>179.33</v>
       </c>
     </row>
     <row r="22">
@@ -10705,12 +10767,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
+          <t xml:space="preserve">Retail – Dillard's</t>
         </is>
       </c>
       <c r="H22" s="3">
         <f>SUMIF($C$4:$C$110,G22,$E$4:$E$110)</f>
-        <v>171.55</v>
+        <v>174.74</v>
       </c>
     </row>
     <row r="23">
@@ -10737,12 +10799,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
         </is>
       </c>
       <c r="H23" s="3">
         <f>SUMIF($C$4:$C$110,G23,$E$4:$E$110)</f>
-        <v>167.24</v>
+        <v>171.55</v>
       </c>
     </row>
     <row r="24">
@@ -10769,12 +10831,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Hobby Lobby</t>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
         </is>
       </c>
       <c r="H24" s="3">
         <f>SUMIF($C$4:$C$110,G24,$E$4:$E$110)</f>
-        <v>165.67</v>
+        <v>167.24</v>
       </c>
     </row>
     <row r="25">
@@ -10801,12 +10863,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
+          <t xml:space="preserve">Retail – Hobby Lobby</t>
         </is>
       </c>
       <c r="H25" s="3">
         <f>SUMIF($C$4:$C$110,G25,$E$4:$E$110)</f>
-        <v>161.58</v>
+        <v>165.67</v>
       </c>
     </row>
     <row r="26">
@@ -10833,12 +10895,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="H26" s="3">
         <f>SUMIF($C$4:$C$110,G26,$E$4:$E$110)</f>
-        <v>160.37</v>
+        <v>161.58</v>
       </c>
     </row>
     <row r="27">
@@ -10865,12 +10927,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – YouTube TV (Google)</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="H27" s="3">
         <f>SUMIF($C$4:$C$110,G27,$E$4:$E$110)</f>
-        <v>89.0</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="28">
@@ -10897,12 +10959,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – HomeSense</t>
+          <t xml:space="preserve">Streaming – YouTube TV (Google)</t>
         </is>
       </c>
       <c r="H28" s="3">
         <f>SUMIF($C$4:$C$110,G28,$E$4:$E$110)</f>
-        <v>88.7</v>
+        <v>89.0</v>
       </c>
     </row>
     <row r="29">
@@ -10929,12 +10991,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grocery – Food Lion</t>
+          <t xml:space="preserve">Retail – HomeSense</t>
         </is>
       </c>
       <c r="H29" s="3">
         <f>SUMIF($C$4:$C$110,G29,$E$4:$E$110)</f>
-        <v>77.34</v>
+        <v>88.7</v>
       </c>
     </row>
     <row r="30">
@@ -10961,12 +11023,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">Grocery – Food Lion</t>
         </is>
       </c>
       <c r="H30" s="3">
         <f>SUMIF($C$4:$C$110,G30,$E$4:$E$110)</f>
-        <v>73.61</v>
+        <v>77.34</v>
       </c>
     </row>
     <row r="31">
@@ -10993,12 +11055,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="H31" s="3">
         <f>SUMIF($C$4:$C$110,G31,$E$4:$E$110)</f>
-        <v>69.36</v>
+        <v>73.61</v>
       </c>
     </row>
     <row r="32">
@@ -11025,12 +11087,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Software &amp; Online Subscriptions</t>
+          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
         </is>
       </c>
       <c r="H32" s="3">
         <f>SUMIF($C$4:$C$110,G32,$E$4:$E$110)</f>
-        <v>65.98</v>
+        <v>69.36</v>
       </c>
     </row>
     <row r="33">
@@ -11057,12 +11119,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Tractor Supply</t>
+          <t xml:space="preserve">Software &amp; Online Subscriptions</t>
         </is>
       </c>
       <c r="H33" s="3">
         <f>SUMIF($C$4:$C$110,G33,$E$4:$E$110)</f>
-        <v>29.86</v>
+        <v>65.98</v>
       </c>
     </row>
     <row r="34">
@@ -11089,12 +11151,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Frndly TV</t>
+          <t xml:space="preserve">Retail – Tractor Supply</t>
         </is>
       </c>
       <c r="H34" s="3">
         <f>SUMIF($C$4:$C$110,G34,$E$4:$E$110)</f>
-        <v>22.41</v>
+        <v>29.86</v>
       </c>
     </row>
     <row r="35">
@@ -11121,12 +11183,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
+          <t xml:space="preserve">Streaming – Frndly TV</t>
         </is>
       </c>
       <c r="H35" s="3">
         <f>SUMIF($C$4:$C$110,G35,$E$4:$E$110)</f>
-        <v>20.27</v>
+        <v>22.41</v>
       </c>
     </row>
     <row r="36">
@@ -11140,7 +11202,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -11153,12 +11215,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tolls &amp; Parking</t>
+          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
         </is>
       </c>
       <c r="H36" s="3">
         <f>SUMIF($C$4:$C$110,G36,$E$4:$E$110)</f>
-        <v>18.44</v>
+        <v>20.27</v>
       </c>
     </row>
     <row r="37">
@@ -11185,12 +11247,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+          <t xml:space="preserve">Tolls &amp; Parking</t>
         </is>
       </c>
       <c r="H37" s="3">
         <f>SUMIF($C$4:$C$110,G37,$E$4:$E$110)</f>
-        <v>17.35</v>
+        <v>18.44</v>
       </c>
     </row>
     <row r="38">
@@ -11217,12 +11279,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
         </is>
       </c>
       <c r="H38" s="3">
         <f>SUMIF($C$4:$C$110,G38,$E$4:$E$110)</f>
-        <v>13.87</v>
+        <v>17.35</v>
       </c>
     </row>
     <row r="39">
@@ -11249,12 +11311,12 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
         </is>
       </c>
       <c r="H39" s="3">
         <f>SUMIF($C$4:$C$110,G39,$E$4:$E$110)</f>
-        <v>13.5</v>
+        <v>13.87</v>
       </c>
     </row>
     <row r="40">
@@ -11281,12 +11343,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Hulu</t>
+          <t xml:space="preserve">Entertainment &amp; Events</t>
         </is>
       </c>
       <c r="H40" s="3">
         <f>SUMIF($C$4:$C$110,G40,$E$4:$E$110)</f>
-        <v>12.8</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="41">
@@ -11313,12 +11375,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Other Food Stores (Harris Teeter, Beach Pantry)</t>
+          <t xml:space="preserve">Streaming – Hulu</t>
         </is>
       </c>
       <c r="H41" s="3">
         <f>SUMIF($C$4:$C$110,G41,$E$4:$E$110)</f>
-        <v>5.85</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="42">
@@ -11343,14 +11405,14 @@
       <c r="E42" s="3">
         <v>115.0</v>
       </c>
-      <c r="G42" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total spending</t>
-        </is>
-      </c>
-      <c r="H42" s="9">
-        <f>SUM(H4:H41)</f>
-        <v>15086.64</v>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Other Food Stores (Harris Teeter, Beach Pantry)</t>
+        </is>
+      </c>
+      <c r="H42" s="3">
+        <f>SUMIF($C$4:$C$110,G42,$E$4:$E$110)</f>
+        <v>5.85</v>
       </c>
     </row>
     <row r="43">
@@ -11375,6 +11437,15 @@
       <c r="E43" s="3">
         <v>239.44</v>
       </c>
+      <c r="G43" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total spending</t>
+        </is>
+      </c>
+      <c r="H43" s="9">
+        <f>SUM(H4:H42)</f>
+        <v>15086.64</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4">
@@ -11398,12 +11469,6 @@
       <c r="E44" s="3">
         <v>9.47</v>
       </c>
-      <c r="G44" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not counted as spending</t>
-        </is>
-      </c>
-      <c r="H44" s="7"/>
     </row>
     <row r="45">
       <c r="A45" s="4">
@@ -11427,15 +11492,12 @@
       <c r="E45" s="3">
         <v>46.23</v>
       </c>
-      <c r="G45" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Checks Written (payee not shown)</t>
-        </is>
-      </c>
-      <c r="H45" s="3">
-        <f>SUMIF($C$4:$C$110,G45,$E$4:$E$110)</f>
-        <v>728.0</v>
-      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not counted as spending</t>
+        </is>
+      </c>
+      <c r="H45" s="7"/>
     </row>
     <row r="46">
       <c r="A46" s="4">
@@ -11461,12 +11523,12 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
+          <t xml:space="preserve">Checks Written (payee not shown)</t>
         </is>
       </c>
       <c r="H46" s="3">
         <f>SUMIF($C$4:$C$110,G46,$E$4:$E$110)</f>
-        <v>4593.08</v>
+        <v>728.0</v>
       </c>
     </row>
     <row r="47">
@@ -11493,12 +11555,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="H47" s="3">
         <f>SUMIF($C$4:$C$110,G47,$E$4:$E$110)</f>
-        <v>2576.0</v>
+        <v>4593.08</v>
       </c>
     </row>
     <row r="48">
@@ -11523,6 +11585,15 @@
       <c r="E48" s="3">
         <v>17.35</v>
       </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+        </is>
+      </c>
+      <c r="H48" s="3">
+        <f>SUMIF($C$4:$C$110,G48,$E$4:$E$110)</f>
+        <v>2576.0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4">
@@ -11719,7 +11790,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -12156,7 +12227,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -12230,7 +12301,7 @@
       </c>
       <c r="D79" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
       <c r="E79" s="3">
@@ -12616,7 +12687,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -13147,7 +13218,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -13480,7 +13551,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="H17" s="3">
@@ -14287,7 +14358,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -14577,7 +14648,7 @@
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
       <c r="E55" s="3">
@@ -17246,7 +17317,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
       <c r="F69" s="3">
@@ -18445,7 +18516,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -18501,7 +18572,7 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
@@ -19453,7 +19524,7 @@
       </c>
       <c r="D148" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="E148" s="2" t="inlineStr">
@@ -20489,7 +20560,7 @@
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="E185" s="2" t="inlineStr">
@@ -20802,7 +20873,7 @@
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
       <c r="F196" s="3">
@@ -21665,7 +21736,7 @@
       </c>
       <c r="D227" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="E227" s="2" t="inlineStr">
@@ -22533,7 +22604,7 @@
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
@@ -23065,7 +23136,7 @@
       </c>
       <c r="D277" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="E277" s="2" t="inlineStr">
@@ -23653,7 +23724,7 @@
       </c>
       <c r="D298" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="E298" s="2" t="inlineStr">
@@ -24185,7 +24256,7 @@
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="E317" s="2" t="inlineStr">
@@ -24274,7 +24345,7 @@
       </c>
       <c r="E320" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
       <c r="F320" s="3">
@@ -24745,7 +24816,7 @@
       </c>
       <c r="D337" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="E337" s="2" t="inlineStr">
@@ -25249,7 +25320,7 @@
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
@@ -26257,7 +26328,7 @@
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical &amp; Pharmacy</t>
+          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr">
@@ -26598,7 +26669,7 @@
       </c>
       <c r="E403" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Debt Payments</t>
+          <t xml:space="preserve">Student Loan</t>
         </is>
       </c>
       <c r="F403" s="3">

</xml_diff>

<commit_message>
Break out medical providers as separate line items
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -1022,7 +1022,7 @@
       </c>
       <c r="C42" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A42,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>935.1</v>
+        <v>909.94</v>
       </c>
       <c r="D42" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A42,'All Transactions'!$A$5:$A$436,D$4)</f>
@@ -1030,15 +1030,15 @@
       </c>
       <c r="E42" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A42,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>848.05</v>
+        <v>839.3</v>
       </c>
       <c r="F42" s="3">
         <f>SUM(B42:E42)</f>
-        <v>3765.22</v>
+        <v>3731.31</v>
       </c>
       <c r="G42" s="3">
         <f>F42/4</f>
-        <v>941.305</v>
+        <v>932.8275</v>
       </c>
     </row>
     <row r="43">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="C43" s="6">
         <f>SUM(C41:C42)</f>
-        <v>935.1</v>
+        <v>909.94</v>
       </c>
       <c r="D43" s="6">
         <f>SUM(D41:D42)</f>
@@ -1061,15 +1061,15 @@
       </c>
       <c r="E43" s="6">
         <f>SUM(E41:E42)</f>
-        <v>848.05</v>
+        <v>839.3</v>
       </c>
       <c r="F43" s="6">
         <f>SUM(F41:F42)</f>
-        <v>4034.42</v>
+        <v>4000.51</v>
       </c>
       <c r="G43" s="6">
         <f>F43/4</f>
-        <v>1008.605</v>
+        <v>1000.1275</v>
       </c>
     </row>
     <row r="45">
@@ -1130,15 +1130,15 @@
       </c>
       <c r="E47" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A47,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>74.24</v>
+        <v>68.24</v>
       </c>
       <c r="F47" s="3">
         <f>SUM(B47:E47)</f>
-        <v>98.52</v>
+        <v>92.52</v>
       </c>
       <c r="G47" s="3">
         <f>F47/4</f>
-        <v>24.63</v>
+        <v>23.13</v>
       </c>
     </row>
     <row r="48">
@@ -1161,15 +1161,15 @@
       </c>
       <c r="E48" s="6">
         <f>SUM(E46:E47)</f>
-        <v>313.22</v>
+        <v>307.22</v>
       </c>
       <c r="F48" s="6">
         <f>SUM(F46:F47)</f>
-        <v>891.51</v>
+        <v>885.51</v>
       </c>
       <c r="G48" s="6">
         <f>F48/4</f>
-        <v>222.8775</v>
+        <v>221.3775</v>
       </c>
     </row>
     <row r="50">
@@ -1568,7 +1568,7 @@
     <row r="67">
       <c r="A67" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="B67" s="3">
@@ -1585,296 +1585,296 @@
       </c>
       <c r="E67" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A67,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>160.28</v>
+        <v>100.28</v>
       </c>
       <c r="F67" s="3">
         <f>SUM(B67:E67)</f>
-        <v>627.94</v>
+        <v>567.94</v>
       </c>
       <c r="G67" s="3">
         <f>F67/4</f>
-        <v>156.985</v>
+        <v>141.985</v>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="7" t="inlineStr">
+      <c r="A68" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medical – Wilmington Eye</t>
+        </is>
+      </c>
+      <c r="B68" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A68,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C68" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A68,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D68" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A68,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E68" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A68,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>60.0</v>
+      </c>
+      <c r="F68" s="3">
+        <f>SUM(B68:E68)</f>
+        <v>60.0</v>
+      </c>
+      <c r="G68" s="3">
+        <f>F68/4</f>
+        <v>15.0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
+        </is>
+      </c>
+      <c r="B69" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A69,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C69" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A69,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>25.16</v>
+      </c>
+      <c r="D69" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A69,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E69" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A69,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F69" s="3">
+        <f>SUM(B69:E69)</f>
+        <v>25.16</v>
+      </c>
+      <c r="G69" s="3">
+        <f>F69/4</f>
+        <v>6.29</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medical – Duke Hospital (Durham, food &amp; parking)</t>
+        </is>
+      </c>
+      <c r="B70" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C70" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D70" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E70" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A70,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>14.75</v>
+      </c>
+      <c r="F70" s="3">
+        <f>SUM(B70:E70)</f>
+        <v>14.75</v>
+      </c>
+      <c r="G70" s="3">
+        <f>F70/4</f>
+        <v>3.6875</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Health</t>
         </is>
       </c>
-      <c r="B68" s="6">
-        <f>SUM(B66:B67)</f>
+      <c r="B71" s="6">
+        <f>SUM(B66:B70)</f>
         <v>160.07</v>
       </c>
-      <c r="C68" s="6">
-        <f>SUM(C66:C67)</f>
-        <v>100.93</v>
-      </c>
-      <c r="D68" s="6">
-        <f>SUM(D66:D67)</f>
+      <c r="C71" s="6">
+        <f>SUM(C66:C70)</f>
+        <v>126.09</v>
+      </c>
+      <c r="D71" s="6">
+        <f>SUM(D66:D70)</f>
         <v>850.9</v>
       </c>
-      <c r="E68" s="6">
-        <f>SUM(E66:E67)</f>
-        <v>160.28</v>
-      </c>
-      <c r="F68" s="6">
-        <f>SUM(F66:F67)</f>
-        <v>1272.18</v>
-      </c>
-      <c r="G68" s="6">
-        <f>F68/4</f>
-        <v>318.045</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="5" t="inlineStr">
+      <c r="E71" s="6">
+        <f>SUM(E66:E70)</f>
+        <v>175.03</v>
+      </c>
+      <c r="F71" s="6">
+        <f>SUM(F66:F70)</f>
+        <v>1312.09</v>
+      </c>
+      <c r="G71" s="6">
+        <f>F71/4</f>
+        <v>328.0225</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Personal</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="12" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
-      <c r="B71" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B74" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>182.5</v>
       </c>
-      <c r="C71" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C74" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D71" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D74" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>182.5</v>
       </c>
-      <c r="E71" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A71,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E74" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A74,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>32.5</v>
       </c>
-      <c r="F71" s="3">
-        <f>SUM(B71:E71)</f>
+      <c r="F74" s="3">
+        <f>SUM(B74:E74)</f>
         <v>397.5</v>
       </c>
-      <c r="G71" s="3">
-        <f>F71/4</f>
+      <c r="G74" s="3">
+        <f>F74/4</f>
         <v>99.375</v>
       </c>
     </row>
-    <row r="72">
-      <c r="A72" s="12" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Personal Care – Simple Beauty</t>
         </is>
       </c>
-      <c r="B72" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B75" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C72" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C75" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D72" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D75" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E72" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A72,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E75" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A75,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>82.0</v>
       </c>
-      <c r="F72" s="3">
-        <f>SUM(B72:E72)</f>
+      <c r="F75" s="3">
+        <f>SUM(B75:E75)</f>
         <v>82.0</v>
       </c>
-      <c r="G72" s="3">
-        <f>F72/4</f>
+      <c r="G75" s="3">
+        <f>F75/4</f>
         <v>20.5</v>
       </c>
     </row>
-    <row r="73">
-      <c r="A73" s="7" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Personal</t>
         </is>
       </c>
-      <c r="B73" s="6">
-        <f>SUM(B71:B72)</f>
+      <c r="B76" s="6">
+        <f>SUM(B74:B75)</f>
         <v>182.5</v>
       </c>
-      <c r="C73" s="6">
-        <f>SUM(C71:C72)</f>
+      <c r="C76" s="6">
+        <f>SUM(C74:C75)</f>
         <v>0</v>
       </c>
-      <c r="D73" s="6">
-        <f>SUM(D71:D72)</f>
+      <c r="D76" s="6">
+        <f>SUM(D74:D75)</f>
         <v>182.5</v>
       </c>
-      <c r="E73" s="6">
-        <f>SUM(E71:E72)</f>
+      <c r="E76" s="6">
+        <f>SUM(E74:E75)</f>
         <v>114.5</v>
       </c>
-      <c r="F73" s="6">
-        <f>SUM(F71:F72)</f>
+      <c r="F76" s="6">
+        <f>SUM(F74:F75)</f>
         <v>479.5</v>
       </c>
-      <c r="G73" s="6">
-        <f>F73/4</f>
+      <c r="G76" s="6">
+        <f>F76/4</f>
         <v>119.875</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="5" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Retail</t>
         </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Walmart</t>
-        </is>
-      </c>
-      <c r="B76" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C76" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>132.66</v>
-      </c>
-      <c r="D76" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1732.6</v>
-      </c>
-      <c r="E76" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A76,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.63</v>
-      </c>
-      <c r="F76" s="3">
-        <f>SUM(B76:E76)</f>
-        <v>1897.89</v>
-      </c>
-      <c r="G76" s="3">
-        <f>F76/4</f>
-        <v>474.4725</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Belk (store card payments)</t>
-        </is>
-      </c>
-      <c r="B77" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>386.69</v>
-      </c>
-      <c r="C77" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>948.04</v>
-      </c>
-      <c r="D77" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E77" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A77,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F77" s="3">
-        <f>SUM(B77:E77)</f>
-        <v>1334.73</v>
-      </c>
-      <c r="G77" s="3">
-        <f>F77/4</f>
-        <v>333.6825</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Marshalls</t>
-        </is>
-      </c>
-      <c r="B78" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C78" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D78" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E78" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A78,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>41.59</v>
-      </c>
-      <c r="F78" s="3">
-        <f>SUM(B78:E78)</f>
-        <v>41.59</v>
-      </c>
-      <c r="G78" s="3">
-        <f>F78/4</f>
-        <v>10.3975</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ross</t>
+          <t xml:space="preserve">Retail – Walmart</t>
         </is>
       </c>
       <c r="B79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>48.03</v>
+        <v>0</v>
       </c>
       <c r="C79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>132.66</v>
       </c>
       <c r="D79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1732.6</v>
       </c>
       <c r="E79" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A79,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>16.32</v>
+        <v>32.63</v>
       </c>
       <c r="F79" s="3">
         <f>SUM(B79:E79)</f>
-        <v>64.35</v>
+        <v>1897.89</v>
       </c>
       <c r="G79" s="3">
         <f>F79/4</f>
-        <v>16.0875</v>
+        <v>474.4725</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dillard's</t>
+          <t xml:space="preserve">Retail – Belk (store card payments)</t>
         </is>
       </c>
       <c r="B80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>386.69</v>
       </c>
       <c r="C80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>948.04</v>
       </c>
       <c r="D80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>174.74</v>
+        <v>0</v>
       </c>
       <c r="E80" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A80,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -1882,22 +1882,22 @@
       </c>
       <c r="F80" s="3">
         <f>SUM(B80:E80)</f>
-        <v>174.74</v>
+        <v>1334.73</v>
       </c>
       <c r="G80" s="3">
         <f>F80/4</f>
-        <v>43.685</v>
+        <v>333.6825</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Target</t>
+          <t xml:space="preserve">Retail – Marshalls</t>
         </is>
       </c>
       <c r="B81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>58.98</v>
+        <v>0</v>
       </c>
       <c r="C81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1909,26 +1909,26 @@
       </c>
       <c r="E81" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A81,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>41.59</v>
       </c>
       <c r="F81" s="3">
         <f>SUM(B81:E81)</f>
-        <v>58.98</v>
+        <v>41.59</v>
       </c>
       <c r="G81" s="3">
         <f>F81/4</f>
-        <v>14.745</v>
+        <v>10.3975</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – HomeSense</t>
+          <t xml:space="preserve">Retail – Ross</t>
         </is>
       </c>
       <c r="B82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>48.03</v>
       </c>
       <c r="C82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1936,25 +1936,25 @@
       </c>
       <c r="D82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>88.7</v>
+        <v>0</v>
       </c>
       <c r="E82" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A82,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>16.32</v>
       </c>
       <c r="F82" s="3">
         <f>SUM(B82:E82)</f>
-        <v>88.7</v>
+        <v>64.35</v>
       </c>
       <c r="G82" s="3">
         <f>F82/4</f>
-        <v>22.175</v>
+        <v>16.0875</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Hobby Lobby</t>
+          <t xml:space="preserve">Retail – Dillard's</t>
         </is>
       </c>
       <c r="B83" s="3">
@@ -1967,30 +1967,30 @@
       </c>
       <c r="D83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>165.67</v>
+        <v>174.74</v>
       </c>
       <c r="E83" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A83,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>37.33</v>
+        <v>0</v>
       </c>
       <c r="F83" s="3">
         <f>SUM(B83:E83)</f>
-        <v>203.0</v>
+        <v>174.74</v>
       </c>
       <c r="G83" s="3">
         <f>F83/4</f>
-        <v>50.75</v>
+        <v>43.685</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
+          <t xml:space="preserve">Retail – Target</t>
         </is>
       </c>
       <c r="B84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>27.67</v>
+        <v>58.98</v>
       </c>
       <c r="C84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -1998,25 +1998,25 @@
       </c>
       <c r="D84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>171.55</v>
+        <v>0</v>
       </c>
       <c r="E84" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A84,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>85.27</v>
+        <v>0</v>
       </c>
       <c r="F84" s="3">
         <f>SUM(B84:E84)</f>
-        <v>284.49</v>
+        <v>58.98</v>
       </c>
       <c r="G84" s="3">
         <f>F84/4</f>
-        <v>71.1225</v>
+        <v>14.745</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Cat on a Whisk</t>
+          <t xml:space="preserve">Retail – HomeSense</t>
         </is>
       </c>
       <c r="B85" s="3">
@@ -2029,25 +2029,25 @@
       </c>
       <c r="D85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>88.7</v>
       </c>
       <c r="E85" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A85,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>24.51</v>
+        <v>0</v>
       </c>
       <c r="F85" s="3">
         <f>SUM(B85:E85)</f>
-        <v>24.51</v>
+        <v>88.7</v>
       </c>
       <c r="G85" s="3">
         <f>F85/4</f>
-        <v>6.1275</v>
+        <v>22.175</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Tractor Supply</t>
+          <t xml:space="preserve">Retail – Hobby Lobby</t>
         </is>
       </c>
       <c r="B86" s="3">
@@ -2060,61 +2060,61 @@
       </c>
       <c r="D86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>29.86</v>
+        <v>165.67</v>
       </c>
       <c r="E86" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A86,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>37.33</v>
       </c>
       <c r="F86" s="3">
         <f>SUM(B86:E86)</f>
-        <v>29.86</v>
+        <v>203.0</v>
       </c>
       <c r="G86" s="3">
         <f>F86/4</f>
-        <v>7.465</v>
+        <v>50.75</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
+          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
         </is>
       </c>
       <c r="B87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>27.67</v>
       </c>
       <c r="C87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>63.61</v>
+        <v>0</v>
       </c>
       <c r="D87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>171.55</v>
       </c>
       <c r="E87" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A87,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>85.27</v>
       </c>
       <c r="F87" s="3">
         <f>SUM(B87:E87)</f>
-        <v>63.61</v>
+        <v>284.49</v>
       </c>
       <c r="G87" s="3">
         <f>F87/4</f>
-        <v>15.9025</v>
+        <v>71.1225</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ulta Beauty</t>
+          <t xml:space="preserve">Retail – Cat on a Whisk</t>
         </is>
       </c>
       <c r="B88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>134.71</v>
+        <v>0</v>
       </c>
       <c r="C88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -2126,26 +2126,26 @@
       </c>
       <c r="E88" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A88,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>24.51</v>
       </c>
       <c r="F88" s="3">
         <f>SUM(B88:E88)</f>
-        <v>134.71</v>
+        <v>24.51</v>
       </c>
       <c r="G88" s="3">
         <f>F88/4</f>
-        <v>33.6775</v>
+        <v>6.1275</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
+          <t xml:space="preserve">Retail – Tractor Supply</t>
         </is>
       </c>
       <c r="B89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>51.31</v>
+        <v>0</v>
       </c>
       <c r="C89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -2153,7 +2153,7 @@
       </c>
       <c r="D89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>29.86</v>
       </c>
       <c r="E89" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A89,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2161,17 +2161,17 @@
       </c>
       <c r="F89" s="3">
         <f>SUM(B89:E89)</f>
-        <v>51.31</v>
+        <v>29.86</v>
       </c>
       <c r="G89" s="3">
         <f>F89/4</f>
-        <v>12.8275</v>
+        <v>7.465</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
         </is>
       </c>
       <c r="B90" s="3">
@@ -2180,11 +2180,11 @@
       </c>
       <c r="C90" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>5.87</v>
+        <v>63.61</v>
       </c>
       <c r="D90" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>17.35</v>
+        <v>0</v>
       </c>
       <c r="E90" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A90,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2192,22 +2192,22 @@
       </c>
       <c r="F90" s="3">
         <f>SUM(B90:E90)</f>
-        <v>23.22</v>
+        <v>63.61</v>
       </c>
       <c r="G90" s="3">
         <f>F90/4</f>
-        <v>5.805</v>
+        <v>15.9025</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+          <t xml:space="preserve">Retail – Ulta Beauty</t>
         </is>
       </c>
       <c r="B91" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.03</v>
+        <v>134.71</v>
       </c>
       <c r="C91" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,C$4)</f>
@@ -2219,652 +2219,652 @@
       </c>
       <c r="E91" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A91,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>119.97</v>
+        <v>0</v>
       </c>
       <c r="F91" s="3">
         <f>SUM(B91:E91)</f>
-        <v>228.0</v>
+        <v>134.71</v>
       </c>
       <c r="G91" s="3">
         <f>F91/4</f>
+        <v>33.6775</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Bath &amp; Body Works</t>
+        </is>
+      </c>
+      <c r="B92" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>51.31</v>
+      </c>
+      <c r="C92" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D92" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E92" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A92,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F92" s="3">
+        <f>SUM(B92:E92)</f>
+        <v>51.31</v>
+      </c>
+      <c r="G92" s="3">
+        <f>F92/4</f>
+        <v>12.8275</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+        </is>
+      </c>
+      <c r="B93" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C93" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>5.87</v>
+      </c>
+      <c r="D93" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>17.35</v>
+      </c>
+      <c r="E93" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A93,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F93" s="3">
+        <f>SUM(B93:E93)</f>
+        <v>23.22</v>
+      </c>
+      <c r="G93" s="3">
+        <f>F93/4</f>
+        <v>5.805</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+        </is>
+      </c>
+      <c r="B94" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.03</v>
+      </c>
+      <c r="C94" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D94" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E94" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A94,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>119.97</v>
+      </c>
+      <c r="F94" s="3">
+        <f>SUM(B94:E94)</f>
+        <v>228.0</v>
+      </c>
+      <c r="G94" s="3">
+        <f>F94/4</f>
         <v>57.0</v>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="7" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Retail</t>
         </is>
       </c>
-      <c r="B92" s="6">
-        <f>SUM(B76:B91)</f>
+      <c r="B95" s="6">
+        <f>SUM(B79:B94)</f>
         <v>815.42</v>
       </c>
-      <c r="C92" s="6">
-        <f>SUM(C76:C91)</f>
+      <c r="C95" s="6">
+        <f>SUM(C79:C94)</f>
         <v>1150.18</v>
       </c>
-      <c r="D92" s="6">
-        <f>SUM(D76:D91)</f>
+      <c r="D95" s="6">
+        <f>SUM(D79:D94)</f>
         <v>2380.47</v>
       </c>
-      <c r="E92" s="6">
-        <f>SUM(E76:E91)</f>
+      <c r="E95" s="6">
+        <f>SUM(E79:E94)</f>
         <v>357.62</v>
       </c>
-      <c r="F92" s="6">
-        <f>SUM(F76:F91)</f>
+      <c r="F95" s="6">
+        <f>SUM(F79:F94)</f>
         <v>4703.69</v>
       </c>
-      <c r="G92" s="6">
-        <f>F92/4</f>
+      <c r="G95" s="6">
+        <f>F95/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="5" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Home</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="12" t="inlineStr">
+    <row r="98">
+      <c r="A98" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
-      <c r="B95" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B98" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>60.0</v>
       </c>
-      <c r="C95" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C98" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>100.0</v>
       </c>
-      <c r="D95" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D98" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>220.0</v>
       </c>
-      <c r="E95" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A95,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E98" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A98,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>120.0</v>
       </c>
-      <c r="F95" s="3">
-        <f>SUM(B95:E95)</f>
+      <c r="F98" s="3">
+        <f>SUM(B98:E98)</f>
         <v>500.0</v>
       </c>
-      <c r="G95" s="3">
-        <f>F95/4</f>
+      <c r="G98" s="3">
+        <f>F98/4</f>
         <v>125.0</v>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="12" t="inlineStr">
+    <row r="99">
+      <c r="A99" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
         </is>
       </c>
-      <c r="B96" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B99" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C96" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C99" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>242.05</v>
       </c>
-      <c r="D96" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D99" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>536.6</v>
       </c>
-      <c r="E96" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A96,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E99" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F96" s="3">
-        <f>SUM(B96:E96)</f>
+      <c r="F99" s="3">
+        <f>SUM(B99:E99)</f>
         <v>778.65</v>
       </c>
-      <c r="G96" s="3">
-        <f>F96/4</f>
+      <c r="G99" s="3">
+        <f>F99/4</f>
         <v>194.6625</v>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" s="7" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Home</t>
         </is>
       </c>
-      <c r="B97" s="6">
-        <f>SUM(B95:B96)</f>
+      <c r="B100" s="6">
+        <f>SUM(B98:B99)</f>
         <v>60.0</v>
       </c>
-      <c r="C97" s="6">
-        <f>SUM(C95:C96)</f>
+      <c r="C100" s="6">
+        <f>SUM(C98:C99)</f>
         <v>342.05</v>
       </c>
-      <c r="D97" s="6">
-        <f>SUM(D95:D96)</f>
+      <c r="D100" s="6">
+        <f>SUM(D98:D99)</f>
         <v>756.6</v>
       </c>
-      <c r="E97" s="6">
-        <f>SUM(E95:E96)</f>
+      <c r="E100" s="6">
+        <f>SUM(E98:E99)</f>
         <v>120.0</v>
       </c>
-      <c r="F97" s="6">
-        <f>SUM(F95:F96)</f>
+      <c r="F100" s="6">
+        <f>SUM(F98:F99)</f>
         <v>1278.65</v>
       </c>
-      <c r="G97" s="6">
-        <f>F97/4</f>
+      <c r="G100" s="6">
+        <f>F100/4</f>
         <v>319.6625</v>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="5" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="12" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Travel (Lyft, Hotel)</t>
         </is>
       </c>
-      <c r="B100" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B103" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>102.65</v>
       </c>
-      <c r="C100" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C103" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D100" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D103" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E100" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A100,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E103" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A103,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F100" s="3">
-        <f>SUM(B100:E100)</f>
+      <c r="F103" s="3">
+        <f>SUM(B103:E103)</f>
         <v>102.65</v>
       </c>
-      <c r="G100" s="3">
-        <f>F100/4</f>
+      <c r="G103" s="3">
+        <f>F103/4</f>
         <v>25.6625</v>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="7" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Travel</t>
         </is>
       </c>
-      <c r="B101" s="6">
-        <f>SUM(B100:B100)</f>
+      <c r="B104" s="6">
+        <f>SUM(B103:B103)</f>
         <v>102.65</v>
       </c>
-      <c r="C101" s="6">
-        <f>SUM(C100:C100)</f>
+      <c r="C104" s="6">
+        <f>SUM(C103:C103)</f>
         <v>0</v>
       </c>
-      <c r="D101" s="6">
-        <f>SUM(D100:D100)</f>
+      <c r="D104" s="6">
+        <f>SUM(D103:D103)</f>
         <v>0</v>
       </c>
-      <c r="E101" s="6">
-        <f>SUM(E100:E100)</f>
+      <c r="E104" s="6">
+        <f>SUM(E103:E103)</f>
         <v>0</v>
       </c>
-      <c r="F101" s="6">
-        <f>SUM(F100:F100)</f>
+      <c r="F104" s="6">
+        <f>SUM(F103:F103)</f>
         <v>102.65</v>
       </c>
-      <c r="G101" s="6">
-        <f>F101/4</f>
+      <c r="G104" s="6">
+        <f>F104/4</f>
         <v>25.6625</v>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="5" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Recreation</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="12" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">St. James Marina</t>
         </is>
       </c>
-      <c r="B104" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B107" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C104" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C107" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>33.54</v>
       </c>
-      <c r="D104" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D107" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E104" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A104,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E107" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A107,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F104" s="3">
-        <f>SUM(B104:E104)</f>
+      <c r="F107" s="3">
+        <f>SUM(B107:E107)</f>
         <v>33.54</v>
       </c>
-      <c r="G104" s="3">
-        <f>F104/4</f>
+      <c r="G107" s="3">
+        <f>F107/4</f>
         <v>8.385</v>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="12" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Entertainment &amp; Events</t>
         </is>
       </c>
-      <c r="B105" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B108" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C105" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C108" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>400.0</v>
       </c>
-      <c r="D105" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D108" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>13.5</v>
       </c>
-      <c r="E105" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A105,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E108" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>0</v>
       </c>
-      <c r="F105" s="3">
-        <f>SUM(B105:E105)</f>
+      <c r="F108" s="3">
+        <f>SUM(B108:E108)</f>
         <v>413.5</v>
       </c>
-      <c r="G105" s="3">
-        <f>F105/4</f>
+      <c r="G108" s="3">
+        <f>F108/4</f>
         <v>103.375</v>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="7" t="inlineStr">
+    <row r="109">
+      <c r="A109" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Recreation</t>
         </is>
       </c>
-      <c r="B106" s="6">
-        <f>SUM(B104:B105)</f>
+      <c r="B109" s="6">
+        <f>SUM(B107:B108)</f>
         <v>0</v>
       </c>
-      <c r="C106" s="6">
-        <f>SUM(C104:C105)</f>
+      <c r="C109" s="6">
+        <f>SUM(C107:C108)</f>
         <v>433.54</v>
       </c>
-      <c r="D106" s="6">
-        <f>SUM(D104:D105)</f>
+      <c r="D109" s="6">
+        <f>SUM(D107:D108)</f>
         <v>13.5</v>
       </c>
-      <c r="E106" s="6">
-        <f>SUM(E104:E105)</f>
+      <c r="E109" s="6">
+        <f>SUM(E107:E108)</f>
         <v>0</v>
       </c>
-      <c r="F106" s="6">
-        <f>SUM(F104:F105)</f>
+      <c r="F109" s="6">
+        <f>SUM(F107:F108)</f>
         <v>447.04</v>
       </c>
-      <c r="G106" s="6">
-        <f>F106/4</f>
+      <c r="G109" s="6">
+        <f>F109/4</f>
         <v>111.76</v>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="5" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="12" t="inlineStr">
+    <row r="112">
+      <c r="A112" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
         </is>
       </c>
-      <c r="B109" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B112" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>75.0</v>
       </c>
-      <c r="C109" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C112" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>764.05</v>
       </c>
-      <c r="D109" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D112" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>331.5</v>
       </c>
-      <c r="E109" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A109,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E112" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A112,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>130.0</v>
       </c>
-      <c r="F109" s="3">
-        <f>SUM(B109:E109)</f>
+      <c r="F112" s="3">
+        <f>SUM(B112:E112)</f>
         <v>1300.55</v>
       </c>
-      <c r="G109" s="3">
-        <f>F109/4</f>
+      <c r="G112" s="3">
+        <f>F112/4</f>
         <v>325.1375</v>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" s="7" t="inlineStr">
+    <row r="113">
+      <c r="A113" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Transfers</t>
         </is>
       </c>
-      <c r="B110" s="6">
-        <f>SUM(B109:B109)</f>
+      <c r="B113" s="6">
+        <f>SUM(B112:B112)</f>
         <v>75.0</v>
       </c>
-      <c r="C110" s="6">
-        <f>SUM(C109:C109)</f>
+      <c r="C113" s="6">
+        <f>SUM(C112:C112)</f>
         <v>764.05</v>
       </c>
-      <c r="D110" s="6">
-        <f>SUM(D109:D109)</f>
+      <c r="D113" s="6">
+        <f>SUM(D112:D112)</f>
         <v>331.5</v>
       </c>
-      <c r="E110" s="6">
-        <f>SUM(E109:E109)</f>
+      <c r="E113" s="6">
+        <f>SUM(E112:E112)</f>
         <v>130.0</v>
       </c>
-      <c r="F110" s="6">
-        <f>SUM(F109:F109)</f>
+      <c r="F113" s="6">
+        <f>SUM(F112:F112)</f>
         <v>1300.55</v>
       </c>
-      <c r="G110" s="6">
-        <f>F110/4</f>
+      <c r="G113" s="6">
+        <f>F113/4</f>
         <v>325.1375</v>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="5" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Other</t>
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" s="12" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Donations &amp; Clubs (Kiwanis)</t>
         </is>
       </c>
-      <c r="B113" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B116" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A116,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C113" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C116" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A116,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D113" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D116" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A116,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E113" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A113,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E116" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A116,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>200.0</v>
       </c>
-      <c r="F113" s="3">
-        <f>SUM(B113:E113)</f>
+      <c r="F116" s="3">
+        <f>SUM(B116:E116)</f>
         <v>200.0</v>
       </c>
-      <c r="G113" s="3">
-        <f>F113/4</f>
+      <c r="G116" s="3">
+        <f>F116/4</f>
         <v>50.0</v>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" s="12" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
         </is>
       </c>
-      <c r="B114" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B117" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A117,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>0</v>
       </c>
-      <c r="C114" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C117" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A117,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D114" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D117" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A117,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>0</v>
       </c>
-      <c r="E114" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A114,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E117" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A117,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>147.0</v>
       </c>
-      <c r="F114" s="3">
-        <f>SUM(B114:E114)</f>
+      <c r="F117" s="3">
+        <f>SUM(B117:E117)</f>
         <v>147.0</v>
       </c>
-      <c r="G114" s="3">
-        <f>F114/4</f>
+      <c r="G117" s="3">
+        <f>F117/4</f>
         <v>36.75</v>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="7" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total Other</t>
         </is>
       </c>
-      <c r="B115" s="6">
-        <f>SUM(B113:B114)</f>
+      <c r="B118" s="6">
+        <f>SUM(B116:B117)</f>
         <v>0</v>
       </c>
-      <c r="C115" s="6">
-        <f>SUM(C113:C114)</f>
+      <c r="C118" s="6">
+        <f>SUM(C116:C117)</f>
         <v>0</v>
       </c>
-      <c r="D115" s="6">
-        <f>SUM(D113:D114)</f>
+      <c r="D118" s="6">
+        <f>SUM(D116:D117)</f>
         <v>0</v>
       </c>
-      <c r="E115" s="6">
-        <f>SUM(E113:E114)</f>
+      <c r="E118" s="6">
+        <f>SUM(E116:E117)</f>
         <v>347.0</v>
       </c>
-      <c r="F115" s="6">
-        <f>SUM(F113:F114)</f>
+      <c r="F118" s="6">
+        <f>SUM(F116:F117)</f>
         <v>347.0</v>
       </c>
-      <c r="G115" s="6">
-        <f>F115/4</f>
+      <c r="G118" s="6">
+        <f>F118/4</f>
         <v>86.75</v>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="8" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">TOTAL SPENDING</t>
         </is>
       </c>
-      <c r="B117" s="9">
-        <f>B10+B18+B23+B28+B32+B38+B43+B48+B59+B63+B68+B73+B92+B97+B101+B106+B110+B115</f>
+      <c r="B120" s="9">
+        <f>B10+B18+B23+B28+B32+B38+B43+B48+B59+B63+B71+B76+B95+B100+B104+B109+B113+B118</f>
         <v>12135.81</v>
       </c>
-      <c r="C117" s="9">
-        <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C68+C73+C92+C97+C101+C106+C110+C115</f>
+      <c r="C120" s="9">
+        <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C71+C76+C95+C100+C104+C109+C113+C118</f>
         <v>12663.24</v>
       </c>
-      <c r="D117" s="9">
-        <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D68+D73+D92+D97+D101+D106+D110+D115</f>
+      <c r="D120" s="9">
+        <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D71+D76+D95+D100+D104+D109+D113+D118</f>
         <v>15086.64</v>
       </c>
-      <c r="E117" s="9">
-        <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E68+E73+E92+E97+E101+E106+E110+E115</f>
+      <c r="E120" s="9">
+        <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E71+E76+E95+E100+E104+E109+E113+E118</f>
         <v>11515.63</v>
       </c>
-      <c r="F117" s="9">
-        <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F68+F73+F92+F97+F101+F106+F110+F115</f>
+      <c r="F120" s="9">
+        <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F71+F76+F95+F100+F104+F109+F113+F118</f>
         <v>51401.32</v>
       </c>
-      <c r="G117" s="9">
-        <f>F117/4</f>
+      <c r="G120" s="9">
+        <f>F120/4</f>
         <v>12850.33</v>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="5" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Not counted as spending</t>
         </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
-        </is>
-      </c>
-      <c r="B120" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="C120" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="D120" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="E120" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A120,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>2576.0</v>
-      </c>
-      <c r="F120" s="3">
-        <f>SUM(B120:E120)</f>
-        <v>10304.0</v>
-      </c>
-      <c r="G120" s="3">
-        <f>F120/4</f>
-        <v>2576.0</v>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
-        </is>
-      </c>
-      <c r="B121" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C121" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>7227.09</v>
-      </c>
-      <c r="D121" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>4593.08</v>
-      </c>
-      <c r="E121" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A121,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>4738.51</v>
-      </c>
-      <c r="F121" s="3">
-        <f>SUM(B121:E121)</f>
-        <v>16558.68</v>
-      </c>
-      <c r="G121" s="3">
-        <f>F121/4</f>
-        <v>4139.67</v>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Sloane Realty</t>
-        </is>
-      </c>
-      <c r="B122" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
-      </c>
-      <c r="C122" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>2891.98</v>
-      </c>
-      <c r="D122" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E122" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A122,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F122" s="3">
-        <f>SUM(B122:E122)</f>
-        <v>2891.98</v>
-      </c>
-      <c r="G122" s="3">
-        <f>F122/4</f>
-        <v>722.995</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checks Written (payee not shown)</t>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
         </is>
       </c>
       <c r="B123" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2630.0</v>
+        <v>2576.0</v>
       </c>
       <c r="C123" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>2576.0</v>
       </c>
       <c r="D123" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>728.0</v>
+        <v>2576.0</v>
       </c>
       <c r="E123" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A123,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>2576.0</v>
       </c>
       <c r="F123" s="3">
         <f>SUM(B123:E123)</f>
-        <v>3358.0</v>
+        <v>10304.0</v>
       </c>
       <c r="G123" s="3">
         <f>F123/4</f>
-        <v>839.5</v>
+        <v>2576.0</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="B124" s="3">
@@ -2873,831 +2873,924 @@
       </c>
       <c r="C124" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3.26</v>
+        <v>7227.09</v>
       </c>
       <c r="D124" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>4593.08</v>
       </c>
       <c r="E124" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A124,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>4738.51</v>
       </c>
       <c r="F124" s="3">
         <f>SUM(B124:E124)</f>
-        <v>3.26</v>
+        <v>16558.68</v>
       </c>
       <c r="G124" s="3">
         <f>F124/4</f>
-        <v>0.815</v>
+        <v>4139.67</v>
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total not counted as spending</t>
-        </is>
-      </c>
-      <c r="B125" s="6">
-        <f>SUM(B120:B124)</f>
-        <v>5206.0</v>
-      </c>
-      <c r="C125" s="6">
-        <f>SUM(C120:C124)</f>
-        <v>12698.33</v>
-      </c>
-      <c r="D125" s="6">
-        <f>SUM(D120:D124)</f>
-        <v>7897.08</v>
-      </c>
-      <c r="E125" s="6">
-        <f>SUM(E120:E124)</f>
-        <v>7314.51</v>
-      </c>
-      <c r="F125" s="6">
-        <f>SUM(F120:F124)</f>
-        <v>33115.92</v>
-      </c>
-      <c r="G125" s="6">
+      <c r="A125" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sloane Realty</t>
+        </is>
+      </c>
+      <c r="B125" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A125,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C125" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A125,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>2891.98</v>
+      </c>
+      <c r="D125" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A125,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E125" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A125,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F125" s="3">
+        <f>SUM(B125:E125)</f>
+        <v>2891.98</v>
+      </c>
+      <c r="G125" s="3">
         <f>F125/4</f>
-        <v>8278.98</v>
+        <v>722.995</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Checks Written (payee not shown)</t>
+        </is>
+      </c>
+      <c r="B126" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>2630.0</v>
+      </c>
+      <c r="C126" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D126" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>728.0</v>
+      </c>
+      <c r="E126" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F126" s="3">
+        <f>SUM(B126:E126)</f>
+        <v>3358.0</v>
+      </c>
+      <c r="G126" s="3">
+        <f>F126/4</f>
+        <v>839.5</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
+        </is>
+      </c>
+      <c r="B127" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C127" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>3.26</v>
+      </c>
+      <c r="D127" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E127" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F127" s="3">
+        <f>SUM(B127:E127)</f>
+        <v>3.26</v>
+      </c>
+      <c r="G127" s="3">
+        <f>F127/4</f>
+        <v>0.815</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total not counted as spending</t>
+        </is>
+      </c>
+      <c r="B128" s="6">
+        <f>SUM(B123:B127)</f>
+        <v>5206.0</v>
+      </c>
+      <c r="C128" s="6">
+        <f>SUM(C123:C127)</f>
+        <v>12698.33</v>
+      </c>
+      <c r="D128" s="6">
+        <f>SUM(D123:D127)</f>
+        <v>7897.08</v>
+      </c>
+      <c r="E128" s="6">
+        <f>SUM(E123:E127)</f>
+        <v>7314.51</v>
+      </c>
+      <c r="F128" s="6">
+        <f>SUM(F123:F127)</f>
+        <v>33115.92</v>
+      </c>
+      <c r="G128" s="6">
+        <f>F128/4</f>
+        <v>8278.98</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Check: spending + not-counted items</t>
         </is>
       </c>
-      <c r="B127" s="3">
-        <f>B117+B125</f>
+      <c r="B130" s="3">
+        <f>B120+B128</f>
         <v>17341.81</v>
       </c>
-      <c r="C127" s="3">
-        <f>C117+C125</f>
+      <c r="C130" s="3">
+        <f>C120+C128</f>
         <v>25361.57</v>
       </c>
-      <c r="D127" s="3">
-        <f>D117+D125</f>
+      <c r="D130" s="3">
+        <f>D120+D128</f>
         <v>22983.72</v>
       </c>
-      <c r="E127" s="3">
-        <f>E117+E125</f>
+      <c r="E130" s="3">
+        <f>E120+E128</f>
         <v>18830.14</v>
       </c>
-      <c r="F127" s="3">
-        <f>F117+F125</f>
+      <c r="F130" s="3">
+        <f>F120+F128</f>
         <v>84517.24</v>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="12" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
         </is>
       </c>
-      <c r="B128" s="13">
+      <c r="B131" s="13">
         <v>17341.81</v>
       </c>
-      <c r="C128" s="13">
+      <c r="C131" s="13">
         <v>25361.57</v>
       </c>
-      <c r="D128" s="13">
+      <c r="D131" s="13">
         <v>22983.72</v>
       </c>
-      <c r="E128" s="13">
+      <c r="E131" s="13">
         <v>18830.14</v>
       </c>
-      <c r="F128" s="3">
-        <f>SUM(B128:E128)</f>
+      <c r="F131" s="3">
+        <f>SUM(B131:E131)</f>
         <v>84517.24</v>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="12" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Difference (should be $0 = every dollar accounted for)</t>
         </is>
       </c>
-      <c r="B129" s="3">
-        <f>B127-B128</f>
+      <c r="B132" s="3">
+        <f>B130-B131</f>
         <v>0.0</v>
       </c>
-      <c r="C129" s="3">
-        <f>C127-C128</f>
+      <c r="C132" s="3">
+        <f>C130-C131</f>
         <v>0.0</v>
       </c>
-      <c r="D129" s="3">
-        <f>D127-D128</f>
+      <c r="D132" s="3">
+        <f>D130-D131</f>
         <v>0.0</v>
       </c>
-      <c r="E129" s="3">
-        <f>E127-E128</f>
+      <c r="E132" s="3">
+        <f>E130-E131</f>
         <v>0.0</v>
       </c>
-      <c r="F129" s="3">
-        <f>F127-F128</f>
+      <c r="F132" s="3">
+        <f>F130-F131</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="5" t="inlineStr">
+    <row r="134">
+      <c r="A134" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Key Bills at a Glance</t>
         </is>
       </c>
     </row>
-    <row r="132">
-      <c r="A132" s="15" t="inlineStr">
+    <row r="135">
+      <c r="A135" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Bill</t>
         </is>
       </c>
-      <c r="B132" s="1" t="inlineStr">
+      <c r="B135" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">June 2026</t>
         </is>
       </c>
-      <c r="C132" s="1" t="inlineStr">
+      <c r="C135" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">July 2026</t>
         </is>
       </c>
-      <c r="D132" s="1" t="inlineStr">
+      <c r="D135" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">August 2026</t>
         </is>
       </c>
-      <c r="E132" s="1" t="inlineStr">
+      <c r="E135" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">September 2026</t>
         </is>
       </c>
-      <c r="F132" s="1" t="inlineStr">
+      <c r="F135" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">4-Month Total</t>
         </is>
       </c>
-      <c r="G132" s="1" t="inlineStr">
+      <c r="G135" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Monthly Avg</t>
         </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A&amp;D Mortgage</t>
-        </is>
-      </c>
-      <c r="B133" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="C133" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="D133" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="E133" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A133,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="F133" s="3">
-        <f>SUM(B133:E133)</f>
-        <v>13644.4</v>
-      </c>
-      <c r="G133" s="3">
-        <f>F133/4</f>
-        <v>3411.1</v>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">St. James Membership (Club)</t>
-        </is>
-      </c>
-      <c r="B134" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1591.78</v>
-      </c>
-      <c r="C134" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>1601.56</v>
-      </c>
-      <c r="D134" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1492.11</v>
-      </c>
-      <c r="E134" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A134,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>1767.0</v>
-      </c>
-      <c r="F134" s="3">
-        <f>SUM(B134:E134)</f>
-        <v>6452.45</v>
-      </c>
-      <c r="G134" s="3">
-        <f>F134/4</f>
-        <v>1613.1125</v>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">St. James Plantation POA Dues</t>
-        </is>
-      </c>
-      <c r="B135" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>692.95</v>
-      </c>
-      <c r="C135" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D135" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
-      </c>
-      <c r="E135" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A135,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
-      </c>
-      <c r="F135" s="3">
-        <f>SUM(B135:E135)</f>
-        <v>692.95</v>
-      </c>
-      <c r="G135" s="3">
-        <f>F135/4</f>
-        <v>173.2375</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">A&amp;D Mortgage</t>
         </is>
       </c>
       <c r="B136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>360.42</v>
+        <v>3411.1</v>
       </c>
       <c r="C136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>360.42</v>
+        <v>3411.1</v>
       </c>
       <c r="D136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>475.42</v>
+        <v>3411.1</v>
       </c>
       <c r="E136" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>354.17</v>
+        <v>3411.1</v>
       </c>
       <c r="F136" s="3">
         <f>SUM(B136:E136)</f>
-        <v>1550.43</v>
+        <v>13644.4</v>
       </c>
       <c r="G136" s="3">
         <f>F136/4</f>
-        <v>387.6075</v>
+        <v>3411.1</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">St. James Membership (Club)</t>
         </is>
       </c>
       <c r="B137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>79.21</v>
+        <v>1591.78</v>
       </c>
       <c r="C137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>73.61</v>
+        <v>1601.56</v>
       </c>
       <c r="D137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>73.61</v>
+        <v>1492.11</v>
       </c>
       <c r="E137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>73.61</v>
+        <v>1767.0</v>
       </c>
       <c r="F137" s="3">
         <f>SUM(B137:E137)</f>
-        <v>300.04</v>
+        <v>6452.45</v>
       </c>
       <c r="G137" s="3">
         <f>F137/4</f>
-        <v>75.01</v>
+        <v>1613.1125</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Banner Life Insurance</t>
+          <t xml:space="preserve">St. James Plantation POA Dues</t>
         </is>
       </c>
       <c r="B138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>710.06</v>
+        <v>692.95</v>
       </c>
       <c r="C138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>710.06</v>
+        <v>0</v>
       </c>
       <c r="D138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>710.06</v>
+        <v>0</v>
       </c>
       <c r="E138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>710.06</v>
+        <v>0</v>
       </c>
       <c r="F138" s="3">
         <f>SUM(B138:E138)</f>
-        <v>2840.24</v>
+        <v>692.95</v>
       </c>
       <c r="G138" s="3">
         <f>F138/4</f>
-        <v>710.06</v>
+        <v>173.2375</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="B139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>360.42</v>
       </c>
       <c r="C139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>360.42</v>
       </c>
       <c r="D139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>475.42</v>
       </c>
       <c r="E139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>354.17</v>
       </c>
       <c r="F139" s="3">
         <f>SUM(B139:E139)</f>
-        <v>1412.24</v>
+        <v>1550.43</v>
       </c>
       <c r="G139" s="3">
         <f>F139/4</f>
-        <v>353.06</v>
+        <v>387.6075</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="B140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.37</v>
+        <v>79.21</v>
       </c>
       <c r="C140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>160.37</v>
+        <v>73.61</v>
       </c>
       <c r="D140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>160.37</v>
+        <v>73.61</v>
       </c>
       <c r="E140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>160.37</v>
+        <v>73.61</v>
       </c>
       <c r="F140" s="3">
         <f>SUM(B140:E140)</f>
-        <v>641.48</v>
+        <v>300.04</v>
       </c>
       <c r="G140" s="3">
         <f>F140/4</f>
-        <v>160.37</v>
+        <v>75.01</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVS Pharmacy</t>
+          <t xml:space="preserve">Banner Life Insurance</t>
         </is>
       </c>
       <c r="B141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.07</v>
+        <v>710.06</v>
       </c>
       <c r="C141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.93</v>
+        <v>710.06</v>
       </c>
       <c r="D141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>383.24</v>
+        <v>710.06</v>
       </c>
       <c r="E141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>710.06</v>
       </c>
       <c r="F141" s="3">
         <f>SUM(B141:E141)</f>
-        <v>644.24</v>
+        <v>2840.24</v>
       </c>
       <c r="G141" s="3">
         <f>F141/4</f>
-        <v>161.06</v>
+        <v>710.06</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>294.57</v>
       </c>
       <c r="C142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>294.8</v>
       </c>
       <c r="D142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>436.02</v>
       </c>
       <c r="E142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>386.85</v>
       </c>
       <c r="F142" s="3">
         <f>SUM(B142:E142)</f>
-        <v>1162.97</v>
+        <v>1412.24</v>
       </c>
       <c r="G142" s="3">
         <f>F142/4</f>
-        <v>290.7425</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="B143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>160.37</v>
       </c>
       <c r="C143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>160.37</v>
       </c>
       <c r="D143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>160.37</v>
       </c>
       <c r="E143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>160.37</v>
       </c>
       <c r="F143" s="3">
         <f>SUM(B143:E143)</f>
-        <v>342.43</v>
+        <v>641.48</v>
       </c>
       <c r="G143" s="3">
         <f>F143/4</f>
-        <v>85.6075</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">CVS Pharmacy</t>
+        </is>
+      </c>
+      <c r="B144" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>160.07</v>
+      </c>
+      <c r="C144" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>100.93</v>
+      </c>
+      <c r="D144" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>383.24</v>
+      </c>
+      <c r="E144" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F144" s="3">
+        <f>SUM(B144:E144)</f>
+        <v>644.24</v>
+      </c>
+      <c r="G144" s="3">
+        <f>F144/4</f>
+        <v>161.06</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+        </is>
+      </c>
+      <c r="B145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>336.35</v>
+      </c>
+      <c r="D145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>406.96</v>
+      </c>
+      <c r="E145" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>419.66</v>
+      </c>
+      <c r="F145" s="3">
+        <f>SUM(B145:E145)</f>
+        <v>1162.97</v>
+      </c>
+      <c r="G145" s="3">
+        <f>F145/4</f>
+        <v>290.7425</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+        </is>
+      </c>
+      <c r="B146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>179.33</v>
+      </c>
+      <c r="E146" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>84.26</v>
+      </c>
+      <c r="F146" s="3">
+        <f>SUM(B146:E146)</f>
+        <v>342.43</v>
+      </c>
+      <c r="G146" s="3">
+        <f>F146/4</f>
+        <v>85.6075</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
-      <c r="B144" s="3">
+      <c r="B147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>78.84</v>
       </c>
-      <c r="C144" s="3">
+      <c r="C147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
-      <c r="D144" s="3">
+      <c r="D147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>586.29</v>
       </c>
-      <c r="E144" s="3">
+      <c r="E147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>503.92</v>
       </c>
-      <c r="F144" s="3">
-        <f>SUM(B144:E144)</f>
-        <v>1505.4</v>
-      </c>
-      <c r="G144" s="3">
-        <f>F144/4</f>
-        <v>376.35</v>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
-        </is>
-      </c>
-      <c r="B145" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="C145" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D145" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
-      </c>
-      <c r="E145" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="F145" s="3">
-        <f>SUM(B145:E145)</f>
-        <v>323.16</v>
-      </c>
-      <c r="G145" s="3">
-        <f>F145/4</f>
-        <v>80.79</v>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
-        </is>
-      </c>
-      <c r="B146" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
-      </c>
-      <c r="C146" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>935.1</v>
-      </c>
-      <c r="D146" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
-      </c>
-      <c r="E146" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>848.05</v>
-      </c>
-      <c r="F146" s="3">
-        <f>SUM(B146:E146)</f>
-        <v>3765.22</v>
-      </c>
-      <c r="G146" s="3">
-        <f>F146/4</f>
-        <v>941.305</v>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
-        </is>
-      </c>
-      <c r="B147" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
-      </c>
-      <c r="C147" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
-      </c>
-      <c r="D147" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
-      </c>
-      <c r="E147" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
-      </c>
       <c r="F147" s="3">
         <f>SUM(B147:E147)</f>
-        <v>792.99</v>
+        <v>1505.4</v>
       </c>
       <c r="G147" s="3">
         <f>F147/4</f>
-        <v>198.2475</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
+        </is>
+      </c>
+      <c r="B148" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>80.79</v>
+      </c>
+      <c r="C148" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D148" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>161.58</v>
+      </c>
+      <c r="E148" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>80.79</v>
+      </c>
+      <c r="F148" s="3">
+        <f>SUM(B148:E148)</f>
+        <v>323.16</v>
+      </c>
+      <c r="G148" s="3">
+        <f>F148/4</f>
+        <v>80.79</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+        </is>
+      </c>
+      <c r="B149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>1019.45</v>
+      </c>
+      <c r="C149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>909.94</v>
+      </c>
+      <c r="D149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>962.62</v>
+      </c>
+      <c r="E149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>839.3</v>
+      </c>
+      <c r="F149" s="3">
+        <f>SUM(B149:E149)</f>
+        <v>3731.31</v>
+      </c>
+      <c r="G149" s="3">
+        <f>F149/4</f>
+        <v>932.8275</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B150" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C150" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D150" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E150" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F150" s="3">
+        <f>SUM(B150:E150)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G150" s="3">
+        <f>F150/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B148" s="3">
+      <c r="B151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C148" s="3">
+      <c r="C151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D148" s="3">
+      <c r="D151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E148" s="3">
+      <c r="E151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F148" s="3">
-        <f>SUM(B148:E148)</f>
+      <c r="F151" s="3">
+        <f>SUM(B151:E151)</f>
         <v>4932.41</v>
       </c>
-      <c r="G148" s="3">
-        <f>F148/4</f>
+      <c r="G151" s="3">
+        <f>F151/4</f>
         <v>1233.1025</v>
       </c>
     </row>
-    <row r="149">
-      <c r="A149" s="12" t="inlineStr">
+    <row r="152">
+      <c r="A152" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
-      <c r="B149" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,B$4)</f>
+      <c r="B152" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>182.5</v>
       </c>
-      <c r="C149" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,C$4)</f>
+      <c r="C152" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>0</v>
       </c>
-      <c r="D149" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,D$4)</f>
+      <c r="D152" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>182.5</v>
       </c>
-      <c r="E149" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,E$4)</f>
+      <c r="E152" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>32.5</v>
       </c>
-      <c r="F149" s="3">
-        <f>SUM(B149:E149)</f>
+      <c r="F152" s="3">
+        <f>SUM(B152:E152)</f>
         <v>397.5</v>
       </c>
-      <c r="G149" s="3">
-        <f>F149/4</f>
+      <c r="G152" s="3">
+        <f>F152/4</f>
         <v>99.375</v>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="12" t="inlineStr">
+    <row r="153">
+      <c r="A153" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B150" s="3">
+      <c r="B153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C150" s="3">
+      <c r="C153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D150" s="3">
+      <c r="D153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E150" s="3">
+      <c r="E153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>357.62</v>
       </c>
-      <c r="F150" s="3">
-        <f>SUM(B150:E150)</f>
+      <c r="F153" s="3">
+        <f>SUM(B153:E153)</f>
         <v>4703.69</v>
       </c>
-      <c r="G150" s="3">
-        <f>F150/4</f>
+      <c r="G153" s="3">
+        <f>F153/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="12" t="inlineStr">
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B151" s="3">
+      <c r="B154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C151" s="3">
+      <c r="C154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D151" s="3">
+      <c r="D154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E151" s="3">
+      <c r="E154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F151" s="3">
-        <f>SUM(B151:E151)</f>
+      <c r="F154" s="3">
+        <f>SUM(B154:E154)</f>
         <v>737.73</v>
       </c>
-      <c r="G151" s="3">
-        <f>F151/4</f>
+      <c r="G154" s="3">
+        <f>F154/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="153">
-      <c r="A153" s="5" t="inlineStr">
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="154" ht="27" customHeight="1">
-      <c r="A154" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="27" customHeight="1">
-      <c r="A155" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" ht="27" customHeight="1">
-      <c r="A156" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="157" ht="27" customHeight="1">
       <c r="A157" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="158" ht="27" customHeight="1">
       <c r="A158" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="159" ht="27" customHeight="1">
       <c r="A159" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="160" ht="27" customHeight="1">
       <c r="A160" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Small hospital-cafeteria charges (Granville Med, Duke) are counted as Restaurants.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="27" customHeight="1">
+      <c r="A161" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="27" customHeight="1">
+      <c r="A162" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="27" customHeight="1">
+      <c r="A163" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Granville Medical and Duke charges are small hospital food/parking charges, listed under Health.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A154:G154"/>
-    <mergeCell ref="A155:G155"/>
-    <mergeCell ref="A156:G156"/>
     <mergeCell ref="A157:G157"/>
     <mergeCell ref="A158:G158"/>
     <mergeCell ref="A159:G159"/>
     <mergeCell ref="A160:G160"/>
+    <mergeCell ref="A161:G161"/>
+    <mergeCell ref="A162:G162"/>
+    <mergeCell ref="A163:G163"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -7011,7 +7104,7 @@
       </c>
       <c r="H7" s="3">
         <f>SUMIF($C$4:$C$127,G7,$E$4:$E$127)</f>
-        <v>935.1</v>
+        <v>909.94</v>
       </c>
     </row>
     <row r="8">
@@ -7710,12 +7803,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Frndly TV</t>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
         </is>
       </c>
       <c r="H29" s="3">
         <f>SUMIF($C$4:$C$127,G29,$E$4:$E$127)</f>
-        <v>22.41</v>
+        <v>25.16</v>
       </c>
     </row>
     <row r="30">
@@ -7742,12 +7835,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
+          <t xml:space="preserve">Streaming – Frndly TV</t>
         </is>
       </c>
       <c r="H30" s="3">
         <f>SUMIF($C$4:$C$127,G30,$E$4:$E$127)</f>
-        <v>20.27</v>
+        <v>22.41</v>
       </c>
     </row>
     <row r="31">
@@ -7774,12 +7867,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – HBO Max</t>
+          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
         </is>
       </c>
       <c r="H31" s="3">
         <f>SUMIF($C$4:$C$127,G31,$E$4:$E$127)</f>
-        <v>19.74</v>
+        <v>20.27</v>
       </c>
     </row>
     <row r="32">
@@ -7806,12 +7899,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+          <t xml:space="preserve">Streaming – HBO Max</t>
         </is>
       </c>
       <c r="H32" s="3">
         <f>SUMIF($C$4:$C$127,G32,$E$4:$E$127)</f>
-        <v>13.87</v>
+        <v>19.74</v>
       </c>
     </row>
     <row r="33">
@@ -7825,12 +7918,12 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="E33" s="3">
@@ -7838,12 +7931,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Hulu</t>
+          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
         </is>
       </c>
       <c r="H33" s="3">
         <f>SUMIF($C$4:$C$127,G33,$E$4:$E$127)</f>
-        <v>12.8</v>
+        <v>13.87</v>
       </c>
     </row>
     <row r="34">
@@ -7870,12 +7963,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Peacock (via Roku)</t>
+          <t xml:space="preserve">Streaming – Hulu</t>
         </is>
       </c>
       <c r="H34" s="3">
         <f>SUMIF($C$4:$C$127,G34,$E$4:$E$127)</f>
-        <v>11.73</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="35">
@@ -7902,12 +7995,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+          <t xml:space="preserve">Streaming – Peacock (via Roku)</t>
         </is>
       </c>
       <c r="H35" s="3">
         <f>SUMIF($C$4:$C$127,G35,$E$4:$E$127)</f>
-        <v>5.87</v>
+        <v>11.73</v>
       </c>
     </row>
     <row r="36">
@@ -7921,25 +8014,25 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="E36" s="3">
         <v>8.85</v>
       </c>
-      <c r="G36" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total spending</t>
-        </is>
-      </c>
-      <c r="H36" s="9">
-        <f>SUM(H4:H35)</f>
-        <v>12663.24</v>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
+        </is>
+      </c>
+      <c r="H36" s="3">
+        <f>SUMIF($C$4:$C$127,G36,$E$4:$E$127)</f>
+        <v>5.87</v>
       </c>
     </row>
     <row r="37">
@@ -7964,6 +8057,15 @@
       <c r="E37" s="3">
         <v>24.15</v>
       </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total spending</t>
+        </is>
+      </c>
+      <c r="H37" s="9">
+        <f>SUM(H4:H36)</f>
+        <v>12663.24</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4">
@@ -7987,12 +8089,6 @@
       <c r="E38" s="3">
         <v>24.34</v>
       </c>
-      <c r="G38" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not counted as spending</t>
-        </is>
-      </c>
-      <c r="H38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="4">
@@ -8016,15 +8112,12 @@
       <c r="E39" s="3">
         <v>12.21</v>
       </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
-        </is>
-      </c>
-      <c r="H39" s="3">
-        <f>SUMIF($C$4:$C$127,G39,$E$4:$E$127)</f>
-        <v>7227.09</v>
-      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not counted as spending</t>
+        </is>
+      </c>
+      <c r="H39" s="7"/>
     </row>
     <row r="40">
       <c r="A40" s="4">
@@ -8050,12 +8143,12 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sloane Realty</t>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
         </is>
       </c>
       <c r="H40" s="3">
         <f>SUMIF($C$4:$C$127,G40,$E$4:$E$127)</f>
-        <v>2891.98</v>
+        <v>7227.09</v>
       </c>
     </row>
     <row r="41">
@@ -8082,12 +8175,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Sloane Realty</t>
         </is>
       </c>
       <c r="H41" s="3">
         <f>SUMIF($C$4:$C$127,G41,$E$4:$E$127)</f>
-        <v>3.26</v>
+        <v>2891.98</v>
       </c>
     </row>
     <row r="42">
@@ -8101,12 +8194,12 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="E42" s="3">
@@ -8114,12 +8207,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
         </is>
       </c>
       <c r="H42" s="3">
         <f>SUMIF($C$4:$C$127,G42,$E$4:$E$127)</f>
-        <v>2576.0</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="43">
@@ -8143,6 +8236,15 @@
       </c>
       <c r="E43" s="3">
         <v>49.87</v>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+        </is>
+      </c>
+      <c r="H43" s="3">
+        <f>SUMIF($C$4:$C$127,G43,$E$4:$E$127)</f>
+        <v>2576.0</v>
       </c>
     </row>
     <row r="44">
@@ -10479,7 +10581,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="H13" s="3">
@@ -10594,7 +10696,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -12227,7 +12329,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -13204,7 +13306,7 @@
       </c>
       <c r="H6" s="3">
         <f>SUMIF($C$4:$C$88,G6,$E$4:$E$88)</f>
-        <v>848.05</v>
+        <v>839.3</v>
       </c>
     </row>
     <row r="7">
@@ -13218,7 +13320,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Wilmington Eye</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -13551,12 +13653,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
         </is>
       </c>
       <c r="H17" s="3">
         <f>SUMIF($C$4:$C$88,G17,$E$4:$E$88)</f>
-        <v>160.28</v>
+        <v>147.0</v>
       </c>
     </row>
     <row r="18">
@@ -13583,12 +13685,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cash (ATM) &amp; Bank Fees</t>
+          <t xml:space="preserve">Streaming – YouTube TV (Google)</t>
         </is>
       </c>
       <c r="H18" s="3">
         <f>SUMIF($C$4:$C$88,G18,$E$4:$E$88)</f>
-        <v>147.0</v>
+        <v>132.43</v>
       </c>
     </row>
     <row r="19">
@@ -13615,12 +13717,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – YouTube TV (Google)</t>
+          <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
         </is>
       </c>
       <c r="H19" s="3">
         <f>SUMIF($C$4:$C$88,G19,$E$4:$E$88)</f>
-        <v>132.43</v>
+        <v>130.0</v>
       </c>
     </row>
     <row r="20">
@@ -13647,12 +13749,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
+          <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
       <c r="H20" s="3">
         <f>SUMIF($C$4:$C$88,G20,$E$4:$E$88)</f>
-        <v>130.0</v>
+        <v>120.0</v>
       </c>
     </row>
     <row r="21">
@@ -13679,12 +13781,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yard Company (NextGen)</t>
+          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
         </is>
       </c>
       <c r="H21" s="3">
         <f>SUMIF($C$4:$C$88,G21,$E$4:$E$88)</f>
-        <v>120.0</v>
+        <v>119.97</v>
       </c>
     </row>
     <row r="22">
@@ -13711,12 +13813,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Local shops (Hippie Chick, Southport Spices, Mad River, Coastal Carolina)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="H22" s="3">
         <f>SUMIF($C$4:$C$88,G22,$E$4:$E$88)</f>
-        <v>119.97</v>
+        <v>100.28</v>
       </c>
     </row>
     <row r="23">
@@ -13871,12 +13973,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tolls &amp; Parking</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="H27" s="3">
         <f>SUMIF($C$4:$C$88,G27,$E$4:$E$88)</f>
-        <v>74.24</v>
+        <v>73.61</v>
       </c>
     </row>
     <row r="28">
@@ -13903,12 +14005,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
         </is>
       </c>
       <c r="H28" s="3">
         <f>SUMIF($C$4:$C$88,G28,$E$4:$E$88)</f>
-        <v>73.61</v>
+        <v>69.36</v>
       </c>
     </row>
     <row r="29">
@@ -13935,12 +14037,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
+          <t xml:space="preserve">Tolls &amp; Parking</t>
         </is>
       </c>
       <c r="H29" s="3">
         <f>SUMIF($C$4:$C$88,G29,$E$4:$E$88)</f>
-        <v>69.36</v>
+        <v>68.24</v>
       </c>
     </row>
     <row r="30">
@@ -13967,12 +14069,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Marshalls</t>
+          <t xml:space="preserve">Medical – Wilmington Eye</t>
         </is>
       </c>
       <c r="H30" s="3">
         <f>SUMIF($C$4:$C$88,G30,$E$4:$E$88)</f>
-        <v>41.59</v>
+        <v>60.0</v>
       </c>
     </row>
     <row r="31">
@@ -13999,12 +14101,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Hobby Lobby</t>
+          <t xml:space="preserve">Retail – Marshalls</t>
         </is>
       </c>
       <c r="H31" s="3">
         <f>SUMIF($C$4:$C$88,G31,$E$4:$E$88)</f>
-        <v>37.33</v>
+        <v>41.59</v>
       </c>
     </row>
     <row r="32">
@@ -14031,12 +14133,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Walmart</t>
+          <t xml:space="preserve">Retail – Hobby Lobby</t>
         </is>
       </c>
       <c r="H32" s="3">
         <f>SUMIF($C$4:$C$88,G32,$E$4:$E$88)</f>
-        <v>32.63</v>
+        <v>37.33</v>
       </c>
     </row>
     <row r="33">
@@ -14063,12 +14165,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
+          <t xml:space="preserve">Retail – Walmart</t>
         </is>
       </c>
       <c r="H33" s="3">
         <f>SUMIF($C$4:$C$88,G33,$E$4:$E$88)</f>
-        <v>32.5</v>
+        <v>32.63</v>
       </c>
     </row>
     <row r="34">
@@ -14095,12 +14197,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Cat on a Whisk</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="H34" s="3">
         <f>SUMIF($C$4:$C$88,G34,$E$4:$E$88)</f>
-        <v>24.51</v>
+        <v>32.5</v>
       </c>
     </row>
     <row r="35">
@@ -14127,12 +14229,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Frndly TV</t>
+          <t xml:space="preserve">Retail – Cat on a Whisk</t>
         </is>
       </c>
       <c r="H35" s="3">
         <f>SUMIF($C$4:$C$88,G35,$E$4:$E$88)</f>
-        <v>22.41</v>
+        <v>24.51</v>
       </c>
     </row>
     <row r="36">
@@ -14159,12 +14261,12 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
+          <t xml:space="preserve">Streaming – Frndly TV</t>
         </is>
       </c>
       <c r="H36" s="3">
         <f>SUMIF($C$4:$C$88,G36,$E$4:$E$88)</f>
-        <v>20.27</v>
+        <v>22.41</v>
       </c>
     </row>
     <row r="37">
@@ -14191,12 +14293,12 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Ross</t>
+          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
         </is>
       </c>
       <c r="H37" s="3">
         <f>SUMIF($C$4:$C$88,G37,$E$4:$E$88)</f>
-        <v>16.32</v>
+        <v>20.27</v>
       </c>
     </row>
     <row r="38">
@@ -14223,12 +14325,12 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+          <t xml:space="preserve">Retail – Ross</t>
         </is>
       </c>
       <c r="H38" s="3">
         <f>SUMIF($C$4:$C$88,G38,$E$4:$E$88)</f>
-        <v>13.87</v>
+        <v>16.32</v>
       </c>
     </row>
     <row r="39">
@@ -14253,14 +14355,14 @@
       <c r="E39" s="3">
         <v>221.77</v>
       </c>
-      <c r="G39" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total spending</t>
-        </is>
-      </c>
-      <c r="H39" s="9">
-        <f>SUM(H4:H38)</f>
-        <v>11515.63</v>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Medical – Duke Hospital (Durham, food &amp; parking)</t>
+        </is>
+      </c>
+      <c r="H39" s="3">
+        <f>SUMIF($C$4:$C$88,G39,$E$4:$E$88)</f>
+        <v>14.75</v>
       </c>
     </row>
     <row r="40">
@@ -14285,6 +14387,15 @@
       <c r="E40" s="3">
         <v>2576.0</v>
       </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+        </is>
+      </c>
+      <c r="H40" s="3">
+        <f>SUMIF($C$4:$C$88,G40,$E$4:$E$88)</f>
+        <v>13.87</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4">
@@ -14308,12 +14419,15 @@
       <c r="E41" s="3">
         <v>68.24</v>
       </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not counted as spending</t>
-        </is>
-      </c>
-      <c r="H41" s="7"/>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total spending</t>
+        </is>
+      </c>
+      <c r="H41" s="9">
+        <f>SUM(H4:H40)</f>
+        <v>11515.63</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4">
@@ -14337,15 +14451,6 @@
       <c r="E42" s="3">
         <v>216.25</v>
       </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Credit Card Payoff – American Express</t>
-        </is>
-      </c>
-      <c r="H42" s="3">
-        <f>SUMIF($C$4:$C$88,G42,$E$4:$E$88)</f>
-        <v>4738.51</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" s="4">
@@ -14358,7 +14463,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -14369,15 +14474,12 @@
       <c r="E43" s="3">
         <v>100.28</v>
       </c>
-      <c r="G43" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
-        </is>
-      </c>
-      <c r="H43" s="3">
-        <f>SUMIF($C$4:$C$88,G43,$E$4:$E$88)</f>
-        <v>2576.0</v>
-      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not counted as spending</t>
+        </is>
+      </c>
+      <c r="H43" s="7"/>
     </row>
     <row r="44">
       <c r="A44" s="4">
@@ -14401,6 +14503,15 @@
       <c r="E44" s="3">
         <v>419.66</v>
       </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Credit Card Payoff – American Express</t>
+        </is>
+      </c>
+      <c r="H44" s="3">
+        <f>SUMIF($C$4:$C$88,G44,$E$4:$E$88)</f>
+        <v>4738.51</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4">
@@ -14424,6 +14535,15 @@
       <c r="E45" s="3">
         <v>80.79</v>
       </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+        </is>
+      </c>
+      <c r="H45" s="3">
+        <f>SUMIF($C$4:$C$88,G45,$E$4:$E$88)</f>
+        <v>2576.0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4">
@@ -14666,12 +14786,12 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Medical – Duke Hospital (Durham, food &amp; parking)</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="E56" s="3">
@@ -14712,12 +14832,12 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tolls &amp; Parking</t>
+          <t xml:space="preserve">Medical – Duke Hospital (Durham, food &amp; parking)</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transportation</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="E58" s="3">
@@ -19580,12 +19700,12 @@
       </c>
       <c r="D150" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
         </is>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="F150" s="3">
@@ -19664,12 +19784,12 @@
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
         </is>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="F153" s="3">
@@ -19832,12 +19952,12 @@
       </c>
       <c r="D159" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
         </is>
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="F159" s="3">
@@ -22604,7 +22724,7 @@
       </c>
       <c r="D258" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="E258" s="2" t="inlineStr">
@@ -24256,7 +24376,7 @@
       </c>
       <c r="D317" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="E317" s="2" t="inlineStr">
@@ -25320,7 +25440,7 @@
       </c>
       <c r="D355" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Wilmington Eye</t>
         </is>
       </c>
       <c r="E355" s="2" t="inlineStr">
@@ -26328,7 +26448,7 @@
       </c>
       <c r="D391" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical (Dosher Hospital, Wilmington Eye)</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="E391" s="2" t="inlineStr">
@@ -26692,12 +26812,12 @@
       </c>
       <c r="D404" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Medical – Duke Hospital (Durham, food &amp; parking)</t>
         </is>
       </c>
       <c r="E404" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Food</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="F404" s="3">
@@ -26748,12 +26868,12 @@
       </c>
       <c r="D406" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tolls &amp; Parking</t>
+          <t xml:space="preserve">Medical – Duke Hospital (Durham, food &amp; parking)</t>
         </is>
       </c>
       <c r="E406" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transportation</t>
+          <t xml:space="preserve">Health</t>
         </is>
       </c>
       <c r="F406" s="3">

</xml_diff>

<commit_message>
Exclude Dust and Mop House from spending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -2395,7 +2395,7 @@
     <row r="99">
       <c r="A99" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
         </is>
       </c>
       <c r="B99" s="3">
@@ -2404,11 +2404,11 @@
       </c>
       <c r="C99" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>242.05</v>
+        <v>142.05</v>
       </c>
       <c r="D99" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>536.6</v>
+        <v>104.0</v>
       </c>
       <c r="E99" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A99,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2416,11 +2416,11 @@
       </c>
       <c r="F99" s="3">
         <f>SUM(B99:E99)</f>
-        <v>778.65</v>
+        <v>246.05</v>
       </c>
       <c r="G99" s="3">
         <f>F99/4</f>
-        <v>194.6625</v>
+        <v>61.5125</v>
       </c>
     </row>
     <row r="100">
@@ -2435,11 +2435,11 @@
       </c>
       <c r="C100" s="6">
         <f>SUM(C98:C99)</f>
-        <v>342.05</v>
+        <v>242.05</v>
       </c>
       <c r="D100" s="6">
         <f>SUM(D98:D99)</f>
-        <v>756.6</v>
+        <v>324.0</v>
       </c>
       <c r="E100" s="6">
         <f>SUM(E98:E99)</f>
@@ -2447,11 +2447,11 @@
       </c>
       <c r="F100" s="6">
         <f>SUM(F98:F99)</f>
-        <v>1278.65</v>
+        <v>746.05</v>
       </c>
       <c r="G100" s="6">
         <f>F100/4</f>
-        <v>319.6625</v>
+        <v>186.5125</v>
       </c>
     </row>
     <row r="102">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="C120" s="9">
         <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C71+C76+C95+C100+C104+C109+C113+C118</f>
-        <v>12663.24</v>
+        <v>12563.24</v>
       </c>
       <c r="D120" s="9">
         <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D71+D76+D95+D100+D104+D109+D113+D118</f>
-        <v>15086.64</v>
+        <v>14654.04</v>
       </c>
       <c r="E120" s="9">
         <f>E10+E18+E23+E28+E32+E38+E43+E48+E59+E63+E71+E76+E95+E100+E104+E109+E113+E118</f>
@@ -2816,11 +2816,11 @@
       </c>
       <c r="F120" s="9">
         <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F71+F76+F95+F100+F104+F109+F113+F118</f>
-        <v>51401.32</v>
+        <v>50868.72</v>
       </c>
       <c r="G120" s="9">
         <f>F120/4</f>
-        <v>12850.33</v>
+        <v>12717.18</v>
       </c>
     </row>
     <row r="122">
@@ -2926,20 +2926,20 @@
     <row r="126">
       <c r="A126" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checks Written (payee not shown)</t>
+          <t xml:space="preserve">Dust and Mop House</t>
         </is>
       </c>
       <c r="B126" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2630.0</v>
+        <v>0</v>
       </c>
       <c r="C126" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>100.0</v>
       </c>
       <c r="D126" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>728.0</v>
+        <v>432.6</v>
       </c>
       <c r="E126" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A126,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2947,30 +2947,30 @@
       </c>
       <c r="F126" s="3">
         <f>SUM(B126:E126)</f>
-        <v>3358.0</v>
+        <v>532.6</v>
       </c>
       <c r="G126" s="3">
         <f>F126/4</f>
-        <v>839.5</v>
+        <v>133.15</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Checks Written (payee not shown)</t>
         </is>
       </c>
       <c r="B127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>2630.0</v>
       </c>
       <c r="C127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3.26</v>
+        <v>0</v>
       </c>
       <c r="D127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>728.0</v>
       </c>
       <c r="E127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2978,819 +2978,850 @@
       </c>
       <c r="F127" s="3">
         <f>SUM(B127:E127)</f>
-        <v>3.26</v>
+        <v>3358.0</v>
       </c>
       <c r="G127" s="3">
         <f>F127/4</f>
+        <v>839.5</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
+        </is>
+      </c>
+      <c r="B128" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C128" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>3.26</v>
+      </c>
+      <c r="D128" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E128" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F128" s="3">
+        <f>SUM(B128:E128)</f>
+        <v>3.26</v>
+      </c>
+      <c r="G128" s="3">
+        <f>F128/4</f>
         <v>0.815</v>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="7" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total not counted as spending</t>
         </is>
       </c>
-      <c r="B128" s="6">
-        <f>SUM(B123:B127)</f>
+      <c r="B129" s="6">
+        <f>SUM(B123:B128)</f>
         <v>5206.0</v>
       </c>
-      <c r="C128" s="6">
-        <f>SUM(C123:C127)</f>
-        <v>12698.33</v>
-      </c>
-      <c r="D128" s="6">
-        <f>SUM(D123:D127)</f>
-        <v>7897.08</v>
-      </c>
-      <c r="E128" s="6">
-        <f>SUM(E123:E127)</f>
+      <c r="C129" s="6">
+        <f>SUM(C123:C128)</f>
+        <v>12798.33</v>
+      </c>
+      <c r="D129" s="6">
+        <f>SUM(D123:D128)</f>
+        <v>8329.68</v>
+      </c>
+      <c r="E129" s="6">
+        <f>SUM(E123:E128)</f>
         <v>7314.51</v>
       </c>
-      <c r="F128" s="6">
-        <f>SUM(F123:F127)</f>
-        <v>33115.92</v>
-      </c>
-      <c r="G128" s="6">
-        <f>F128/4</f>
-        <v>8278.98</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Check: spending + not-counted items</t>
-        </is>
-      </c>
-      <c r="B130" s="3">
-        <f>B120+B128</f>
-        <v>17341.81</v>
-      </c>
-      <c r="C130" s="3">
-        <f>C120+C128</f>
-        <v>25361.57</v>
-      </c>
-      <c r="D130" s="3">
-        <f>D120+D128</f>
-        <v>22983.72</v>
-      </c>
-      <c r="E130" s="3">
-        <f>E120+E128</f>
-        <v>18830.14</v>
-      </c>
-      <c r="F130" s="3">
-        <f>F120+F128</f>
-        <v>84517.24</v>
+      <c r="F129" s="6">
+        <f>SUM(F123:F128)</f>
+        <v>33648.52</v>
+      </c>
+      <c r="G129" s="6">
+        <f>F129/4</f>
+        <v>8412.13</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
-        </is>
-      </c>
-      <c r="B131" s="13">
+          <t xml:space="preserve">Check: spending + not-counted items</t>
+        </is>
+      </c>
+      <c r="B131" s="3">
+        <f>B120+B129</f>
         <v>17341.81</v>
       </c>
-      <c r="C131" s="13">
+      <c r="C131" s="3">
+        <f>C120+C129</f>
         <v>25361.57</v>
       </c>
-      <c r="D131" s="13">
+      <c r="D131" s="3">
+        <f>D120+D129</f>
         <v>22983.72</v>
       </c>
-      <c r="E131" s="13">
+      <c r="E131" s="3">
+        <f>E120+E129</f>
         <v>18830.14</v>
       </c>
       <c r="F131" s="3">
-        <f>SUM(B131:E131)</f>
+        <f>F120+F129</f>
         <v>84517.24</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
+        </is>
+      </c>
+      <c r="B132" s="13">
+        <v>17341.81</v>
+      </c>
+      <c r="C132" s="13">
+        <v>25361.57</v>
+      </c>
+      <c r="D132" s="13">
+        <v>22983.72</v>
+      </c>
+      <c r="E132" s="13">
+        <v>18830.14</v>
+      </c>
+      <c r="F132" s="3">
+        <f>SUM(B132:E132)</f>
+        <v>84517.24</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Difference (should be $0 = every dollar accounted for)</t>
         </is>
       </c>
-      <c r="B132" s="3">
-        <f>B130-B131</f>
+      <c r="B133" s="3">
+        <f>B131-B132</f>
         <v>0.0</v>
       </c>
-      <c r="C132" s="3">
-        <f>C130-C131</f>
+      <c r="C133" s="3">
+        <f>C131-C132</f>
         <v>0.0</v>
       </c>
-      <c r="D132" s="3">
-        <f>D130-D131</f>
+      <c r="D133" s="3">
+        <f>D131-D132</f>
         <v>0.0</v>
       </c>
-      <c r="E132" s="3">
-        <f>E130-E131</f>
+      <c r="E133" s="3">
+        <f>E131-E132</f>
         <v>0.0</v>
       </c>
-      <c r="F132" s="3">
-        <f>F130-F131</f>
+      <c r="F133" s="3">
+        <f>F131-F132</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="134">
-      <c r="A134" s="5" t="inlineStr">
+    <row r="135">
+      <c r="A135" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Key Bills at a Glance</t>
         </is>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="15" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Bill</t>
         </is>
       </c>
-      <c r="B135" s="1" t="inlineStr">
+      <c r="B136" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">June 2026</t>
         </is>
       </c>
-      <c r="C135" s="1" t="inlineStr">
+      <c r="C136" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">July 2026</t>
         </is>
       </c>
-      <c r="D135" s="1" t="inlineStr">
+      <c r="D136" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">August 2026</t>
         </is>
       </c>
-      <c r="E135" s="1" t="inlineStr">
+      <c r="E136" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">September 2026</t>
         </is>
       </c>
-      <c r="F135" s="1" t="inlineStr">
+      <c r="F136" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">4-Month Total</t>
         </is>
       </c>
-      <c r="G135" s="1" t="inlineStr">
+      <c r="G136" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Monthly Avg</t>
         </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A&amp;D Mortgage</t>
-        </is>
-      </c>
-      <c r="B136" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="C136" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="D136" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="E136" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A136,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="F136" s="3">
-        <f>SUM(B136:E136)</f>
-        <v>13644.4</v>
-      </c>
-      <c r="G136" s="3">
-        <f>F136/4</f>
-        <v>3411.1</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Membership (Club)</t>
+          <t xml:space="preserve">A&amp;D Mortgage</t>
         </is>
       </c>
       <c r="B137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1591.78</v>
+        <v>3411.1</v>
       </c>
       <c r="C137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>1601.56</v>
+        <v>3411.1</v>
       </c>
       <c r="D137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1492.11</v>
+        <v>3411.1</v>
       </c>
       <c r="E137" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>1767.0</v>
+        <v>3411.1</v>
       </c>
       <c r="F137" s="3">
         <f>SUM(B137:E137)</f>
-        <v>6452.45</v>
+        <v>13644.4</v>
       </c>
       <c r="G137" s="3">
         <f>F137/4</f>
-        <v>1613.1125</v>
+        <v>3411.1</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Plantation POA Dues</t>
+          <t xml:space="preserve">St. James Membership (Club)</t>
         </is>
       </c>
       <c r="B138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>692.95</v>
+        <v>1591.78</v>
       </c>
       <c r="C138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>1601.56</v>
       </c>
       <c r="D138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1492.11</v>
       </c>
       <c r="E138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>1767.0</v>
       </c>
       <c r="F138" s="3">
         <f>SUM(B138:E138)</f>
-        <v>692.95</v>
+        <v>6452.45</v>
       </c>
       <c r="G138" s="3">
         <f>F138/4</f>
-        <v>173.2375</v>
+        <v>1613.1125</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">St. James Plantation POA Dues</t>
         </is>
       </c>
       <c r="B139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>360.42</v>
+        <v>692.95</v>
       </c>
       <c r="C139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>360.42</v>
+        <v>0</v>
       </c>
       <c r="D139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>475.42</v>
+        <v>0</v>
       </c>
       <c r="E139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>354.17</v>
+        <v>0</v>
       </c>
       <c r="F139" s="3">
         <f>SUM(B139:E139)</f>
-        <v>1550.43</v>
+        <v>692.95</v>
       </c>
       <c r="G139" s="3">
         <f>F139/4</f>
-        <v>387.6075</v>
+        <v>173.2375</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="B140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>79.21</v>
+        <v>360.42</v>
       </c>
       <c r="C140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>73.61</v>
+        <v>360.42</v>
       </c>
       <c r="D140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>73.61</v>
+        <v>475.42</v>
       </c>
       <c r="E140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>73.61</v>
+        <v>354.17</v>
       </c>
       <c r="F140" s="3">
         <f>SUM(B140:E140)</f>
-        <v>300.04</v>
+        <v>1550.43</v>
       </c>
       <c r="G140" s="3">
         <f>F140/4</f>
-        <v>75.01</v>
+        <v>387.6075</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Banner Life Insurance</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="B141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>710.06</v>
+        <v>79.21</v>
       </c>
       <c r="C141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="D141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="E141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="F141" s="3">
         <f>SUM(B141:E141)</f>
-        <v>2840.24</v>
+        <v>300.04</v>
       </c>
       <c r="G141" s="3">
         <f>F141/4</f>
-        <v>710.06</v>
+        <v>75.01</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Banner Life Insurance</t>
         </is>
       </c>
       <c r="B142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>710.06</v>
       </c>
       <c r="C142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>710.06</v>
       </c>
       <c r="D142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>710.06</v>
       </c>
       <c r="E142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>710.06</v>
       </c>
       <c r="F142" s="3">
         <f>SUM(B142:E142)</f>
-        <v>1412.24</v>
+        <v>2840.24</v>
       </c>
       <c r="G142" s="3">
         <f>F142/4</f>
-        <v>353.06</v>
+        <v>710.06</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.37</v>
+        <v>294.57</v>
       </c>
       <c r="C143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>160.37</v>
+        <v>294.8</v>
       </c>
       <c r="D143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>160.37</v>
+        <v>436.02</v>
       </c>
       <c r="E143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>160.37</v>
+        <v>386.85</v>
       </c>
       <c r="F143" s="3">
         <f>SUM(B143:E143)</f>
-        <v>641.48</v>
+        <v>1412.24</v>
       </c>
       <c r="G143" s="3">
         <f>F143/4</f>
-        <v>160.37</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVS Pharmacy</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="B144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.07</v>
+        <v>160.37</v>
       </c>
       <c r="C144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.93</v>
+        <v>160.37</v>
       </c>
       <c r="D144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>383.24</v>
+        <v>160.37</v>
       </c>
       <c r="E144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>160.37</v>
       </c>
       <c r="F144" s="3">
         <f>SUM(B144:E144)</f>
-        <v>644.24</v>
+        <v>641.48</v>
       </c>
       <c r="G144" s="3">
         <f>F144/4</f>
-        <v>161.06</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="B145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>160.07</v>
       </c>
       <c r="C145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>100.93</v>
       </c>
       <c r="D145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>383.24</v>
       </c>
       <c r="E145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>0</v>
       </c>
       <c r="F145" s="3">
         <f>SUM(B145:E145)</f>
-        <v>1162.97</v>
+        <v>644.24</v>
       </c>
       <c r="G145" s="3">
         <f>F145/4</f>
-        <v>290.7425</v>
+        <v>161.06</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>0</v>
       </c>
       <c r="C146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>336.35</v>
       </c>
       <c r="D146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>406.96</v>
       </c>
       <c r="E146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>419.66</v>
       </c>
       <c r="F146" s="3">
         <f>SUM(B146:E146)</f>
-        <v>342.43</v>
+        <v>1162.97</v>
       </c>
       <c r="G146" s="3">
         <f>F146/4</f>
-        <v>85.6075</v>
+        <v>290.7425</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+        </is>
+      </c>
+      <c r="B147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>179.33</v>
+      </c>
+      <c r="E147" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>84.26</v>
+      </c>
+      <c r="F147" s="3">
+        <f>SUM(B147:E147)</f>
+        <v>342.43</v>
+      </c>
+      <c r="G147" s="3">
+        <f>F147/4</f>
+        <v>85.6075</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
-      <c r="B147" s="3">
+      <c r="B148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>78.84</v>
       </c>
-      <c r="C147" s="3">
+      <c r="C148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
-      <c r="D147" s="3">
+      <c r="D148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>586.29</v>
       </c>
-      <c r="E147" s="3">
+      <c r="E148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>503.92</v>
       </c>
-      <c r="F147" s="3">
-        <f>SUM(B147:E147)</f>
-        <v>1505.4</v>
-      </c>
-      <c r="G147" s="3">
-        <f>F147/4</f>
-        <v>376.35</v>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
-        </is>
-      </c>
-      <c r="B148" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="C148" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D148" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
-      </c>
-      <c r="E148" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
-      </c>
       <c r="F148" s="3">
         <f>SUM(B148:E148)</f>
-        <v>323.16</v>
+        <v>1505.4</v>
       </c>
       <c r="G148" s="3">
         <f>F148/4</f>
-        <v>80.79</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="B149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <v>80.79</v>
       </c>
       <c r="C149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>909.94</v>
+        <v>0</v>
       </c>
       <c r="D149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <v>161.58</v>
       </c>
       <c r="E149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>839.3</v>
+        <v>80.79</v>
       </c>
       <c r="F149" s="3">
         <f>SUM(B149:E149)</f>
-        <v>3731.31</v>
+        <v>323.16</v>
       </c>
       <c r="G149" s="3">
         <f>F149/4</f>
-        <v>932.8275</v>
+        <v>80.79</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
         </is>
       </c>
       <c r="B150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>1019.45</v>
       </c>
       <c r="C150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>909.94</v>
       </c>
       <c r="D150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>962.62</v>
       </c>
       <c r="E150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>839.3</v>
       </c>
       <c r="F150" s="3">
         <f>SUM(B150:E150)</f>
-        <v>792.99</v>
+        <v>3731.31</v>
       </c>
       <c r="G150" s="3">
         <f>F150/4</f>
-        <v>198.2475</v>
+        <v>932.8275</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B151" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C151" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D151" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E151" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F151" s="3">
+        <f>SUM(B151:E151)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G151" s="3">
+        <f>F151/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B151" s="3">
+      <c r="B152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C151" s="3">
+      <c r="C152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D151" s="3">
+      <c r="D152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E151" s="3">
+      <c r="E152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F151" s="3">
-        <f>SUM(B151:E151)</f>
-        <v>4932.41</v>
-      </c>
-      <c r="G151" s="3">
-        <f>F151/4</f>
-        <v>1233.1025</v>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
-        </is>
-      </c>
-      <c r="B152" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="C152" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D152" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="E152" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.5</v>
-      </c>
       <c r="F152" s="3">
         <f>SUM(B152:E152)</f>
-        <v>397.5</v>
+        <v>4932.41</v>
       </c>
       <c r="G152" s="3">
         <f>F152/4</f>
-        <v>99.375</v>
+        <v>1233.1025</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
+        </is>
+      </c>
+      <c r="B153" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="C153" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D153" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="E153" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>32.5</v>
+      </c>
+      <c r="F153" s="3">
+        <f>SUM(B153:E153)</f>
+        <v>397.5</v>
+      </c>
+      <c r="G153" s="3">
+        <f>F153/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B153" s="3">
+      <c r="B154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C153" s="3">
+      <c r="C154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D153" s="3">
+      <c r="D154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E153" s="3">
+      <c r="E154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>357.62</v>
       </c>
-      <c r="F153" s="3">
-        <f>SUM(B153:E153)</f>
+      <c r="F154" s="3">
+        <f>SUM(B154:E154)</f>
         <v>4703.69</v>
       </c>
-      <c r="G153" s="3">
-        <f>F153/4</f>
+      <c r="G154" s="3">
+        <f>F154/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="12" t="inlineStr">
+    <row r="155">
+      <c r="A155" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B154" s="3">
+      <c r="B155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C154" s="3">
+      <c r="C155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D154" s="3">
+      <c r="D155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E154" s="3">
+      <c r="E155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F154" s="3">
-        <f>SUM(B154:E154)</f>
+      <c r="F155" s="3">
+        <f>SUM(B155:E155)</f>
         <v>737.73</v>
       </c>
-      <c r="G154" s="3">
-        <f>F154/4</f>
+      <c r="G155" s="3">
+        <f>F155/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="5" t="inlineStr">
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="27" customHeight="1">
-      <c r="A157" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="158" ht="27" customHeight="1">
       <c r="A158" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="159" ht="27" customHeight="1">
       <c r="A159" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="160" ht="27" customHeight="1">
       <c r="A160" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="161" ht="27" customHeight="1">
       <c r="A161" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, Dust and Mop House, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="162" ht="27" customHeight="1">
       <c r="A162" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
         </is>
       </c>
     </row>
     <row r="163" ht="27" customHeight="1">
       <c r="A163" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="27" customHeight="1">
+      <c r="A164" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Granville Medical and Duke charges are small hospital food/parking charges, listed under Health.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A157:G157"/>
     <mergeCell ref="A158:G158"/>
     <mergeCell ref="A159:G159"/>
     <mergeCell ref="A160:G160"/>
     <mergeCell ref="A161:G161"/>
     <mergeCell ref="A162:G162"/>
     <mergeCell ref="A163:G163"/>
+    <mergeCell ref="A164:G164"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -7451,12 +7482,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Software &amp; Online Subscriptions</t>
         </is>
       </c>
       <c r="H18" s="3">
         <f>SUMIF($C$4:$C$127,G18,$E$4:$E$127)</f>
-        <v>242.05</v>
+        <v>161.05</v>
       </c>
     </row>
     <row r="19">
@@ -7483,12 +7514,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Software &amp; Online Subscriptions</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="H19" s="3">
         <f>SUMIF($C$4:$C$127,G19,$E$4:$E$127)</f>
-        <v>161.05</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="20">
@@ -7515,12 +7546,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
         </is>
       </c>
       <c r="H20" s="3">
         <f>SUMIF($C$4:$C$127,G20,$E$4:$E$127)</f>
-        <v>160.37</v>
+        <v>142.05</v>
       </c>
     </row>
     <row r="21">
@@ -8064,7 +8095,7 @@
       </c>
       <c r="H37" s="9">
         <f>SUM(H4:H36)</f>
-        <v>12663.24</v>
+        <v>12563.24</v>
       </c>
     </row>
     <row r="38">
@@ -8175,12 +8206,12 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sloane Realty</t>
+          <t xml:space="preserve">Dust and Mop House</t>
         </is>
       </c>
       <c r="H41" s="3">
         <f>SUMIF($C$4:$C$127,G41,$E$4:$E$127)</f>
-        <v>2891.98</v>
+        <v>100.0</v>
       </c>
     </row>
     <row r="42">
@@ -8207,12 +8238,12 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Sloane Realty</t>
         </is>
       </c>
       <c r="H42" s="3">
         <f>SUMIF($C$4:$C$127,G42,$E$4:$E$127)</f>
-        <v>3.26</v>
+        <v>2891.98</v>
       </c>
     </row>
     <row r="43">
@@ -8239,12 +8270,12 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
         </is>
       </c>
       <c r="H43" s="3">
         <f>SUMIF($C$4:$C$127,G43,$E$4:$E$127)</f>
-        <v>2576.0</v>
+        <v>3.26</v>
       </c>
     </row>
     <row r="44">
@@ -8269,6 +8300,15 @@
       <c r="E44" s="3">
         <v>50.74</v>
       </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+        </is>
+      </c>
+      <c r="H44" s="3">
+        <f>SUMIF($C$4:$C$127,G44,$E$4:$E$127)</f>
+        <v>2576.0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4">
@@ -9109,7 +9149,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -10144,12 +10184,12 @@
       </c>
       <c r="C126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Dust and Mop House</t>
         </is>
       </c>
       <c r="D126" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="E126" s="3">
@@ -10190,7 +10230,7 @@
       </c>
       <c r="E128" s="9">
         <f>SUMIF(D4:D127,"&lt;&gt;Excluded",E4:E127)</f>
-        <v>12663.24</v>
+        <v>12563.24</v>
       </c>
     </row>
     <row r="129">
@@ -10201,7 +10241,7 @@
       </c>
       <c r="E129" s="6">
         <f>SUMIF(D4:D127,"Excluded",E4:E127)</f>
-        <v>12698.33</v>
+        <v>12798.33</v>
       </c>
     </row>
   </sheetData>
@@ -10485,12 +10525,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Grocery – Publix</t>
         </is>
       </c>
       <c r="H10" s="3">
         <f>SUMIF($C$4:$C$110,G10,$E$4:$E$110)</f>
-        <v>536.6</v>
+        <v>522.68</v>
       </c>
     </row>
     <row r="11">
@@ -10517,12 +10557,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grocery – Publix</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="H11" s="3">
         <f>SUMIF($C$4:$C$110,G11,$E$4:$E$110)</f>
-        <v>522.68</v>
+        <v>475.42</v>
       </c>
     </row>
     <row r="12">
@@ -10549,12 +10589,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
         </is>
       </c>
       <c r="H12" s="3">
         <f>SUMIF($C$4:$C$110,G12,$E$4:$E$110)</f>
-        <v>475.42</v>
+        <v>467.66</v>
       </c>
     </row>
     <row r="13">
@@ -10581,12 +10621,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical – Dosher Hospital (Southport)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="H13" s="3">
         <f>SUMIF($C$4:$C$110,G13,$E$4:$E$110)</f>
-        <v>467.66</v>
+        <v>436.02</v>
       </c>
     </row>
     <row r="14">
@@ -10613,12 +10653,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Health Insurance – Blue Cross NC</t>
         </is>
       </c>
       <c r="H14" s="3">
         <f>SUMIF($C$4:$C$110,G14,$E$4:$E$110)</f>
-        <v>436.02</v>
+        <v>432.5</v>
       </c>
     </row>
     <row r="15">
@@ -10645,12 +10685,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Health Insurance – Blue Cross NC</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="H15" s="3">
         <f>SUMIF($C$4:$C$110,G15,$E$4:$E$110)</f>
-        <v>432.5</v>
+        <v>406.96</v>
       </c>
     </row>
     <row r="16">
@@ -10677,12 +10717,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="H16" s="3">
         <f>SUMIF($C$4:$C$110,G16,$E$4:$E$110)</f>
-        <v>406.96</v>
+        <v>383.24</v>
       </c>
     </row>
     <row r="17">
@@ -10709,12 +10749,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVS Pharmacy</t>
+          <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
         </is>
       </c>
       <c r="H17" s="3">
         <f>SUMIF($C$4:$C$110,G17,$E$4:$E$110)</f>
-        <v>383.24</v>
+        <v>331.5</v>
       </c>
     </row>
     <row r="18">
@@ -10741,12 +10781,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfers to People (Venmo/Zelle)</t>
+          <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
       <c r="H18" s="3">
         <f>SUMIF($C$4:$C$110,G18,$E$4:$E$110)</f>
-        <v>331.5</v>
+        <v>220.0</v>
       </c>
     </row>
     <row r="19">
@@ -10773,12 +10813,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yard Company (NextGen)</t>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
         </is>
       </c>
       <c r="H19" s="3">
         <f>SUMIF($C$4:$C$110,G19,$E$4:$E$110)</f>
-        <v>220.0</v>
+        <v>182.5</v>
       </c>
     </row>
     <row r="20">
@@ -10805,12 +10845,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
         </is>
       </c>
       <c r="H20" s="3">
         <f>SUMIF($C$4:$C$110,G20,$E$4:$E$110)</f>
-        <v>182.5</v>
+        <v>179.33</v>
       </c>
     </row>
     <row r="21">
@@ -10824,7 +10864,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -10837,12 +10877,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Retail – Dillard's</t>
         </is>
       </c>
       <c r="H21" s="3">
         <f>SUMIF($C$4:$C$110,G21,$E$4:$E$110)</f>
-        <v>179.33</v>
+        <v>174.74</v>
       </c>
     </row>
     <row r="22">
@@ -10869,12 +10909,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dillard's</t>
+          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
         </is>
       </c>
       <c r="H22" s="3">
         <f>SUMIF($C$4:$C$110,G22,$E$4:$E$110)</f>
-        <v>174.74</v>
+        <v>171.55</v>
       </c>
     </row>
     <row r="23">
@@ -10901,12 +10941,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Lowe's (home improvement)</t>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
         </is>
       </c>
       <c r="H23" s="3">
         <f>SUMIF($C$4:$C$110,G23,$E$4:$E$110)</f>
-        <v>171.55</v>
+        <v>167.24</v>
       </c>
     </row>
     <row r="24">
@@ -10933,12 +10973,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Retail – Hobby Lobby</t>
         </is>
       </c>
       <c r="H24" s="3">
         <f>SUMIF($C$4:$C$110,G24,$E$4:$E$110)</f>
-        <v>167.24</v>
+        <v>165.67</v>
       </c>
     </row>
     <row r="25">
@@ -10965,12 +11005,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Hobby Lobby</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="H25" s="3">
         <f>SUMIF($C$4:$C$110,G25,$E$4:$E$110)</f>
-        <v>165.67</v>
+        <v>161.58</v>
       </c>
     </row>
     <row r="26">
@@ -10997,12 +11037,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="H26" s="3">
         <f>SUMIF($C$4:$C$110,G26,$E$4:$E$110)</f>
-        <v>161.58</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="27">
@@ -11029,12 +11069,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
         </is>
       </c>
       <c r="H27" s="3">
         <f>SUMIF($C$4:$C$110,G27,$E$4:$E$110)</f>
-        <v>160.37</v>
+        <v>104.0</v>
       </c>
     </row>
     <row r="28">
@@ -11546,7 +11586,7 @@
       </c>
       <c r="H43" s="9">
         <f>SUM(H4:H42)</f>
-        <v>15086.64</v>
+        <v>14654.04</v>
       </c>
     </row>
     <row r="44">
@@ -11689,12 +11729,12 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+          <t xml:space="preserve">Dust and Mop House</t>
         </is>
       </c>
       <c r="H48" s="3">
         <f>SUMIF($C$4:$C$110,G48,$E$4:$E$110)</f>
-        <v>2576.0</v>
+        <v>432.6</v>
       </c>
     </row>
     <row r="49">
@@ -11719,6 +11759,15 @@
       <c r="E49" s="3">
         <v>20.66</v>
       </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WTW Health Premium (reimbursed by Via Benefits)</t>
+        </is>
+      </c>
+      <c r="H49" s="3">
+        <f>SUMIF($C$4:$C$110,G49,$E$4:$E$110)</f>
+        <v>2576.0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4">
@@ -11846,12 +11895,12 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Dust and Mop House</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="E55" s="3">
@@ -13134,7 +13183,7 @@
       </c>
       <c r="E111" s="9">
         <f>SUMIF(D4:D110,"&lt;&gt;Excluded",E4:E110)</f>
-        <v>15086.64</v>
+        <v>14654.04</v>
       </c>
     </row>
     <row r="112">
@@ -13145,7 +13194,7 @@
       </c>
       <c r="E112" s="6">
         <f>SUMIF(D4:D110,"Excluded",E4:E110)</f>
-        <v>7897.08</v>
+        <v>8329.68</v>
       </c>
     </row>
   </sheetData>
@@ -21044,7 +21093,7 @@
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr">
@@ -22304,12 +22353,12 @@
       </c>
       <c r="D243" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Dust and Mop House</t>
         </is>
       </c>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="F243" s="3">
@@ -22836,7 +22885,7 @@
       </c>
       <c r="D262" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
         </is>
       </c>
       <c r="E262" s="2" t="inlineStr">
@@ -23788,12 +23837,12 @@
       </c>
       <c r="D296" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Cleaning, Pest, Lawn)</t>
+          <t xml:space="preserve">Dust and Mop House</t>
         </is>
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="F296" s="3">

</xml_diff>

<commit_message>
Add Delta Dental to Key Bills
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -3357,471 +3357,502 @@
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
         </is>
       </c>
       <c r="B143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>69.36</v>
       </c>
       <c r="C143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>69.36</v>
       </c>
       <c r="D143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>69.36</v>
       </c>
       <c r="E143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>69.36</v>
       </c>
       <c r="F143" s="3">
         <f>SUM(B143:E143)</f>
-        <v>1412.24</v>
+        <v>277.44</v>
       </c>
       <c r="G143" s="3">
         <f>F143/4</f>
-        <v>353.06</v>
+        <v>69.36</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.37</v>
+        <v>294.57</v>
       </c>
       <c r="C144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>160.37</v>
+        <v>294.8</v>
       </c>
       <c r="D144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>160.37</v>
+        <v>436.02</v>
       </c>
       <c r="E144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>160.37</v>
+        <v>386.85</v>
       </c>
       <c r="F144" s="3">
         <f>SUM(B144:E144)</f>
-        <v>641.48</v>
+        <v>1412.24</v>
       </c>
       <c r="G144" s="3">
         <f>F144/4</f>
-        <v>160.37</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVS Pharmacy</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="B145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.07</v>
+        <v>160.37</v>
       </c>
       <c r="C145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.93</v>
+        <v>160.37</v>
       </c>
       <c r="D145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>383.24</v>
+        <v>160.37</v>
       </c>
       <c r="E145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>160.37</v>
       </c>
       <c r="F145" s="3">
         <f>SUM(B145:E145)</f>
-        <v>644.24</v>
+        <v>641.48</v>
       </c>
       <c r="G145" s="3">
         <f>F145/4</f>
-        <v>161.06</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="B146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>160.07</v>
       </c>
       <c r="C146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>100.93</v>
       </c>
       <c r="D146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>383.24</v>
       </c>
       <c r="E146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>0</v>
       </c>
       <c r="F146" s="3">
         <f>SUM(B146:E146)</f>
-        <v>1162.97</v>
+        <v>644.24</v>
       </c>
       <c r="G146" s="3">
         <f>F146/4</f>
-        <v>290.7425</v>
+        <v>161.06</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>0</v>
       </c>
       <c r="C147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>336.35</v>
       </c>
       <c r="D147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>406.96</v>
       </c>
       <c r="E147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>419.66</v>
       </c>
       <c r="F147" s="3">
         <f>SUM(B147:E147)</f>
-        <v>342.43</v>
+        <v>1162.97</v>
       </c>
       <c r="G147" s="3">
         <f>F147/4</f>
-        <v>85.6075</v>
+        <v>290.7425</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+        </is>
+      </c>
+      <c r="B148" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C148" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D148" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>179.33</v>
+      </c>
+      <c r="E148" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>84.26</v>
+      </c>
+      <c r="F148" s="3">
+        <f>SUM(B148:E148)</f>
+        <v>342.43</v>
+      </c>
+      <c r="G148" s="3">
+        <f>F148/4</f>
+        <v>85.6075</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
-      <c r="B148" s="3">
+      <c r="B149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>78.84</v>
       </c>
-      <c r="C148" s="3">
+      <c r="C149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
-      <c r="D148" s="3">
+      <c r="D149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>586.29</v>
       </c>
-      <c r="E148" s="3">
+      <c r="E149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>503.92</v>
       </c>
-      <c r="F148" s="3">
-        <f>SUM(B148:E148)</f>
-        <v>1505.4</v>
-      </c>
-      <c r="G148" s="3">
-        <f>F148/4</f>
-        <v>376.35</v>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
-        </is>
-      </c>
-      <c r="B149" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="C149" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D149" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
-      </c>
-      <c r="E149" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
-      </c>
       <c r="F149" s="3">
         <f>SUM(B149:E149)</f>
-        <v>323.16</v>
+        <v>1505.4</v>
       </c>
       <c r="G149" s="3">
         <f>F149/4</f>
-        <v>80.79</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="B150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <v>80.79</v>
       </c>
       <c r="C150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>909.94</v>
+        <v>0</v>
       </c>
       <c r="D150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <v>161.58</v>
       </c>
       <c r="E150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>839.3</v>
+        <v>80.79</v>
       </c>
       <c r="F150" s="3">
         <f>SUM(B150:E150)</f>
-        <v>3731.31</v>
+        <v>323.16</v>
       </c>
       <c r="G150" s="3">
         <f>F150/4</f>
-        <v>932.8275</v>
+        <v>80.79</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
         </is>
       </c>
       <c r="B151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>1019.45</v>
       </c>
       <c r="C151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>909.94</v>
       </c>
       <c r="D151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>962.62</v>
       </c>
       <c r="E151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>839.3</v>
       </c>
       <c r="F151" s="3">
         <f>SUM(B151:E151)</f>
-        <v>792.99</v>
+        <v>3731.31</v>
       </c>
       <c r="G151" s="3">
         <f>F151/4</f>
-        <v>198.2475</v>
+        <v>932.8275</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B152" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C152" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D152" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E152" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F152" s="3">
+        <f>SUM(B152:E152)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G152" s="3">
+        <f>F152/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B152" s="3">
+      <c r="B153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C152" s="3">
+      <c r="C153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D152" s="3">
+      <c r="D153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E152" s="3">
+      <c r="E153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F152" s="3">
-        <f>SUM(B152:E152)</f>
-        <v>4932.41</v>
-      </c>
-      <c r="G152" s="3">
-        <f>F152/4</f>
-        <v>1233.1025</v>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
-        </is>
-      </c>
-      <c r="B153" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="C153" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D153" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="E153" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.5</v>
-      </c>
       <c r="F153" s="3">
         <f>SUM(B153:E153)</f>
-        <v>397.5</v>
+        <v>4932.41</v>
       </c>
       <c r="G153" s="3">
         <f>F153/4</f>
-        <v>99.375</v>
+        <v>1233.1025</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
+        </is>
+      </c>
+      <c r="B154" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="C154" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D154" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="E154" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>32.5</v>
+      </c>
+      <c r="F154" s="3">
+        <f>SUM(B154:E154)</f>
+        <v>397.5</v>
+      </c>
+      <c r="G154" s="3">
+        <f>F154/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B154" s="3">
+      <c r="B155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C154" s="3">
+      <c r="C155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D154" s="3">
+      <c r="D155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E154" s="3">
+      <c r="E155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>357.62</v>
       </c>
-      <c r="F154" s="3">
-        <f>SUM(B154:E154)</f>
+      <c r="F155" s="3">
+        <f>SUM(B155:E155)</f>
         <v>4703.69</v>
       </c>
-      <c r="G154" s="3">
-        <f>F154/4</f>
+      <c r="G155" s="3">
+        <f>F155/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" s="12" t="inlineStr">
+    <row r="156">
+      <c r="A156" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B155" s="3">
+      <c r="B156" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C155" s="3">
+      <c r="C156" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D155" s="3">
+      <c r="D156" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E155" s="3">
+      <c r="E156" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F155" s="3">
-        <f>SUM(B155:E155)</f>
+      <c r="F156" s="3">
+        <f>SUM(B156:E156)</f>
         <v>737.73</v>
       </c>
-      <c r="G155" s="3">
-        <f>F155/4</f>
+      <c r="G156" s="3">
+        <f>F156/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="5" t="inlineStr">
+    <row r="158">
+      <c r="A158" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="158" ht="27" customHeight="1">
-      <c r="A158" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="159" ht="27" customHeight="1">
       <c r="A159" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="160" ht="27" customHeight="1">
       <c r="A160" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="161" ht="27" customHeight="1">
       <c r="A161" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, Dust and Mop House, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="162" ht="27" customHeight="1">
       <c r="A162" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, Dust and Mop House, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="163" ht="27" customHeight="1">
       <c r="A163" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
         </is>
       </c>
     </row>
     <row r="164" ht="27" customHeight="1">
       <c r="A164" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="27" customHeight="1">
+      <c r="A165" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Granville Medical and Duke charges are small hospital food/parking charges, listed under Health.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A158:G158"/>
     <mergeCell ref="A159:G159"/>
     <mergeCell ref="A160:G160"/>
     <mergeCell ref="A161:G161"/>
     <mergeCell ref="A162:G162"/>
     <mergeCell ref="A163:G163"/>
     <mergeCell ref="A164:G164"/>
+    <mergeCell ref="A165:G165"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>

</xml_diff>

<commit_message>
Add Blue Cross NC to Key Bills
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -3357,502 +3357,533 @@
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
+          <t xml:space="preserve">Health Insurance – Blue Cross NC</t>
         </is>
       </c>
       <c r="B143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>69.36</v>
+        <v>216.25</v>
       </c>
       <c r="C143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>69.36</v>
+        <v>0</v>
       </c>
       <c r="D143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>69.36</v>
+        <v>432.5</v>
       </c>
       <c r="E143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>69.36</v>
+        <v>216.25</v>
       </c>
       <c r="F143" s="3">
         <f>SUM(B143:E143)</f>
-        <v>277.44</v>
+        <v>865.0</v>
       </c>
       <c r="G143" s="3">
         <f>F143/4</f>
-        <v>69.36</v>
+        <v>216.25</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
         </is>
       </c>
       <c r="B144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>69.36</v>
       </c>
       <c r="C144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>69.36</v>
       </c>
       <c r="D144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>69.36</v>
       </c>
       <c r="E144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>69.36</v>
       </c>
       <c r="F144" s="3">
         <f>SUM(B144:E144)</f>
-        <v>1412.24</v>
+        <v>277.44</v>
       </c>
       <c r="G144" s="3">
         <f>F144/4</f>
-        <v>353.06</v>
+        <v>69.36</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.37</v>
+        <v>294.57</v>
       </c>
       <c r="C145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>160.37</v>
+        <v>294.8</v>
       </c>
       <c r="D145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>160.37</v>
+        <v>436.02</v>
       </c>
       <c r="E145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>160.37</v>
+        <v>386.85</v>
       </c>
       <c r="F145" s="3">
         <f>SUM(B145:E145)</f>
-        <v>641.48</v>
+        <v>1412.24</v>
       </c>
       <c r="G145" s="3">
         <f>F145/4</f>
-        <v>160.37</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVS Pharmacy</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="B146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.07</v>
+        <v>160.37</v>
       </c>
       <c r="C146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.93</v>
+        <v>160.37</v>
       </c>
       <c r="D146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>383.24</v>
+        <v>160.37</v>
       </c>
       <c r="E146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>160.37</v>
       </c>
       <c r="F146" s="3">
         <f>SUM(B146:E146)</f>
-        <v>644.24</v>
+        <v>641.48</v>
       </c>
       <c r="G146" s="3">
         <f>F146/4</f>
-        <v>161.06</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="B147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>160.07</v>
       </c>
       <c r="C147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>100.93</v>
       </c>
       <c r="D147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>383.24</v>
       </c>
       <c r="E147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>0</v>
       </c>
       <c r="F147" s="3">
         <f>SUM(B147:E147)</f>
-        <v>1162.97</v>
+        <v>644.24</v>
       </c>
       <c r="G147" s="3">
         <f>F147/4</f>
-        <v>290.7425</v>
+        <v>161.06</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>0</v>
       </c>
       <c r="C148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>336.35</v>
       </c>
       <c r="D148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>406.96</v>
       </c>
       <c r="E148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>419.66</v>
       </c>
       <c r="F148" s="3">
         <f>SUM(B148:E148)</f>
-        <v>342.43</v>
+        <v>1162.97</v>
       </c>
       <c r="G148" s="3">
         <f>F148/4</f>
-        <v>85.6075</v>
+        <v>290.7425</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+        </is>
+      </c>
+      <c r="B149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>179.33</v>
+      </c>
+      <c r="E149" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>84.26</v>
+      </c>
+      <c r="F149" s="3">
+        <f>SUM(B149:E149)</f>
+        <v>342.43</v>
+      </c>
+      <c r="G149" s="3">
+        <f>F149/4</f>
+        <v>85.6075</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
-      <c r="B149" s="3">
+      <c r="B150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>78.84</v>
       </c>
-      <c r="C149" s="3">
+      <c r="C150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
-      <c r="D149" s="3">
+      <c r="D150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>586.29</v>
       </c>
-      <c r="E149" s="3">
+      <c r="E150" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>503.92</v>
       </c>
-      <c r="F149" s="3">
-        <f>SUM(B149:E149)</f>
-        <v>1505.4</v>
-      </c>
-      <c r="G149" s="3">
-        <f>F149/4</f>
-        <v>376.35</v>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
-        </is>
-      </c>
-      <c r="B150" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="C150" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D150" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
-      </c>
-      <c r="E150" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
-      </c>
       <c r="F150" s="3">
         <f>SUM(B150:E150)</f>
-        <v>323.16</v>
+        <v>1505.4</v>
       </c>
       <c r="G150" s="3">
         <f>F150/4</f>
-        <v>80.79</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="B151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <v>80.79</v>
       </c>
       <c r="C151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>909.94</v>
+        <v>0</v>
       </c>
       <c r="D151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <v>161.58</v>
       </c>
       <c r="E151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>839.3</v>
+        <v>80.79</v>
       </c>
       <c r="F151" s="3">
         <f>SUM(B151:E151)</f>
-        <v>3731.31</v>
+        <v>323.16</v>
       </c>
       <c r="G151" s="3">
         <f>F151/4</f>
-        <v>932.8275</v>
+        <v>80.79</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
         </is>
       </c>
       <c r="B152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>1019.45</v>
       </c>
       <c r="C152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>909.94</v>
       </c>
       <c r="D152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>962.62</v>
       </c>
       <c r="E152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>839.3</v>
       </c>
       <c r="F152" s="3">
         <f>SUM(B152:E152)</f>
-        <v>792.99</v>
+        <v>3731.31</v>
       </c>
       <c r="G152" s="3">
         <f>F152/4</f>
-        <v>198.2475</v>
+        <v>932.8275</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B153" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C153" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D153" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E153" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F153" s="3">
+        <f>SUM(B153:E153)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G153" s="3">
+        <f>F153/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B153" s="3">
+      <c r="B154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C153" s="3">
+      <c r="C154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D153" s="3">
+      <c r="D154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E153" s="3">
+      <c r="E154" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F153" s="3">
-        <f>SUM(B153:E153)</f>
-        <v>4932.41</v>
-      </c>
-      <c r="G153" s="3">
-        <f>F153/4</f>
-        <v>1233.1025</v>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
-        </is>
-      </c>
-      <c r="B154" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="C154" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D154" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="E154" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.5</v>
-      </c>
       <c r="F154" s="3">
         <f>SUM(B154:E154)</f>
-        <v>397.5</v>
+        <v>4932.41</v>
       </c>
       <c r="G154" s="3">
         <f>F154/4</f>
-        <v>99.375</v>
+        <v>1233.1025</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
+        </is>
+      </c>
+      <c r="B155" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A155,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="C155" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A155,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D155" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A155,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="E155" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A155,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>32.5</v>
+      </c>
+      <c r="F155" s="3">
+        <f>SUM(B155:E155)</f>
+        <v>397.5</v>
+      </c>
+      <c r="G155" s="3">
+        <f>F155/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B155" s="3">
+      <c r="B156" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C155" s="3">
+      <c r="C156" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D155" s="3">
+      <c r="D156" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E155" s="3">
+      <c r="E156" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>357.62</v>
       </c>
-      <c r="F155" s="3">
-        <f>SUM(B155:E155)</f>
+      <c r="F156" s="3">
+        <f>SUM(B156:E156)</f>
         <v>4703.69</v>
       </c>
-      <c r="G155" s="3">
-        <f>F155/4</f>
+      <c r="G156" s="3">
+        <f>F156/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="156">
-      <c r="A156" s="12" t="inlineStr">
+    <row r="157">
+      <c r="A157" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B156" s="3">
+      <c r="B157" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C156" s="3">
+      <c r="C157" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D156" s="3">
+      <c r="D157" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E156" s="3">
+      <c r="E157" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F156" s="3">
-        <f>SUM(B156:E156)</f>
+      <c r="F157" s="3">
+        <f>SUM(B157:E157)</f>
         <v>737.73</v>
       </c>
-      <c r="G156" s="3">
-        <f>F156/4</f>
+      <c r="G157" s="3">
+        <f>F157/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="158">
-      <c r="A158" s="5" t="inlineStr">
+    <row r="159">
+      <c r="A159" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="159" ht="27" customHeight="1">
-      <c r="A159" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="160" ht="27" customHeight="1">
       <c r="A160" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="161" ht="27" customHeight="1">
       <c r="A161" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="162" ht="27" customHeight="1">
       <c r="A162" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, Dust and Mop House, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="163" ht="27" customHeight="1">
       <c r="A163" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, Dust and Mop House, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="164" ht="27" customHeight="1">
       <c r="A164" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
         </is>
       </c>
     </row>
     <row r="165" ht="27" customHeight="1">
       <c r="A165" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="27" customHeight="1">
+      <c r="A166" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Granville Medical and Duke charges are small hospital food/parking charges, listed under Health.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A159:G159"/>
     <mergeCell ref="A160:G160"/>
     <mergeCell ref="A161:G161"/>
     <mergeCell ref="A162:G162"/>
     <mergeCell ref="A163:G163"/>
     <mergeCell ref="A164:G164"/>
     <mergeCell ref="A165:G165"/>
+    <mergeCell ref="A166:G166"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>

</xml_diff>

<commit_message>
Exclude Bowery West charges from spending
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WCTTaceqo1Qbfa4QQENzNy
</commit_message>
<xml_diff>
--- a/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
+++ b/Dempsey_Checking_Spending_Jun-Sep_2026.xlsx
@@ -2564,7 +2564,7 @@
     <row r="108">
       <c r="A108" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Entertainment (Surf Cinema)</t>
         </is>
       </c>
       <c r="B108" s="3">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="C108" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>400.0</v>
+        <v>0</v>
       </c>
       <c r="D108" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A108,'All Transactions'!$A$5:$A$436,D$4)</f>
@@ -2585,11 +2585,11 @@
       </c>
       <c r="F108" s="3">
         <f>SUM(B108:E108)</f>
-        <v>413.5</v>
+        <v>13.5</v>
       </c>
       <c r="G108" s="3">
         <f>F108/4</f>
-        <v>103.375</v>
+        <v>3.375</v>
       </c>
     </row>
     <row r="109">
@@ -2604,7 +2604,7 @@
       </c>
       <c r="C109" s="6">
         <f>SUM(C107:C108)</f>
-        <v>433.54</v>
+        <v>33.54</v>
       </c>
       <c r="D109" s="6">
         <f>SUM(D107:D108)</f>
@@ -2616,11 +2616,11 @@
       </c>
       <c r="F109" s="6">
         <f>SUM(F107:F108)</f>
-        <v>447.04</v>
+        <v>47.04</v>
       </c>
       <c r="G109" s="6">
         <f>F109/4</f>
-        <v>111.76</v>
+        <v>11.76</v>
       </c>
     </row>
     <row r="111">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="C120" s="9">
         <f>C10+C18+C23+C28+C32+C38+C43+C48+C59+C63+C71+C76+C95+C100+C104+C109+C113+C118</f>
-        <v>12563.24</v>
+        <v>12163.24</v>
       </c>
       <c r="D120" s="9">
         <f>D10+D18+D23+D28+D32+D38+D43+D48+D59+D63+D71+D76+D95+D100+D104+D109+D113+D118</f>
@@ -2816,11 +2816,11 @@
       </c>
       <c r="F120" s="9">
         <f>F10+F18+F23+F28+F32+F38+F43+F48+F59+F63+F71+F76+F95+F100+F104+F109+F113+F118</f>
-        <v>50868.72</v>
+        <v>50468.72</v>
       </c>
       <c r="G120" s="9">
         <f>F120/4</f>
-        <v>12717.18</v>
+        <v>12617.18</v>
       </c>
     </row>
     <row r="122">
@@ -2957,20 +2957,20 @@
     <row r="127">
       <c r="A127" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Checks Written (payee not shown)</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="B127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>2630.0</v>
+        <v>0</v>
       </c>
       <c r="C127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>400.0</v>
       </c>
       <c r="D127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>728.0</v>
+        <v>0</v>
       </c>
       <c r="E127" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A127,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -2978,30 +2978,30 @@
       </c>
       <c r="F127" s="3">
         <f>SUM(B127:E127)</f>
-        <v>3358.0</v>
+        <v>400.0</v>
       </c>
       <c r="G127" s="3">
         <f>F127/4</f>
-        <v>839.5</v>
+        <v>100.0</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Transfer to Own WF Account</t>
+          <t xml:space="preserve">Checks Written (payee not shown)</t>
         </is>
       </c>
       <c r="B128" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>2630.0</v>
       </c>
       <c r="C128" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3.26</v>
+        <v>0</v>
       </c>
       <c r="D128" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>728.0</v>
       </c>
       <c r="E128" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A128,'All Transactions'!$A$5:$A$436,E$4)</f>
@@ -3009,881 +3009,912 @@
       </c>
       <c r="F128" s="3">
         <f>SUM(B128:E128)</f>
-        <v>3.26</v>
+        <v>3358.0</v>
       </c>
       <c r="G128" s="3">
         <f>F128/4</f>
+        <v>839.5</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Transfer to Own WF Account</t>
+        </is>
+      </c>
+      <c r="B129" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A129,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>0</v>
+      </c>
+      <c r="C129" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A129,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>3.26</v>
+      </c>
+      <c r="D129" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A129,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>0</v>
+      </c>
+      <c r="E129" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A129,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>0</v>
+      </c>
+      <c r="F129" s="3">
+        <f>SUM(B129:E129)</f>
+        <v>3.26</v>
+      </c>
+      <c r="G129" s="3">
+        <f>F129/4</f>
         <v>0.815</v>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="7" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Total not counted as spending</t>
         </is>
       </c>
-      <c r="B129" s="6">
-        <f>SUM(B123:B128)</f>
+      <c r="B130" s="6">
+        <f>SUM(B123:B129)</f>
         <v>5206.0</v>
       </c>
-      <c r="C129" s="6">
-        <f>SUM(C123:C128)</f>
-        <v>12798.33</v>
-      </c>
-      <c r="D129" s="6">
-        <f>SUM(D123:D128)</f>
+      <c r="C130" s="6">
+        <f>SUM(C123:C129)</f>
+        <v>13198.33</v>
+      </c>
+      <c r="D130" s="6">
+        <f>SUM(D123:D129)</f>
         <v>8329.68</v>
       </c>
-      <c r="E129" s="6">
-        <f>SUM(E123:E128)</f>
+      <c r="E130" s="6">
+        <f>SUM(E123:E129)</f>
         <v>7314.51</v>
       </c>
-      <c r="F129" s="6">
-        <f>SUM(F123:F128)</f>
-        <v>33648.52</v>
-      </c>
-      <c r="G129" s="6">
-        <f>F129/4</f>
-        <v>8412.13</v>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Check: spending + not-counted items</t>
-        </is>
-      </c>
-      <c r="B131" s="3">
-        <f>B120+B129</f>
-        <v>17341.81</v>
-      </c>
-      <c r="C131" s="3">
-        <f>C120+C129</f>
-        <v>25361.57</v>
-      </c>
-      <c r="D131" s="3">
-        <f>D120+D129</f>
-        <v>22983.72</v>
-      </c>
-      <c r="E131" s="3">
-        <f>E120+E129</f>
-        <v>18830.14</v>
-      </c>
-      <c r="F131" s="3">
-        <f>F120+F129</f>
-        <v>84517.24</v>
+      <c r="F130" s="6">
+        <f>SUM(F123:F129)</f>
+        <v>34048.52</v>
+      </c>
+      <c r="G130" s="6">
+        <f>F130/4</f>
+        <v>8512.13</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
-        </is>
-      </c>
-      <c r="B132" s="13">
+          <t xml:space="preserve">Check: spending + not-counted items</t>
+        </is>
+      </c>
+      <c r="B132" s="3">
+        <f>B120+B130</f>
         <v>17341.81</v>
       </c>
-      <c r="C132" s="13">
+      <c r="C132" s="3">
+        <f>C120+C130</f>
         <v>25361.57</v>
       </c>
-      <c r="D132" s="13">
+      <c r="D132" s="3">
+        <f>D120+D130</f>
         <v>22983.72</v>
       </c>
-      <c r="E132" s="13">
+      <c r="E132" s="3">
+        <f>E120+E130</f>
         <v>18830.14</v>
       </c>
       <c r="F132" s="3">
-        <f>SUM(B132:E132)</f>
+        <f>F120+F130</f>
         <v>84517.24</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Withdrawals/Subtractions per bank statement</t>
+        </is>
+      </c>
+      <c r="B133" s="13">
+        <v>17341.81</v>
+      </c>
+      <c r="C133" s="13">
+        <v>25361.57</v>
+      </c>
+      <c r="D133" s="13">
+        <v>22983.72</v>
+      </c>
+      <c r="E133" s="13">
+        <v>18830.14</v>
+      </c>
+      <c r="F133" s="3">
+        <f>SUM(B133:E133)</f>
+        <v>84517.24</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Difference (should be $0 = every dollar accounted for)</t>
         </is>
       </c>
-      <c r="B133" s="3">
-        <f>B131-B132</f>
+      <c r="B134" s="3">
+        <f>B132-B133</f>
         <v>0.0</v>
       </c>
-      <c r="C133" s="3">
-        <f>C131-C132</f>
+      <c r="C134" s="3">
+        <f>C132-C133</f>
         <v>0.0</v>
       </c>
-      <c r="D133" s="3">
-        <f>D131-D132</f>
+      <c r="D134" s="3">
+        <f>D132-D133</f>
         <v>0.0</v>
       </c>
-      <c r="E133" s="3">
-        <f>E131-E132</f>
+      <c r="E134" s="3">
+        <f>E132-E133</f>
         <v>0.0</v>
       </c>
-      <c r="F133" s="3">
-        <f>F131-F132</f>
+      <c r="F134" s="3">
+        <f>F132-F133</f>
         <v>0.0</v>
       </c>
     </row>
-    <row r="135">
-      <c r="A135" s="5" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Key Bills at a Glance</t>
         </is>
       </c>
     </row>
-    <row r="136">
-      <c r="A136" s="15" t="inlineStr">
+    <row r="137">
+      <c r="A137" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">Bill</t>
         </is>
       </c>
-      <c r="B136" s="1" t="inlineStr">
+      <c r="B137" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">June 2026</t>
         </is>
       </c>
-      <c r="C136" s="1" t="inlineStr">
+      <c r="C137" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">July 2026</t>
         </is>
       </c>
-      <c r="D136" s="1" t="inlineStr">
+      <c r="D137" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">August 2026</t>
         </is>
       </c>
-      <c r="E136" s="1" t="inlineStr">
+      <c r="E137" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">September 2026</t>
         </is>
       </c>
-      <c r="F136" s="1" t="inlineStr">
+      <c r="F137" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">4-Month Total</t>
         </is>
       </c>
-      <c r="G136" s="1" t="inlineStr">
+      <c r="G137" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Monthly Avg</t>
         </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">A&amp;D Mortgage</t>
-        </is>
-      </c>
-      <c r="B137" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="C137" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="D137" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="E137" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A137,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>3411.1</v>
-      </c>
-      <c r="F137" s="3">
-        <f>SUM(B137:E137)</f>
-        <v>13644.4</v>
-      </c>
-      <c r="G137" s="3">
-        <f>F137/4</f>
-        <v>3411.1</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Membership (Club)</t>
+          <t xml:space="preserve">A&amp;D Mortgage</t>
         </is>
       </c>
       <c r="B138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1591.78</v>
+        <v>3411.1</v>
       </c>
       <c r="C138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>1601.56</v>
+        <v>3411.1</v>
       </c>
       <c r="D138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>1492.11</v>
+        <v>3411.1</v>
       </c>
       <c r="E138" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A138,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>1767.0</v>
+        <v>3411.1</v>
       </c>
       <c r="F138" s="3">
         <f>SUM(B138:E138)</f>
-        <v>6452.45</v>
+        <v>13644.4</v>
       </c>
       <c r="G138" s="3">
         <f>F138/4</f>
-        <v>1613.1125</v>
+        <v>3411.1</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Plantation POA Dues</t>
+          <t xml:space="preserve">St. James Membership (Club)</t>
         </is>
       </c>
       <c r="B139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>692.95</v>
+        <v>1591.78</v>
       </c>
       <c r="C139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>1601.56</v>
       </c>
       <c r="D139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>0</v>
+        <v>1492.11</v>
       </c>
       <c r="E139" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A139,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>1767.0</v>
       </c>
       <c r="F139" s="3">
         <f>SUM(B139:E139)</f>
-        <v>692.95</v>
+        <v>6452.45</v>
       </c>
       <c r="G139" s="3">
         <f>F139/4</f>
-        <v>173.2375</v>
+        <v>1613.1125</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">St. James Plantation POA Dues</t>
         </is>
       </c>
       <c r="B140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>360.42</v>
+        <v>692.95</v>
       </c>
       <c r="C140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>360.42</v>
+        <v>0</v>
       </c>
       <c r="D140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>475.42</v>
+        <v>0</v>
       </c>
       <c r="E140" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A140,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>354.17</v>
+        <v>0</v>
       </c>
       <c r="F140" s="3">
         <f>SUM(B140:E140)</f>
-        <v>1550.43</v>
+        <v>692.95</v>
       </c>
       <c r="G140" s="3">
         <f>F140/4</f>
-        <v>387.6075</v>
+        <v>173.2375</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="B141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>79.21</v>
+        <v>360.42</v>
       </c>
       <c r="C141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>73.61</v>
+        <v>360.42</v>
       </c>
       <c r="D141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>73.61</v>
+        <v>475.42</v>
       </c>
       <c r="E141" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A141,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>73.61</v>
+        <v>354.17</v>
       </c>
       <c r="F141" s="3">
         <f>SUM(B141:E141)</f>
-        <v>300.04</v>
+        <v>1550.43</v>
       </c>
       <c r="G141" s="3">
         <f>F141/4</f>
-        <v>75.01</v>
+        <v>387.6075</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Banner Life Insurance</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="B142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>710.06</v>
+        <v>79.21</v>
       </c>
       <c r="C142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="D142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="E142" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A142,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>710.06</v>
+        <v>73.61</v>
       </c>
       <c r="F142" s="3">
         <f>SUM(B142:E142)</f>
-        <v>2840.24</v>
+        <v>300.04</v>
       </c>
       <c r="G142" s="3">
         <f>F142/4</f>
-        <v>710.06</v>
+        <v>75.01</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Health Insurance – Blue Cross NC</t>
+          <t xml:space="preserve">Banner Life Insurance</t>
         </is>
       </c>
       <c r="B143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>216.25</v>
+        <v>710.06</v>
       </c>
       <c r="C143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>710.06</v>
       </c>
       <c r="D143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>432.5</v>
+        <v>710.06</v>
       </c>
       <c r="E143" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A143,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>216.25</v>
+        <v>710.06</v>
       </c>
       <c r="F143" s="3">
         <f>SUM(B143:E143)</f>
-        <v>865.0</v>
+        <v>2840.24</v>
       </c>
       <c r="G143" s="3">
         <f>F143/4</f>
-        <v>216.25</v>
+        <v>710.06</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
+          <t xml:space="preserve">Health Insurance – Blue Cross NC</t>
         </is>
       </c>
       <c r="B144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>69.36</v>
+        <v>216.25</v>
       </c>
       <c r="C144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>69.36</v>
+        <v>0</v>
       </c>
       <c r="D144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>69.36</v>
+        <v>432.5</v>
       </c>
       <c r="E144" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A144,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>69.36</v>
+        <v>216.25</v>
       </c>
       <c r="F144" s="3">
         <f>SUM(B144:E144)</f>
-        <v>277.44</v>
+        <v>865.0</v>
       </c>
       <c r="G144" s="3">
         <f>F144/4</f>
-        <v>69.36</v>
+        <v>216.25</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
         </is>
       </c>
       <c r="B145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>294.57</v>
+        <v>69.36</v>
       </c>
       <c r="C145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>294.8</v>
+        <v>69.36</v>
       </c>
       <c r="D145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>436.02</v>
+        <v>69.36</v>
       </c>
       <c r="E145" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A145,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>386.85</v>
+        <v>69.36</v>
       </c>
       <c r="F145" s="3">
         <f>SUM(B145:E145)</f>
-        <v>1412.24</v>
+        <v>277.44</v>
       </c>
       <c r="G145" s="3">
         <f>F145/4</f>
-        <v>353.06</v>
+        <v>69.36</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="B146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.37</v>
+        <v>294.57</v>
       </c>
       <c r="C146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>160.37</v>
+        <v>294.8</v>
       </c>
       <c r="D146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>160.37</v>
+        <v>436.02</v>
       </c>
       <c r="E146" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A146,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>160.37</v>
+        <v>386.85</v>
       </c>
       <c r="F146" s="3">
         <f>SUM(B146:E146)</f>
-        <v>641.48</v>
+        <v>1412.24</v>
       </c>
       <c r="G146" s="3">
         <f>F146/4</f>
-        <v>160.37</v>
+        <v>353.06</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVS Pharmacy</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="B147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>160.07</v>
+        <v>160.37</v>
       </c>
       <c r="C147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>100.93</v>
+        <v>160.37</v>
       </c>
       <c r="D147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>383.24</v>
+        <v>160.37</v>
       </c>
       <c r="E147" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A147,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>0</v>
+        <v>160.37</v>
       </c>
       <c r="F147" s="3">
         <f>SUM(B147:E147)</f>
-        <v>644.24</v>
+        <v>641.48</v>
       </c>
       <c r="G147" s="3">
         <f>F147/4</f>
-        <v>161.06</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="B148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>0</v>
+        <v>160.07</v>
       </c>
       <c r="C148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>336.35</v>
+        <v>100.93</v>
       </c>
       <c r="D148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>406.96</v>
+        <v>383.24</v>
       </c>
       <c r="E148" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A148,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>419.66</v>
+        <v>0</v>
       </c>
       <c r="F148" s="3">
         <f>SUM(B148:E148)</f>
-        <v>1162.97</v>
+        <v>644.24</v>
       </c>
       <c r="G148" s="3">
         <f>F148/4</f>
-        <v>290.7425</v>
+        <v>161.06</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="B149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>78.84</v>
+        <v>0</v>
       </c>
       <c r="C149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
+        <v>336.35</v>
       </c>
       <c r="D149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>179.33</v>
+        <v>406.96</v>
       </c>
       <c r="E149" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A149,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>84.26</v>
+        <v>419.66</v>
       </c>
       <c r="F149" s="3">
         <f>SUM(B149:E149)</f>
-        <v>342.43</v>
+        <v>1162.97</v>
       </c>
       <c r="G149" s="3">
         <f>F149/4</f>
-        <v>85.6075</v>
+        <v>290.7425</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Utility – Water/Sewer (Brunswick County)</t>
+        </is>
+      </c>
+      <c r="B150" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>78.84</v>
+      </c>
+      <c r="C150" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D150" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>179.33</v>
+      </c>
+      <c r="E150" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A150,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>84.26</v>
+      </c>
+      <c r="F150" s="3">
+        <f>SUM(B150:E150)</f>
+        <v>342.43</v>
+      </c>
+      <c r="G150" s="3">
+        <f>F150/4</f>
+        <v>85.6075</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Utilities total (BEMC + Brunswick County)</t>
         </is>
       </c>
-      <c r="B150" s="3">
+      <c r="B151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>78.84</v>
       </c>
-      <c r="C150" s="3">
+      <c r="C151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>336.35</v>
       </c>
-      <c r="D150" s="3">
+      <c r="D151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>586.29</v>
       </c>
-      <c r="E150" s="3">
+      <c r="E151" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Utilities",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>503.92</v>
       </c>
-      <c r="F150" s="3">
-        <f>SUM(B150:E150)</f>
-        <v>1505.4</v>
-      </c>
-      <c r="G150" s="3">
-        <f>F150/4</f>
-        <v>376.35</v>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Internet – Focus Broadband</t>
-        </is>
-      </c>
-      <c r="B151" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>80.79</v>
-      </c>
-      <c r="C151" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D151" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>161.58</v>
-      </c>
-      <c r="E151" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A151,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>80.79</v>
-      </c>
       <c r="F151" s="3">
         <f>SUM(B151:E151)</f>
-        <v>323.16</v>
+        <v>1505.4</v>
       </c>
       <c r="G151" s="3">
         <f>F151/4</f>
-        <v>80.79</v>
+        <v>376.35</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Restaurants &amp; Takeout</t>
+          <t xml:space="preserve">Internet – Focus Broadband</t>
         </is>
       </c>
       <c r="B152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>1019.45</v>
+        <v>80.79</v>
       </c>
       <c r="C152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>909.94</v>
+        <v>0</v>
       </c>
       <c r="D152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>962.62</v>
+        <v>161.58</v>
       </c>
       <c r="E152" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A152,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>839.3</v>
+        <v>80.79</v>
       </c>
       <c r="F152" s="3">
         <f>SUM(B152:E152)</f>
-        <v>3731.31</v>
+        <v>323.16</v>
       </c>
       <c r="G152" s="3">
         <f>F152/4</f>
-        <v>932.8275</v>
+        <v>80.79</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Restaurants &amp; Takeout</t>
         </is>
       </c>
       <c r="B153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>108.9</v>
+        <v>1019.45</v>
       </c>
       <c r="C153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>277.87</v>
+        <v>909.94</v>
       </c>
       <c r="D153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>167.24</v>
+        <v>962.62</v>
       </c>
       <c r="E153" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A153,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>238.98</v>
+        <v>839.3</v>
       </c>
       <c r="F153" s="3">
         <f>SUM(B153:E153)</f>
-        <v>792.99</v>
+        <v>3731.31</v>
       </c>
       <c r="G153" s="3">
         <f>F153/4</f>
-        <v>198.2475</v>
+        <v>932.8275</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+        </is>
+      </c>
+      <c r="B154" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>108.9</v>
+      </c>
+      <c r="C154" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>277.87</v>
+      </c>
+      <c r="D154" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>167.24</v>
+      </c>
+      <c r="E154" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A154,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>238.98</v>
+      </c>
+      <c r="F154" s="3">
+        <f>SUM(B154:E154)</f>
+        <v>792.99</v>
+      </c>
+      <c r="G154" s="3">
+        <f>F154/4</f>
+        <v>198.2475</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Groceries (Lowes Foods + Publix + Food Lion)</t>
         </is>
       </c>
-      <c r="B154" s="3">
+      <c r="B155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>1266.4</v>
       </c>
-      <c r="C154" s="3">
+      <c r="C155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1279.24</v>
       </c>
-      <c r="D154" s="3">
+      <c r="D155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>1184.27</v>
       </c>
-      <c r="E154" s="3">
+      <c r="E155" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Groceries",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>1202.5</v>
       </c>
-      <c r="F154" s="3">
-        <f>SUM(B154:E154)</f>
-        <v>4932.41</v>
-      </c>
-      <c r="G154" s="3">
-        <f>F154/4</f>
-        <v>1233.1025</v>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Haircuts – The Color Bar</t>
-        </is>
-      </c>
-      <c r="B155" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A155,'All Transactions'!$A$5:$A$436,B$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="C155" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A155,'All Transactions'!$A$5:$A$436,C$4)</f>
-        <v>0</v>
-      </c>
-      <c r="D155" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A155,'All Transactions'!$A$5:$A$436,D$4)</f>
-        <v>182.5</v>
-      </c>
-      <c r="E155" s="3">
-        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A155,'All Transactions'!$A$5:$A$436,E$4)</f>
-        <v>32.5</v>
-      </c>
       <c r="F155" s="3">
         <f>SUM(B155:E155)</f>
-        <v>397.5</v>
+        <v>4932.41</v>
       </c>
       <c r="G155" s="3">
         <f>F155/4</f>
-        <v>99.375</v>
+        <v>1233.1025</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Haircuts – The Color Bar</t>
+        </is>
+      </c>
+      <c r="B156" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A156,'All Transactions'!$A$5:$A$436,B$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="C156" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A156,'All Transactions'!$A$5:$A$436,C$4)</f>
+        <v>0</v>
+      </c>
+      <c r="D156" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A156,'All Transactions'!$A$5:$A$436,D$4)</f>
+        <v>182.5</v>
+      </c>
+      <c r="E156" s="3">
+        <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$D$5:$D$436,$A156,'All Transactions'!$A$5:$A$436,E$4)</f>
+        <v>32.5</v>
+      </c>
+      <c r="F156" s="3">
+        <f>SUM(B156:E156)</f>
+        <v>397.5</v>
+      </c>
+      <c r="G156" s="3">
+        <f>F156/4</f>
+        <v>99.375</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Retail (all retailers)</t>
         </is>
       </c>
-      <c r="B156" s="3">
+      <c r="B157" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>815.42</v>
       </c>
-      <c r="C156" s="3">
+      <c r="C157" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>1150.18</v>
       </c>
-      <c r="D156" s="3">
+      <c r="D157" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>2380.47</v>
       </c>
-      <c r="E156" s="3">
+      <c r="E157" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Retail",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>357.62</v>
       </c>
-      <c r="F156" s="3">
-        <f>SUM(B156:E156)</f>
+      <c r="F157" s="3">
+        <f>SUM(B157:E157)</f>
         <v>4703.69</v>
       </c>
-      <c r="G156" s="3">
-        <f>F156/4</f>
+      <c r="G157" s="3">
+        <f>F157/4</f>
         <v>1175.9225</v>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="12" t="inlineStr">
+    <row r="158">
+      <c r="A158" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Streaming (all services)</t>
         </is>
       </c>
-      <c r="B157" s="3">
+      <c r="B158" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,B$4)</f>
         <v>188.8</v>
       </c>
-      <c r="C157" s="3">
+      <c r="C158" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,C$4)</f>
         <v>201.6</v>
       </c>
-      <c r="D157" s="3">
+      <c r="D158" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,D$4)</f>
         <v>158.35</v>
       </c>
-      <c r="E157" s="3">
+      <c r="E158" s="3">
         <f>SUMIFS('All Transactions'!$F$5:$F$436,'All Transactions'!$E$5:$E$436,"Streaming",'All Transactions'!$A$5:$A$436,E$4)</f>
         <v>188.98</v>
       </c>
-      <c r="F157" s="3">
-        <f>SUM(B157:E157)</f>
+      <c r="F158" s="3">
+        <f>SUM(B158:E158)</f>
         <v>737.73</v>
       </c>
-      <c r="G157" s="3">
-        <f>F157/4</f>
+      <c r="G158" s="3">
+        <f>F158/4</f>
         <v>184.4325</v>
       </c>
     </row>
-    <row r="159">
-      <c r="A159" s="5" t="inlineStr">
+    <row r="160">
+      <c r="A160" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Notes &amp; assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="160" ht="27" customHeight="1">
-      <c r="A160" s="11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="161" ht="27" customHeight="1">
       <c r="A161" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
+          <t xml:space="preserve">• "Month" = the bank statement period (June stmt 5/27–6/24, July 6/25–7/23, Aug 7/24–8/25, Sept 8/26–9/24), not the calendar month.</t>
         </is>
       </c>
     </row>
     <row r="162" ht="27" customHeight="1">
       <c r="A162" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
+          <t xml:space="preserve">• Statement totals in blue are typed from each statement's "Withdrawals/Subtractions" line; the Difference row proves every withdrawal is accounted for. "Autobks*Nextgen" = the yard company (Home group).</t>
         </is>
       </c>
     </row>
     <row r="163" ht="27" customHeight="1">
       <c r="A163" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, Dust and Mop House, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
+          <t xml:space="preserve">• Insurance: Allstate, Life Insurance (Lincoln National "Lifecomm" EDI payments) and Banner Life are kept separate as requested. Allstate on 8/3 ($115.00) is an extra payment beyond the usual monthly draft.</t>
         </is>
       </c>
     </row>
     <row r="164" ht="27" customHeight="1">
       <c r="A164" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
+          <t xml:space="preserve">• Not counted as spending (per your instructions): WTW health premium ($2,576/mo, reimbursed by Via Benefits), American Express credit card payoffs, Sloane Realty, Dust and Mop House, Bowery West, checks #101/102/103/518/520, and a $3.26 transfer to your own Wells Fargo account. They are listed in their own section so the sheet still ties to the bank statement.</t>
         </is>
       </c>
     </row>
     <row r="165" ht="27" customHeight="1">
       <c r="A165" s="11" t="inlineStr">
         <is>
-          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+          <t xml:space="preserve">• Utilities = BEMC (Brunswick Electric Membership Corp, electric) and Brunswick County Utilities (water/sewer, incl. $2.95 online-payment fee). Verizon Wireless and Focus Broadband (internet) are in Phone &amp; Internet.</t>
         </is>
       </c>
     </row>
     <row r="166" ht="27" customHeight="1">
       <c r="A166" s="11" t="inlineStr">
         <is>
+          <t xml:space="preserve">• St. James: "St James 7134 PAP" = club membership monthly draft; "St James Plantation Assn Dues" = POA dues (June only). St. James Marina purchases are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="27" customHeight="1">
+      <c r="A167" s="11" t="inlineStr">
+        <is>
           <t xml:space="preserve">• Streaming: one line per service. No Netflix charges appear on these statements (it may be billed to a credit card). The Sept 13 Google YouTube TV charge ($43.43) is an extra charge on top of the regular $89. Apple.com/Bill charges are in Software &amp; Online Subscriptions because the statement does not say which Apple service they are for. Retail: one line per retailer. Belk appears only as Belk store-card payments (the store purchases themselves are on the card). Walmart may include some groceries. Gas &amp; Convenience includes everything bought at gas stations (fuel and snacks can't be separated). Granville Medical and Duke charges are small hospital food/parking charges, listed under Health.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A160:G160"/>
     <mergeCell ref="A161:G161"/>
     <mergeCell ref="A162:G162"/>
     <mergeCell ref="A163:G163"/>
     <mergeCell ref="A164:G164"/>
     <mergeCell ref="A165:G165"/>
     <mergeCell ref="A166:G166"/>
+    <mergeCell ref="A167:G167"/>
   </mergeCells>
   <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToHeight="0"/>
@@ -7320,12 +7351,12 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Allstate Insurance</t>
         </is>
       </c>
       <c r="H11" s="3">
         <f>SUMIF($C$4:$C$127,G11,$E$4:$E$127)</f>
-        <v>400.0</v>
+        <v>360.42</v>
       </c>
     </row>
     <row r="12">
@@ -7352,12 +7383,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Allstate Insurance</t>
+          <t xml:space="preserve">Grocery – Food Lion</t>
         </is>
       </c>
       <c r="H12" s="3">
         <f>SUMIF($C$4:$C$127,G12,$E$4:$E$127)</f>
-        <v>360.42</v>
+        <v>336.67</v>
       </c>
     </row>
     <row r="13">
@@ -7384,12 +7415,12 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grocery – Food Lion</t>
+          <t xml:space="preserve">Utility – Electric (BEMC)</t>
         </is>
       </c>
       <c r="H13" s="3">
         <f>SUMIF($C$4:$C$127,G13,$E$4:$E$127)</f>
-        <v>336.67</v>
+        <v>336.35</v>
       </c>
     </row>
     <row r="14">
@@ -7416,12 +7447,12 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Utility – Electric (BEMC)</t>
+          <t xml:space="preserve">Grocery – Publix</t>
         </is>
       </c>
       <c r="H14" s="3">
         <f>SUMIF($C$4:$C$127,G14,$E$4:$E$127)</f>
-        <v>336.35</v>
+        <v>331.43</v>
       </c>
     </row>
     <row r="15">
@@ -7448,12 +7479,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grocery – Publix</t>
+          <t xml:space="preserve">Verizon Wireless</t>
         </is>
       </c>
       <c r="H15" s="3">
         <f>SUMIF($C$4:$C$127,G15,$E$4:$E$127)</f>
-        <v>331.43</v>
+        <v>294.8</v>
       </c>
     </row>
     <row r="16">
@@ -7480,12 +7511,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Verizon Wireless</t>
+          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
         </is>
       </c>
       <c r="H16" s="3">
         <f>SUMIF($C$4:$C$127,G16,$E$4:$E$127)</f>
-        <v>294.8</v>
+        <v>277.87</v>
       </c>
     </row>
     <row r="17">
@@ -7512,12 +7543,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gas &amp; Convenience Stores</t>
+          <t xml:space="preserve">Software &amp; Online Subscriptions</t>
         </is>
       </c>
       <c r="H17" s="3">
         <f>SUMIF($C$4:$C$127,G17,$E$4:$E$127)</f>
-        <v>277.87</v>
+        <v>161.05</v>
       </c>
     </row>
     <row r="18">
@@ -7544,12 +7575,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Software &amp; Online Subscriptions</t>
+          <t xml:space="preserve">Student Loan (Dept of Education)</t>
         </is>
       </c>
       <c r="H18" s="3">
         <f>SUMIF($C$4:$C$127,G18,$E$4:$E$127)</f>
-        <v>161.05</v>
+        <v>160.37</v>
       </c>
     </row>
     <row r="19">
@@ -7576,12 +7607,12 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Student Loan (Dept of Education)</t>
+          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
         </is>
       </c>
       <c r="H19" s="3">
         <f>SUMIF($C$4:$C$127,G19,$E$4:$E$127)</f>
-        <v>160.37</v>
+        <v>142.05</v>
       </c>
     </row>
     <row r="20">
@@ -7608,12 +7639,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Home Services (Pest Control, Lawn Treatment)</t>
+          <t xml:space="preserve">Retail – Walmart</t>
         </is>
       </c>
       <c r="H20" s="3">
         <f>SUMIF($C$4:$C$127,G20,$E$4:$E$127)</f>
-        <v>142.05</v>
+        <v>132.66</v>
       </c>
     </row>
     <row r="21">
@@ -7640,12 +7671,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Walmart</t>
+          <t xml:space="preserve">CVS Pharmacy</t>
         </is>
       </c>
       <c r="H21" s="3">
         <f>SUMIF($C$4:$C$127,G21,$E$4:$E$127)</f>
-        <v>132.66</v>
+        <v>100.93</v>
       </c>
     </row>
     <row r="22">
@@ -7672,12 +7703,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CVS Pharmacy</t>
+          <t xml:space="preserve">Streaming – YouTube TV (Google)</t>
         </is>
       </c>
       <c r="H22" s="3">
         <f>SUMIF($C$4:$C$127,G22,$E$4:$E$127)</f>
-        <v>100.93</v>
+        <v>100.78</v>
       </c>
     </row>
     <row r="23">
@@ -7704,12 +7735,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – YouTube TV (Google)</t>
+          <t xml:space="preserve">Yard Company (NextGen)</t>
         </is>
       </c>
       <c r="H23" s="3">
         <f>SUMIF($C$4:$C$127,G23,$E$4:$E$127)</f>
-        <v>100.78</v>
+        <v>100.0</v>
       </c>
     </row>
     <row r="24">
@@ -7736,12 +7767,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Yard Company (NextGen)</t>
+          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
         </is>
       </c>
       <c r="H24" s="3">
         <f>SUMIF($C$4:$C$127,G24,$E$4:$E$127)</f>
-        <v>100.0</v>
+        <v>73.61</v>
       </c>
     </row>
     <row r="25">
@@ -7768,12 +7799,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Life Insurance (Lincoln National)</t>
+          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
         </is>
       </c>
       <c r="H25" s="3">
         <f>SUMIF($C$4:$C$127,G25,$E$4:$E$127)</f>
-        <v>73.61</v>
+        <v>69.36</v>
       </c>
     </row>
     <row r="26">
@@ -7800,12 +7831,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dental Insurance – Delta Dental</t>
+          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
         </is>
       </c>
       <c r="H26" s="3">
         <f>SUMIF($C$4:$C$127,G26,$E$4:$E$127)</f>
-        <v>69.36</v>
+        <v>63.61</v>
       </c>
     </row>
     <row r="27">
@@ -7832,12 +7863,12 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Retail – Dick's Sporting Goods</t>
+          <t xml:space="preserve">St. James Marina</t>
         </is>
       </c>
       <c r="H27" s="3">
         <f>SUMIF($C$4:$C$127,G27,$E$4:$E$127)</f>
-        <v>63.61</v>
+        <v>33.54</v>
       </c>
     </row>
     <row r="28">
@@ -7864,12 +7895,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">St. James Marina</t>
+          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
         </is>
       </c>
       <c r="H28" s="3">
         <f>SUMIF($C$4:$C$127,G28,$E$4:$E$127)</f>
-        <v>33.54</v>
+        <v>25.16</v>
       </c>
     </row>
     <row r="29">
@@ -7896,12 +7927,12 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Medical – Granville Medical Center (Oxford)</t>
+          <t xml:space="preserve">Streaming – Frndly TV</t>
         </is>
       </c>
       <c r="H29" s="3">
         <f>SUMIF($C$4:$C$127,G29,$E$4:$E$127)</f>
-        <v>25.16</v>
+        <v>22.41</v>
       </c>
     </row>
     <row r="30">
@@ -7928,12 +7959,12 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Frndly TV</t>
+          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
         </is>
       </c>
       <c r="H30" s="3">
         <f>SUMIF($C$4:$C$127,G30,$E$4:$E$127)</f>
-        <v>22.41</v>
+        <v>20.27</v>
       </c>
     </row>
     <row r="31">
@@ -7960,12 +7991,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Disney (via Roku)</t>
+          <t xml:space="preserve">Streaming – HBO Max</t>
         </is>
       </c>
       <c r="H31" s="3">
         <f>SUMIF($C$4:$C$127,G31,$E$4:$E$127)</f>
-        <v>20.27</v>
+        <v>19.74</v>
       </c>
     </row>
     <row r="32">
@@ -7992,12 +8023,12 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – HBO Max</t>
+          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
         </is>
       </c>
       <c r="H32" s="3">
         <f>SUMIF($C$4:$C$127,G32,$E$4:$E$127)</f>
-        <v>19.74</v>
+        <v>13.87</v>
       </c>
     </row>
     <row r="33">
@@ -8024,12 +8055,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – ESPN (Sept billed as Disney Plus)</t>
+          <t xml:space="preserve">Streaming – Hulu</t>
         </is>
       </c>
       <c r="H33" s="3">
         <f>SUMIF($C$4:$C$127,G33,$E$4:$E$127)</f>
-        <v>13.87</v>
+        <v>12.8</v>
       </c>
     </row>
     <row r="34">
@@ -8056,12 +8087,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Hulu</t>
+          <t xml:space="preserve">Streaming – Peacock (via Roku)</t>
         </is>
       </c>
       <c r="H34" s="3">
         <f>SUMIF($C$4:$C$127,G34,$E$4:$E$127)</f>
-        <v>12.8</v>
+        <v>11.73</v>
       </c>
     </row>
     <row r="35">
@@ -8088,12 +8119,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Streaming – Peacock (via Roku)</t>
+          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
         </is>
       </c>
       <c r="H35" s="3">
         <f>SUMIF($C$4:$C$127,G35,$E$4:$E$127)</f>
-        <v>11.73</v>
+        <v>5.87</v>
       </c>
     </row>
     <row r="36">
@@ -8118,14 +8149,14 @@
       <c r="E36" s="3">
         <v>8.85</v>
       </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Retail – Dollar Tree / Dollar General</t>
-        </is>
-      </c>
-      <c r="H36" s="3">
-        <f>SUMIF($C$4:$C$127,G36,$E$4:$E$127)</f>
-        <v>5.87</v>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Total spending</t>
+        </is>
+      </c>
+      <c r="H36" s="9">
+        <f>SUM(H4:H35)</f>
+        <v>12163.24</v>
       </c>
     </row>
     <row r="37">
@@ -8150,15 +8181,6 @@
       <c r="E37" s="3">
         <v>24.15</v>
       </c>
-      <c r="G37" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Total spending</t>
-        </is>
-      </c>
-      <c r="H37" s="9">
-        <f>SUM(H4:H36)</f>
-        <v>12563.24</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" s="4">
@@ -8182,6 +8204,12 @@
       <c r="E38" s="3">
         <v>24.34</v>
       </c>
+      <c r="G38" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not counted as spending</t>
+        </is>
+      </c>
+      <c r="H38" s="7"/>
     </row>
     <row r="39">
       <c r="A39" s="4">
@@ -8205,12 +8233,15 @@
       <c r="E39" s="3">
         <v>12.21</v>
       </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Not counted as spending</t>
-        </is>
-      </c>
-      <c r="H39" s="7"/>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bowery West</t>
+        </is>
+      </c>
+      <c r="H39" s="3">
+        <f>SUMIF($C$4:$C$127,G39,$E$4:$E$127)</f>
+        <v>400.0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4">
@@ -9901,12 +9932,12 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recreation</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="E111" s="3">
@@ -9924,12 +9955,12 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recreation</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="E112" s="3">
@@ -9947,12 +9978,12 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recreation</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="E113" s="3">
@@ -9970,12 +10001,12 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recreation</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="E114" s="3">
@@ -10292,7 +10323,7 @@
       </c>
       <c r="E128" s="9">
         <f>SUMIF(D4:D127,"&lt;&gt;Excluded",E4:E127)</f>
-        <v>12563.24</v>
+        <v>12163.24</v>
       </c>
     </row>
     <row r="129">
@@ -10303,7 +10334,7 @@
       </c>
       <c r="E129" s="6">
         <f>SUMIF(D4:D127,"Excluded",E4:E127)</f>
-        <v>12798.33</v>
+        <v>13198.33</v>
       </c>
     </row>
   </sheetData>
@@ -11547,7 +11578,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Entertainment (Surf Cinema)</t>
         </is>
       </c>
       <c r="H40" s="3">
@@ -12187,7 +12218,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Entertainment (Surf Cinema)</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -21995,12 +22026,12 @@
       </c>
       <c r="D228" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recreation</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="F228" s="3">
@@ -22023,12 +22054,12 @@
       </c>
       <c r="D229" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recreation</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="F229" s="3">
@@ -22051,12 +22082,12 @@
       </c>
       <c r="D230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recreation</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="F230" s="3">
@@ -22079,12 +22110,12 @@
       </c>
       <c r="D231" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Bowery West</t>
         </is>
       </c>
       <c r="E231" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Recreation</t>
+          <t xml:space="preserve">Excluded</t>
         </is>
       </c>
       <c r="F231" s="3">
@@ -24179,7 +24210,7 @@
       </c>
       <c r="D306" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Entertainment &amp; Events</t>
+          <t xml:space="preserve">Entertainment (Surf Cinema)</t>
         </is>
       </c>
       <c r="E306" s="2" t="inlineStr">

</xml_diff>